<commit_message>
feat: Update synonyms and metric names in dbt schema for consistency and clarity
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76502C5A-D9B4-A74B-A10D-C8735D63B3EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1E668E0-EF2B-514A-835C-ED06C3B53A47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -192,9 +192,6 @@
     <t>DECIMAL(15,2)</t>
   </si>
   <si>
-    <t>sum, avg, min, max</t>
-  </si>
-  <si>
     <t>Current liquid money available. Use this for 'total savings' or 'wealthiest customers' metrics.</t>
   </si>
   <si>
@@ -204,9 +201,6 @@
     <t>DECIMAL(4,2)</t>
   </si>
   <si>
-    <t>avg, min, max</t>
-  </si>
-  <si>
     <t>The annual percentage yield interest tracking rate assigned to this savings account.</t>
   </si>
   <si>
@@ -306,9 +300,6 @@
     <t>credit_limit</t>
   </si>
   <si>
-    <t>sum, avg</t>
-  </si>
-  <si>
     <t>The maximum revolving credit threshold limit extended to the customer.</t>
   </si>
   <si>
@@ -484,6 +475,15 @@
   </si>
   <si>
     <t>Unsecured personal loan facility.</t>
+  </si>
+  <si>
+    <t>sum, average, min, max</t>
+  </si>
+  <si>
+    <t>average, min, max</t>
+  </si>
+  <si>
+    <t>sum, average</t>
   </si>
 </sst>
 </file>
@@ -1217,13 +1217,13 @@
         <v>33</v>
       </c>
       <c r="G12" t="s">
+        <v>151</v>
+      </c>
+      <c r="H12" t="s">
+        <v>29</v>
+      </c>
+      <c r="J12" t="s">
         <v>56</v>
-      </c>
-      <c r="H12" t="s">
-        <v>29</v>
-      </c>
-      <c r="J12" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
@@ -1231,22 +1231,22 @@
         <v>6</v>
       </c>
       <c r="B13" t="s">
+        <v>57</v>
+      </c>
+      <c r="C13" t="s">
         <v>58</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
+        <v>33</v>
+      </c>
+      <c r="G13" t="s">
+        <v>152</v>
+      </c>
+      <c r="H13" t="s">
+        <v>29</v>
+      </c>
+      <c r="J13" t="s">
         <v>59</v>
-      </c>
-      <c r="D13" t="s">
-        <v>33</v>
-      </c>
-      <c r="G13" t="s">
-        <v>60</v>
-      </c>
-      <c r="H13" t="s">
-        <v>29</v>
-      </c>
-      <c r="J13" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
@@ -1254,7 +1254,7 @@
         <v>6</v>
       </c>
       <c r="B14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C14" t="s">
         <v>32</v>
@@ -1263,13 +1263,13 @@
         <v>33</v>
       </c>
       <c r="H14" t="s">
+        <v>61</v>
+      </c>
+      <c r="I14" t="s">
+        <v>62</v>
+      </c>
+      <c r="J14" t="s">
         <v>63</v>
-      </c>
-      <c r="I14" t="s">
-        <v>64</v>
-      </c>
-      <c r="J14" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
@@ -1277,7 +1277,7 @@
         <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C15" t="s">
         <v>27</v>
@@ -1289,7 +1289,7 @@
         <v>29</v>
       </c>
       <c r="J15" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
@@ -1315,7 +1315,7 @@
         <v>29</v>
       </c>
       <c r="J16" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
@@ -1335,7 +1335,7 @@
         <v>29</v>
       </c>
       <c r="J17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
@@ -1343,7 +1343,7 @@
         <v>8</v>
       </c>
       <c r="B18" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C18" t="s">
         <v>55</v>
@@ -1352,13 +1352,13 @@
         <v>33</v>
       </c>
       <c r="G18" t="s">
-        <v>56</v>
+        <v>151</v>
       </c>
       <c r="H18" t="s">
         <v>29</v>
       </c>
       <c r="J18" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
@@ -1366,7 +1366,7 @@
         <v>8</v>
       </c>
       <c r="B19" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C19" t="s">
         <v>40</v>
@@ -1378,7 +1378,7 @@
         <v>29</v>
       </c>
       <c r="J19" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
@@ -1386,22 +1386,22 @@
         <v>8</v>
       </c>
       <c r="B20" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" t="s">
         <v>58</v>
       </c>
-      <c r="C20" t="s">
-        <v>59</v>
-      </c>
       <c r="D20" t="s">
         <v>33</v>
       </c>
       <c r="G20" t="s">
-        <v>60</v>
+        <v>152</v>
       </c>
       <c r="H20" t="s">
         <v>29</v>
       </c>
       <c r="J20" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
@@ -1409,7 +1409,7 @@
         <v>8</v>
       </c>
       <c r="B21" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C21" t="s">
         <v>32</v>
@@ -1418,13 +1418,13 @@
         <v>33</v>
       </c>
       <c r="H21" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="I21" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J21" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
@@ -1432,7 +1432,7 @@
         <v>10</v>
       </c>
       <c r="B22" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C22" t="s">
         <v>27</v>
@@ -1444,7 +1444,7 @@
         <v>29</v>
       </c>
       <c r="J22" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
@@ -1470,7 +1470,7 @@
         <v>29</v>
       </c>
       <c r="J23" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
@@ -1478,7 +1478,7 @@
         <v>10</v>
       </c>
       <c r="B24" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C24" t="s">
         <v>32</v>
@@ -1487,13 +1487,13 @@
         <v>33</v>
       </c>
       <c r="H24" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="I24" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="J24" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
@@ -1501,7 +1501,7 @@
         <v>10</v>
       </c>
       <c r="B25" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C25" t="s">
         <v>55</v>
@@ -1510,13 +1510,13 @@
         <v>33</v>
       </c>
       <c r="G25" t="s">
-        <v>56</v>
+        <v>151</v>
       </c>
       <c r="H25" t="s">
         <v>29</v>
       </c>
       <c r="J25" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
@@ -1524,7 +1524,7 @@
         <v>10</v>
       </c>
       <c r="B26" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C26" t="s">
         <v>55</v>
@@ -1533,13 +1533,13 @@
         <v>33</v>
       </c>
       <c r="G26" t="s">
-        <v>56</v>
+        <v>151</v>
       </c>
       <c r="H26" t="s">
         <v>29</v>
       </c>
       <c r="J26" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
@@ -1547,7 +1547,7 @@
         <v>10</v>
       </c>
       <c r="B27" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C27" t="s">
         <v>40</v>
@@ -1559,7 +1559,7 @@
         <v>29</v>
       </c>
       <c r="J27" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
@@ -1567,7 +1567,7 @@
         <v>10</v>
       </c>
       <c r="B28" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C28" t="s">
         <v>32</v>
@@ -1576,13 +1576,13 @@
         <v>33</v>
       </c>
       <c r="H28" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="I28" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J28" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
@@ -1590,7 +1590,7 @@
         <v>12</v>
       </c>
       <c r="B29" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C29" t="s">
         <v>27</v>
@@ -1602,7 +1602,7 @@
         <v>29</v>
       </c>
       <c r="J29" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
@@ -1628,7 +1628,7 @@
         <v>29</v>
       </c>
       <c r="J30" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
@@ -1636,7 +1636,7 @@
         <v>12</v>
       </c>
       <c r="B31" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C31" t="s">
         <v>32</v>
@@ -1648,7 +1648,7 @@
         <v>29</v>
       </c>
       <c r="J31" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
@@ -1656,7 +1656,7 @@
         <v>12</v>
       </c>
       <c r="B32" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C32" t="s">
         <v>55</v>
@@ -1665,13 +1665,13 @@
         <v>33</v>
       </c>
       <c r="G32" t="s">
-        <v>94</v>
+        <v>153</v>
       </c>
       <c r="H32" t="s">
         <v>29</v>
       </c>
       <c r="J32" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
@@ -1679,7 +1679,7 @@
         <v>12</v>
       </c>
       <c r="B33" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C33" t="s">
         <v>55</v>
@@ -1688,13 +1688,13 @@
         <v>33</v>
       </c>
       <c r="G33" t="s">
-        <v>56</v>
+        <v>151</v>
       </c>
       <c r="H33" t="s">
         <v>29</v>
       </c>
       <c r="J33" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
@@ -1702,7 +1702,7 @@
         <v>12</v>
       </c>
       <c r="B34" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C34" t="s">
         <v>40</v>
@@ -1714,7 +1714,7 @@
         <v>29</v>
       </c>
       <c r="J34" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
@@ -1722,7 +1722,7 @@
         <v>12</v>
       </c>
       <c r="B35" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C35" t="s">
         <v>32</v>
@@ -1731,13 +1731,13 @@
         <v>33</v>
       </c>
       <c r="H35" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="I35" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="J35" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
@@ -1745,7 +1745,7 @@
         <v>14</v>
       </c>
       <c r="B36" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C36" t="s">
         <v>27</v>
@@ -1757,7 +1757,7 @@
         <v>29</v>
       </c>
       <c r="J36" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
@@ -1774,7 +1774,7 @@
         <v>33</v>
       </c>
       <c r="E37" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="F37" t="s">
         <v>50</v>
@@ -1783,7 +1783,7 @@
         <v>29</v>
       </c>
       <c r="J37" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
@@ -1791,7 +1791,7 @@
         <v>14</v>
       </c>
       <c r="B38" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C38" t="s">
         <v>55</v>
@@ -1800,13 +1800,13 @@
         <v>33</v>
       </c>
       <c r="G38" t="s">
-        <v>56</v>
+        <v>151</v>
       </c>
       <c r="H38" t="s">
         <v>29</v>
       </c>
       <c r="J38" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
@@ -1814,7 +1814,7 @@
         <v>14</v>
       </c>
       <c r="B39" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C39" t="s">
         <v>32</v>
@@ -1823,13 +1823,13 @@
         <v>33</v>
       </c>
       <c r="H39" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="I39" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="J39" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
@@ -1837,10 +1837,10 @@
         <v>14</v>
       </c>
       <c r="B40" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C40" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D40" t="s">
         <v>33</v>
@@ -1849,7 +1849,7 @@
         <v>29</v>
       </c>
       <c r="J40" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
@@ -1857,7 +1857,7 @@
         <v>14</v>
       </c>
       <c r="B41" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C41" t="s">
         <v>32</v>
@@ -1869,7 +1869,7 @@
         <v>29</v>
       </c>
       <c r="J41" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
@@ -1877,7 +1877,7 @@
         <v>16</v>
       </c>
       <c r="B42" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C42" t="s">
         <v>27</v>
@@ -1889,7 +1889,7 @@
         <v>29</v>
       </c>
       <c r="J42" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
@@ -1897,7 +1897,7 @@
         <v>16</v>
       </c>
       <c r="B43" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C43" t="s">
         <v>32</v>
@@ -1909,7 +1909,7 @@
         <v>43</v>
       </c>
       <c r="J43" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.2">
@@ -1917,7 +1917,7 @@
         <v>16</v>
       </c>
       <c r="B44" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C44" t="s">
         <v>32</v>
@@ -1929,7 +1929,7 @@
         <v>43</v>
       </c>
       <c r="J44" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
@@ -1937,7 +1937,7 @@
         <v>16</v>
       </c>
       <c r="B45" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C45" t="s">
         <v>27</v>
@@ -1946,13 +1946,13 @@
         <v>33</v>
       </c>
       <c r="G45" t="s">
-        <v>94</v>
+        <v>153</v>
       </c>
       <c r="H45" t="s">
         <v>29</v>
       </c>
       <c r="J45" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
@@ -1960,22 +1960,22 @@
         <v>16</v>
       </c>
       <c r="B46" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C46" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="D46" t="s">
         <v>33</v>
       </c>
       <c r="G46" t="s">
-        <v>60</v>
+        <v>152</v>
       </c>
       <c r="H46" t="s">
         <v>29</v>
       </c>
       <c r="J46" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -2003,13 +2003,13 @@
         <v>18</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -2017,16 +2017,16 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C2" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E2" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -2034,16 +2034,16 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C3" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D3" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E3" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -2051,16 +2051,16 @@
         <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C4" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D4" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="E4" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -2068,16 +2068,16 @@
         <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C5" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D5" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="E5" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -2088,13 +2088,13 @@
         <v>42</v>
       </c>
       <c r="C6" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="D6" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E6" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -2102,16 +2102,16 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C7" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D7" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="E7" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -2119,16 +2119,16 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C8" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D8" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E8" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -2136,16 +2136,16 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C9" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D9" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E9" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Enhance dbt model SQL files with dynamic schema support and improve value mapping descriptions
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1E668E0-EF2B-514A-835C-ED06C3B53A47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AEA1656-F8F8-A64A-A901-1546E0DBAF9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -505,12 +505,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -540,11 +546,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -852,7 +862,7 @@
   <cols>
     <col min="1" max="1" width="20.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="88.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="88.6640625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -862,7 +872,7 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
@@ -873,7 +883,7 @@
       <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
         <v>5</v>
       </c>
     </row>
@@ -884,7 +894,7 @@
       <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -895,7 +905,7 @@
       <c r="B4" t="s">
         <v>4</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="3" t="s">
         <v>9</v>
       </c>
     </row>
@@ -906,7 +916,7 @@
       <c r="B5" t="s">
         <v>4</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="3" t="s">
         <v>11</v>
       </c>
     </row>
@@ -917,7 +927,7 @@
       <c r="B6" t="s">
         <v>4</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="3" t="s">
         <v>13</v>
       </c>
     </row>
@@ -928,7 +938,7 @@
       <c r="B7" t="s">
         <v>4</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="3" t="s">
         <v>15</v>
       </c>
     </row>
@@ -939,7 +949,7 @@
       <c r="B8" t="s">
         <v>4</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="3" t="s">
         <v>17</v>
       </c>
     </row>
@@ -957,9 +967,9 @@
     <col min="2" max="2" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="47.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="47.83203125" style="3" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="24.5" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="91.6640625" bestFit="1" customWidth="1"/>
@@ -978,7 +988,7 @@
       <c r="D1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>21</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -1170,7 +1180,7 @@
       <c r="D10" t="s">
         <v>33</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="3" t="s">
         <v>49</v>
       </c>
       <c r="F10" t="s">
@@ -1305,7 +1315,7 @@
       <c r="D16" t="s">
         <v>33</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="3" t="s">
         <v>49</v>
       </c>
       <c r="F16" t="s">
@@ -1460,7 +1470,7 @@
       <c r="D23" t="s">
         <v>33</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="3" t="s">
         <v>49</v>
       </c>
       <c r="F23" t="s">
@@ -1618,7 +1628,7 @@
       <c r="D30" t="s">
         <v>33</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E30" s="3" t="s">
         <v>49</v>
       </c>
       <c r="F30" t="s">
@@ -1773,7 +1783,7 @@
       <c r="D37" t="s">
         <v>33</v>
       </c>
-      <c r="E37" t="s">
+      <c r="E37" s="3" t="s">
         <v>101</v>
       </c>
       <c r="F37" t="s">

</xml_diff>

<commit_message>
fix: Update bni_dbt_definitions.xlsx to reflect recent changes in data structure
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AEA1656-F8F8-A64A-A901-1546E0DBAF9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3558B712-47B7-9D4A-B655-B66F96CA2773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -968,7 +968,7 @@
     <col min="3" max="3" width="12.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="47.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="24.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="24.5" bestFit="1" customWidth="1"/>
@@ -991,7 +991,7 @@
       <c r="E1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>22</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -1183,7 +1183,7 @@
       <c r="E10" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="3" t="s">
         <v>50</v>
       </c>
       <c r="H10" t="s">
@@ -1318,7 +1318,7 @@
       <c r="E16" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="3" t="s">
         <v>50</v>
       </c>
       <c r="H16" t="s">
@@ -1473,7 +1473,7 @@
       <c r="E23" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F23" s="3" t="s">
         <v>50</v>
       </c>
       <c r="H23" t="s">
@@ -1631,7 +1631,7 @@
       <c r="E30" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F30" s="3" t="s">
         <v>50</v>
       </c>
       <c r="H30" t="s">
@@ -1786,7 +1786,7 @@
       <c r="E37" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="F37" t="s">
+      <c r="F37" s="3" t="s">
         <v>50</v>
       </c>
       <c r="H37" t="s">

</xml_diff>

<commit_message>
fix: Add YAML and JSON generation scripts for schema definitions and golden queries from Excel
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3558B712-47B7-9D4A-B655-B66F96CA2773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76675445-7905-4C4B-9268-2AD33BD61849}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,13 +16,14 @@
     <sheet name="Tables" sheetId="1" r:id="rId1"/>
     <sheet name="Columns" sheetId="2" r:id="rId2"/>
     <sheet name="Value_Mappings" sheetId="3" r:id="rId3"/>
+    <sheet name="Golden_Queries" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="167">
   <si>
     <t>Table Name</t>
   </si>
@@ -484,13 +485,52 @@
   </si>
   <si>
     <t>sum, average</t>
+  </si>
+  <si>
+    <t>user_intent</t>
+  </si>
+  <si>
+    <t>Show customers who have a birthday this week</t>
+  </si>
+  <si>
+    <t>Show deposits approaching maturity in the next 7 days</t>
+  </si>
+  <si>
+    <t>Show active customers with their savings balance</t>
+  </si>
+  <si>
+    <t>Show top 5 customers with highest savings balance</t>
+  </si>
+  <si>
+    <t>SELECT customer_id, first_name, last_name, birth_date FROM cai_customers WHERE weekofyear(birth_date) = weekofyear(current_date());</t>
+  </si>
+  <si>
+    <t>SELECT deposit_id, customer_id, principal_amount, maturity_date FROM cai_deposits WHERE maturity_date BETWEEN current_date() AND days_add(current_date(), 7);</t>
+  </si>
+  <si>
+    <t>SELECT c.customer_id, c.first_name, c.last_name, s.balance FROM cai_customers c INNER JOIN cai_savings s ON c.customer_id = s.customer_id WHERE s.status = 'ACTIVE';</t>
+  </si>
+  <si>
+    <t>SELECT c.customer_id, c.first_name, c.last_name, s.balance FROM cai_customers c INNER JOIN cai_savings s ON c.customer_id = s.customer_id ORDER BY s.balance DESC LIMIT 5;</t>
+  </si>
+  <si>
+    <t>complexity</t>
+  </si>
+  <si>
+    <t>sql_template</t>
+  </si>
+  <si>
+    <t>simple</t>
+  </si>
+  <si>
+    <t>medium</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -504,19 +544,21 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -546,15 +588,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -862,7 +905,7 @@
   <cols>
     <col min="1" max="1" width="20.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="88.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="88.6640625" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -872,7 +915,7 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
     </row>
@@ -883,7 +926,7 @@
       <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>5</v>
       </c>
     </row>
@@ -894,7 +937,7 @@
       <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>7</v>
       </c>
     </row>
@@ -905,7 +948,7 @@
       <c r="B4" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>9</v>
       </c>
     </row>
@@ -916,7 +959,7 @@
       <c r="B5" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>11</v>
       </c>
     </row>
@@ -927,7 +970,7 @@
       <c r="B6" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>13</v>
       </c>
     </row>
@@ -938,7 +981,7 @@
       <c r="B7" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>15</v>
       </c>
     </row>
@@ -949,7 +992,7 @@
       <c r="B8" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>17</v>
       </c>
     </row>
@@ -967,9 +1010,9 @@
     <col min="2" max="2" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="47.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="47.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.33203125" style="4" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="24.5" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="91.6640625" bestFit="1" customWidth="1"/>
@@ -988,13 +1031,13 @@
       <c r="D1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>23</v>
       </c>
       <c r="H1" s="1" t="s">
@@ -1180,10 +1223,10 @@
       <c r="D10" t="s">
         <v>33</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="4" t="s">
         <v>50</v>
       </c>
       <c r="H10" t="s">
@@ -1226,7 +1269,7 @@
       <c r="D12" t="s">
         <v>33</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="4" t="s">
         <v>151</v>
       </c>
       <c r="H12" t="s">
@@ -1249,7 +1292,7 @@
       <c r="D13" t="s">
         <v>33</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13" s="4" t="s">
         <v>152</v>
       </c>
       <c r="H13" t="s">
@@ -1315,10 +1358,10 @@
       <c r="D16" t="s">
         <v>33</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="F16" s="4" t="s">
         <v>50</v>
       </c>
       <c r="H16" t="s">
@@ -1361,7 +1404,7 @@
       <c r="D18" t="s">
         <v>33</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G18" s="4" t="s">
         <v>151</v>
       </c>
       <c r="H18" t="s">
@@ -1404,7 +1447,7 @@
       <c r="D20" t="s">
         <v>33</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G20" s="4" t="s">
         <v>152</v>
       </c>
       <c r="H20" t="s">
@@ -1470,10 +1513,10 @@
       <c r="D23" t="s">
         <v>33</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E23" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="F23" s="4" t="s">
         <v>50</v>
       </c>
       <c r="H23" t="s">
@@ -1519,7 +1562,7 @@
       <c r="D25" t="s">
         <v>33</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G25" s="4" t="s">
         <v>151</v>
       </c>
       <c r="H25" t="s">
@@ -1542,7 +1585,7 @@
       <c r="D26" t="s">
         <v>33</v>
       </c>
-      <c r="G26" t="s">
+      <c r="G26" s="4" t="s">
         <v>151</v>
       </c>
       <c r="H26" t="s">
@@ -1628,10 +1671,10 @@
       <c r="D30" t="s">
         <v>33</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="E30" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F30" s="3" t="s">
+      <c r="F30" s="4" t="s">
         <v>50</v>
       </c>
       <c r="H30" t="s">
@@ -1674,7 +1717,7 @@
       <c r="D32" t="s">
         <v>33</v>
       </c>
-      <c r="G32" t="s">
+      <c r="G32" s="4" t="s">
         <v>153</v>
       </c>
       <c r="H32" t="s">
@@ -1697,7 +1740,7 @@
       <c r="D33" t="s">
         <v>33</v>
       </c>
-      <c r="G33" t="s">
+      <c r="G33" s="4" t="s">
         <v>151</v>
       </c>
       <c r="H33" t="s">
@@ -1783,10 +1826,10 @@
       <c r="D37" t="s">
         <v>33</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="E37" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="F37" s="3" t="s">
+      <c r="F37" s="4" t="s">
         <v>50</v>
       </c>
       <c r="H37" t="s">
@@ -1809,7 +1852,7 @@
       <c r="D38" t="s">
         <v>33</v>
       </c>
-      <c r="G38" t="s">
+      <c r="G38" s="4" t="s">
         <v>151</v>
       </c>
       <c r="H38" t="s">
@@ -1955,7 +1998,7 @@
       <c r="D45" t="s">
         <v>33</v>
       </c>
-      <c r="G45" t="s">
+      <c r="G45" s="4" t="s">
         <v>153</v>
       </c>
       <c r="H45" t="s">
@@ -1978,7 +2021,7 @@
       <c r="D46" t="s">
         <v>33</v>
       </c>
-      <c r="G46" t="s">
+      <c r="G46" s="4" t="s">
         <v>152</v>
       </c>
       <c r="H46" t="s">
@@ -2161,4 +2204,73 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30159596-74E1-AB4A-8605-D929B81467D2}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="43.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="136.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>156</v>
+      </c>
+      <c r="B3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>157</v>
+      </c>
+      <c r="B4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>158</v>
+      </c>
+      <c r="B5" t="s">
+        <v>162</v>
+      </c>
+      <c r="C5" t="s">
+        <v>166</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Update schema definitions and dbt models for mapping_group_whs
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{608A48B2-363E-3147-A1EB-4A3DC06AFDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43160542-1978-044F-B21D-DBF3FBC5340F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="31980" windowHeight="19740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9295,7 +9295,7 @@
         <v>58</v>
       </c>
       <c r="E341" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I341" t="s">
         <v>11</v>
@@ -9332,7 +9332,7 @@
         <v>37</v>
       </c>
       <c r="D343" t="s">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="E343" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
feat: Enhance time dimension detection and update primary entity definitions in dbt schema
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43160542-1978-044F-B21D-DBF3FBC5340F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{615A734B-D3C6-2348-938D-BF65D15F1327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="31980" windowHeight="19740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9295,7 +9295,7 @@
         <v>58</v>
       </c>
       <c r="E341" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I341" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
feat: Update descriptions in YAML files to include LLM context for clarity and enhanced metadata
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15ACD5B8-D68E-8849-A987-C9A3C752E579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52F8945F-0B71-8D40-90AC-26FB67AE523A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="700" windowWidth="33720" windowHeight="19740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="680" yWindow="700" windowWidth="33720" windowHeight="19740" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tables" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1809" uniqueCount="595">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1874" uniqueCount="628">
   <si>
     <t>Table Name</t>
   </si>
@@ -1811,6 +1811,105 @@
   </si>
   <si>
     <t>Agg Time Dimension</t>
+  </si>
+  <si>
+    <t>API</t>
+  </si>
+  <si>
+    <t>ACQUIRING</t>
+  </si>
+  <si>
+    <t>SPAN</t>
+  </si>
+  <si>
+    <t>WONDR</t>
+  </si>
+  <si>
+    <t>TELLER</t>
+  </si>
+  <si>
+    <t>SMS</t>
+  </si>
+  <si>
+    <t>OTHERS</t>
+  </si>
+  <si>
+    <t>BOP</t>
+  </si>
+  <si>
+    <t>AUTODEBET</t>
+  </si>
+  <si>
+    <t>EDC_NON_BNI</t>
+  </si>
+  <si>
+    <t>NEW_MOB</t>
+  </si>
+  <si>
+    <t>REMITTANCE</t>
+  </si>
+  <si>
+    <t>AGEN_TRX</t>
+  </si>
+  <si>
+    <t>BNIDIRECT</t>
+  </si>
+  <si>
+    <t>ATM</t>
+  </si>
+  <si>
+    <t>NON API</t>
+  </si>
+  <si>
+    <t>Transaksi via Teller</t>
+  </si>
+  <si>
+    <t>Transaksi via Wonder / WONDR</t>
+  </si>
+  <si>
+    <t>Transaksi via SMS</t>
+  </si>
+  <si>
+    <t>Transaksi lainnya</t>
+  </si>
+  <si>
+    <t>Transaksi via Autodebet</t>
+  </si>
+  <si>
+    <t>Transaksi via EDC Non BNI (EDC Bank Lain)</t>
+  </si>
+  <si>
+    <t>Transaksi Remittance</t>
+  </si>
+  <si>
+    <t>Transaksi via Agen</t>
+  </si>
+  <si>
+    <t>Transaksi via BNI Direct</t>
+  </si>
+  <si>
+    <t>Transaksi Non API</t>
+  </si>
+  <si>
+    <t>Transaksi via ATM</t>
+  </si>
+  <si>
+    <t>Transaksi API</t>
+  </si>
+  <si>
+    <t>Transaksi Acquiring</t>
+  </si>
+  <si>
+    <t>Transaksi SPAN</t>
+  </si>
+  <si>
+    <t>Transaksi BOP</t>
+  </si>
+  <si>
+    <t>Transaksi New MOB</t>
+  </si>
+  <si>
+    <t>Wonder</t>
   </si>
 </sst>
 </file>
@@ -2647,7 +2746,7 @@
         <v>0</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>10</v>
+        <v>593</v>
       </c>
       <c r="J17" s="4" t="s">
         <v>348</v>
@@ -9349,14 +9448,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="50" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="32.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
@@ -9388,6 +9487,233 @@
       </c>
       <c r="D2" t="s">
         <v>592</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C3" t="s">
+        <v>595</v>
+      </c>
+      <c r="E3" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" t="s">
+        <v>596</v>
+      </c>
+      <c r="E4" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" t="s">
+        <v>597</v>
+      </c>
+      <c r="E5" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" t="s">
+        <v>598</v>
+      </c>
+      <c r="D6" t="s">
+        <v>627</v>
+      </c>
+      <c r="E6" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" t="s">
+        <v>599</v>
+      </c>
+      <c r="E7" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" t="s">
+        <v>600</v>
+      </c>
+      <c r="E8" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" t="s">
+        <v>601</v>
+      </c>
+      <c r="E9" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A10" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" t="s">
+        <v>602</v>
+      </c>
+      <c r="E10" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" t="s">
+        <v>603</v>
+      </c>
+      <c r="E11" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A12" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" t="s">
+        <v>604</v>
+      </c>
+      <c r="E12" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A13" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" t="s">
+        <v>605</v>
+      </c>
+      <c r="E13" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A14" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C14" t="s">
+        <v>606</v>
+      </c>
+      <c r="E14" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A15" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" t="s">
+        <v>607</v>
+      </c>
+      <c r="E15" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A16" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C16" t="s">
+        <v>608</v>
+      </c>
+      <c r="E16" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A17" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C17" t="s">
+        <v>610</v>
+      </c>
+      <c r="E17" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A18" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C18" t="s">
+        <v>609</v>
+      </c>
+      <c r="E18" t="s">
+        <v>621</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Update litellm_config.yaml to remove unused parameters and standardize retry count
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52F8945F-0B71-8D40-90AC-26FB67AE523A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09E0F96A-74B0-7B4F-8481-A29AA6D275EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="700" windowWidth="33720" windowHeight="19740" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="680" yWindow="700" windowWidth="33720" windowHeight="19740" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tables" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1874" uniqueCount="628">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1875" uniqueCount="629">
   <si>
     <t>Table Name</t>
   </si>
@@ -1910,6 +1910,9 @@
   </si>
   <si>
     <t>Wonder</t>
+  </si>
+  <si>
+    <t>Tampilkan cash out</t>
   </si>
 </sst>
 </file>
@@ -9723,7 +9726,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30159596-74E1-AB4A-8605-D929B81467D2}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="43.1640625" bestFit="1" customWidth="1"/>
@@ -9752,6 +9755,11 @@
         <v>21</v>
       </c>
     </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>628</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Update schema and query definitions for clarity and consistency in descriptions
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09E0F96A-74B0-7B4F-8481-A29AA6D275EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9E7EE77-5D8C-834B-B59D-13A2D31AD240}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="700" windowWidth="33720" windowHeight="19740" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="680" yWindow="660" windowWidth="33720" windowHeight="19740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tables" sheetId="1" r:id="rId1"/>
@@ -1027,9 +1027,6 @@
     <t>group_principal</t>
   </si>
   <si>
-    <t>Tanggal Data</t>
-  </si>
-  <si>
     <t>Waktu Transaksi</t>
   </si>
   <si>
@@ -1069,9 +1066,6 @@
     <t>No Jurnal Transaksi</t>
   </si>
   <si>
-    <t>Nilai Transaksi</t>
-  </si>
-  <si>
     <t>Channel Transaksi</t>
   </si>
   <si>
@@ -1913,6 +1907,12 @@
   </si>
   <si>
     <t>Tampilkan cash out</t>
+  </si>
+  <si>
+    <t>Nilai Transaksi / Amount</t>
+  </si>
+  <si>
+    <t>Tanggal Transaksi Data, digunakan untuk filter tanggal, bulan, tahun</t>
   </si>
 </sst>
 </file>
@@ -2329,7 +2329,7 @@
         <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -2340,7 +2340,7 @@
         <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -2351,18 +2351,18 @@
         <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="B6" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="C6" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
     </row>
   </sheetData>
@@ -2402,7 +2402,7 @@
         <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>6</v>
@@ -2440,7 +2440,7 @@
         <v>10</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>333</v>
+        <v>628</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2460,7 +2460,7 @@
         <v>10</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2477,13 +2477,13 @@
         <v>0</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="32" x14ac:dyDescent="0.2">
@@ -2500,13 +2500,13 @@
         <v>0</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2526,7 +2526,7 @@
         <v>10</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2546,7 +2546,7 @@
         <v>10</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2566,7 +2566,7 @@
         <v>10</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2586,7 +2586,7 @@
         <v>10</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2606,7 +2606,7 @@
         <v>10</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2626,7 +2626,7 @@
         <v>10</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2646,7 +2646,7 @@
         <v>10</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2666,7 +2666,7 @@
         <v>10</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2686,7 +2686,7 @@
         <v>10</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2703,13 +2703,13 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2732,7 +2732,7 @@
         <v>10</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>347</v>
+        <v>627</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2749,10 +2749,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2772,7 +2772,7 @@
         <v>10</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2792,7 +2792,7 @@
         <v>10</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2812,7 +2812,7 @@
         <v>10</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2832,7 +2832,7 @@
         <v>10</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2852,7 +2852,7 @@
         <v>10</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2872,7 +2872,7 @@
         <v>10</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2892,7 +2892,7 @@
         <v>10</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2912,7 +2912,7 @@
         <v>10</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2932,7 +2932,7 @@
         <v>10</v>
       </c>
       <c r="J26" s="4" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2952,7 +2952,7 @@
         <v>10</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2972,7 +2972,7 @@
         <v>10</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2989,13 +2989,13 @@
         <v>0</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="H29" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J29" s="4" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="32" x14ac:dyDescent="0.2">
@@ -3012,13 +3012,13 @@
         <v>0</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="H30" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J30" s="4" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3038,7 +3038,7 @@
         <v>10</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3058,7 +3058,7 @@
         <v>10</v>
       </c>
       <c r="J32" s="4" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3078,7 +3078,7 @@
         <v>10</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3098,7 +3098,7 @@
         <v>10</v>
       </c>
       <c r="J34" s="4" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3118,7 +3118,7 @@
         <v>10</v>
       </c>
       <c r="J35" s="4" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3138,7 +3138,7 @@
         <v>10</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3158,7 +3158,7 @@
         <v>10</v>
       </c>
       <c r="J37" s="4" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="38" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3178,7 +3178,7 @@
         <v>10</v>
       </c>
       <c r="J38" s="4" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3201,7 +3201,7 @@
         <v>10</v>
       </c>
       <c r="J39" s="4" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3221,7 +3221,7 @@
         <v>10</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3241,7 +3241,7 @@
         <v>10</v>
       </c>
       <c r="J41" s="4" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3261,7 +3261,7 @@
         <v>10</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3281,7 +3281,7 @@
         <v>10</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3301,7 +3301,7 @@
         <v>10</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3321,7 +3321,7 @@
         <v>10</v>
       </c>
       <c r="J45" s="4" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="46" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3344,7 +3344,7 @@
         <v>10</v>
       </c>
       <c r="J46" s="4" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="47" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3364,7 +3364,7 @@
         <v>10</v>
       </c>
       <c r="J47" s="4" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="48" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3384,7 +3384,7 @@
         <v>10</v>
       </c>
       <c r="J48" s="4" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3404,7 +3404,7 @@
         <v>10</v>
       </c>
       <c r="J49" s="4" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3424,7 +3424,7 @@
         <v>10</v>
       </c>
       <c r="J50" s="4" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3444,7 +3444,7 @@
         <v>10</v>
       </c>
       <c r="J51" s="4" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="52" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3461,13 +3461,13 @@
         <v>0</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="J52" s="4" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="53" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3487,7 +3487,7 @@
         <v>10</v>
       </c>
       <c r="J53" s="4" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="54" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3507,7 +3507,7 @@
         <v>10</v>
       </c>
       <c r="J54" s="4" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="55" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3527,7 +3527,7 @@
         <v>10</v>
       </c>
       <c r="J55" s="4" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
     </row>
     <row r="56" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3547,7 +3547,7 @@
         <v>10</v>
       </c>
       <c r="J56" s="4" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="57" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3567,7 +3567,7 @@
         <v>10</v>
       </c>
       <c r="J57" s="4" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="58" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3587,7 +3587,7 @@
         <v>10</v>
       </c>
       <c r="J58" s="4" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="59" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3607,7 +3607,7 @@
         <v>10</v>
       </c>
       <c r="J59" s="4" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="60" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3627,7 +3627,7 @@
         <v>10</v>
       </c>
       <c r="J60" s="4" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="61" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3647,7 +3647,7 @@
         <v>10</v>
       </c>
       <c r="J61" s="4" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="62" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3667,7 +3667,7 @@
         <v>10</v>
       </c>
       <c r="J62" s="4" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="63" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3687,7 +3687,7 @@
         <v>10</v>
       </c>
       <c r="J63" s="4" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="64" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3707,7 +3707,7 @@
         <v>10</v>
       </c>
       <c r="J64" s="4" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="65" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3727,7 +3727,7 @@
         <v>10</v>
       </c>
       <c r="J65" s="4" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="66" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3747,7 +3747,7 @@
         <v>10</v>
       </c>
       <c r="J66" s="4" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="67" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3770,7 +3770,7 @@
         <v>10</v>
       </c>
       <c r="J67" s="4" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="68" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3790,7 +3790,7 @@
         <v>10</v>
       </c>
       <c r="J68" s="4" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="69" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3810,7 +3810,7 @@
         <v>10</v>
       </c>
       <c r="J69" s="4" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="70" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3830,7 +3830,7 @@
         <v>10</v>
       </c>
       <c r="J70" s="4" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="71" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3850,7 +3850,7 @@
         <v>10</v>
       </c>
       <c r="J71" s="4" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="72" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3870,7 +3870,7 @@
         <v>10</v>
       </c>
       <c r="J72" s="4" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="73" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3890,7 +3890,7 @@
         <v>10</v>
       </c>
       <c r="J73" s="4" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="74" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3910,7 +3910,7 @@
         <v>10</v>
       </c>
       <c r="J74" s="4" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="75" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3930,7 +3930,7 @@
         <v>10</v>
       </c>
       <c r="J75" s="4" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="76" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3950,7 +3950,7 @@
         <v>10</v>
       </c>
       <c r="J76" s="4" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="77" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3970,7 +3970,7 @@
         <v>10</v>
       </c>
       <c r="J77" s="4" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="78" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3990,7 +3990,7 @@
         <v>10</v>
       </c>
       <c r="J78" s="4" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="79" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4010,7 +4010,7 @@
         <v>10</v>
       </c>
       <c r="J79" s="4" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="80" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4030,7 +4030,7 @@
         <v>10</v>
       </c>
       <c r="J80" s="4" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="81" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4050,7 +4050,7 @@
         <v>10</v>
       </c>
       <c r="J81" s="4" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="82" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4104,7 +4104,7 @@
         <v>10</v>
       </c>
       <c r="J84" s="4" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="85" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4175,7 +4175,7 @@
         <v>10</v>
       </c>
       <c r="J88" s="4" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="89" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4195,7 +4195,7 @@
         <v>10</v>
       </c>
       <c r="J89" s="4" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="90" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4215,7 +4215,7 @@
         <v>10</v>
       </c>
       <c r="J90" s="4" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="91" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4235,7 +4235,7 @@
         <v>10</v>
       </c>
       <c r="J91" s="4" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="92" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4255,7 +4255,7 @@
         <v>10</v>
       </c>
       <c r="J92" s="4" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="93" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4275,7 +4275,7 @@
         <v>10</v>
       </c>
       <c r="J93" s="4" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="94" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4295,7 +4295,7 @@
         <v>10</v>
       </c>
       <c r="J94" s="4" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
     </row>
     <row r="95" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4315,7 +4315,7 @@
         <v>10</v>
       </c>
       <c r="J95" s="4" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="96" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4335,7 +4335,7 @@
         <v>10</v>
       </c>
       <c r="J96" s="4" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
     <row r="97" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4355,7 +4355,7 @@
         <v>10</v>
       </c>
       <c r="J97" s="4" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="98" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4375,7 +4375,7 @@
         <v>10</v>
       </c>
       <c r="J98" s="4" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="99" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4395,7 +4395,7 @@
         <v>10</v>
       </c>
       <c r="J99" s="4" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="100" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4415,7 +4415,7 @@
         <v>10</v>
       </c>
       <c r="J100" s="4" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
     </row>
     <row r="101" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4452,7 +4452,7 @@
         <v>10</v>
       </c>
       <c r="J102" s="4" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="103" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4472,7 +4472,7 @@
         <v>10</v>
       </c>
       <c r="J103" s="4" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
     </row>
     <row r="104" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4495,7 +4495,7 @@
         <v>10</v>
       </c>
       <c r="J104" s="4" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="105" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4555,7 +4555,7 @@
         <v>10</v>
       </c>
       <c r="J107" s="4" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="108" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4609,7 +4609,7 @@
         <v>10</v>
       </c>
       <c r="J110" s="4" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="111" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4629,7 +4629,7 @@
         <v>10</v>
       </c>
       <c r="J111" s="4" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="112" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4649,7 +4649,7 @@
         <v>10</v>
       </c>
       <c r="J112" s="4" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
     </row>
     <row r="113" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4669,7 +4669,7 @@
         <v>10</v>
       </c>
       <c r="J113" s="4" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="114" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4689,7 +4689,7 @@
         <v>10</v>
       </c>
       <c r="J114" s="4" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
     <row r="115" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4709,7 +4709,7 @@
         <v>10</v>
       </c>
       <c r="J115" s="4" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
     </row>
     <row r="116" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4729,7 +4729,7 @@
         <v>10</v>
       </c>
       <c r="J116" s="4" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
     </row>
     <row r="117" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4749,7 +4749,7 @@
         <v>10</v>
       </c>
       <c r="J117" s="4" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
     </row>
     <row r="118" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4769,7 +4769,7 @@
         <v>10</v>
       </c>
       <c r="J118" s="4" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="119" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4789,7 +4789,7 @@
         <v>10</v>
       </c>
       <c r="J119" s="4" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
     </row>
     <row r="120" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4809,7 +4809,7 @@
         <v>10</v>
       </c>
       <c r="J120" s="4" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="121" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4829,7 +4829,7 @@
         <v>10</v>
       </c>
       <c r="J121" s="4" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
     </row>
     <row r="122" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4849,7 +4849,7 @@
         <v>10</v>
       </c>
       <c r="J122" s="4" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="123" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4869,7 +4869,7 @@
         <v>10</v>
       </c>
       <c r="J123" s="4" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
     </row>
     <row r="124" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4889,7 +4889,7 @@
         <v>10</v>
       </c>
       <c r="J124" s="4" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
     </row>
     <row r="125" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4909,7 +4909,7 @@
         <v>10</v>
       </c>
       <c r="J125" s="4" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
     </row>
     <row r="126" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4929,7 +4929,7 @@
         <v>10</v>
       </c>
       <c r="J126" s="4" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
     </row>
     <row r="127" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4949,7 +4949,7 @@
         <v>10</v>
       </c>
       <c r="J127" s="4" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
     </row>
     <row r="128" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4969,7 +4969,7 @@
         <v>10</v>
       </c>
       <c r="J128" s="4" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
     </row>
     <row r="129" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4989,7 +4989,7 @@
         <v>10</v>
       </c>
       <c r="J129" s="4" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
     </row>
     <row r="130" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5009,7 +5009,7 @@
         <v>10</v>
       </c>
       <c r="J130" s="4" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
     </row>
     <row r="131" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5029,7 +5029,7 @@
         <v>10</v>
       </c>
       <c r="J131" s="4" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
     </row>
     <row r="132" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5049,7 +5049,7 @@
         <v>10</v>
       </c>
       <c r="J132" s="4" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
     </row>
     <row r="133" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5069,7 +5069,7 @@
         <v>10</v>
       </c>
       <c r="J133" s="4" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
     </row>
     <row r="134" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5089,7 +5089,7 @@
         <v>10</v>
       </c>
       <c r="J134" s="4" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
     </row>
     <row r="135" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5109,7 +5109,7 @@
         <v>10</v>
       </c>
       <c r="J135" s="4" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
     </row>
     <row r="136" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5129,7 +5129,7 @@
         <v>10</v>
       </c>
       <c r="J136" s="4" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
     </row>
     <row r="137" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5149,7 +5149,7 @@
         <v>10</v>
       </c>
       <c r="J137" s="4" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
     </row>
     <row r="138" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5169,7 +5169,7 @@
         <v>10</v>
       </c>
       <c r="J138" s="4" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
     </row>
     <row r="139" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5189,7 +5189,7 @@
         <v>10</v>
       </c>
       <c r="J139" s="4" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
     </row>
     <row r="140" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5209,7 +5209,7 @@
         <v>10</v>
       </c>
       <c r="J140" s="4" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
     </row>
     <row r="141" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5226,13 +5226,13 @@
         <v>0</v>
       </c>
       <c r="F141" s="4" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="H141" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J141" s="4" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
     </row>
     <row r="142" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5252,7 +5252,7 @@
         <v>10</v>
       </c>
       <c r="J142" s="4" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="143" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5272,7 +5272,7 @@
         <v>10</v>
       </c>
       <c r="J143" s="4" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
     </row>
     <row r="144" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5292,7 +5292,7 @@
         <v>10</v>
       </c>
       <c r="J144" s="4" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
     </row>
     <row r="145" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5312,7 +5312,7 @@
         <v>10</v>
       </c>
       <c r="J145" s="4" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
     <row r="146" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5332,7 +5332,7 @@
         <v>10</v>
       </c>
       <c r="J146" s="4" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
     </row>
     <row r="147" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5352,7 +5352,7 @@
         <v>10</v>
       </c>
       <c r="J147" s="4" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
     <row r="148" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5372,7 +5372,7 @@
         <v>10</v>
       </c>
       <c r="J148" s="4" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
     <row r="149" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5392,7 +5392,7 @@
         <v>10</v>
       </c>
       <c r="J149" s="4" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
     </row>
     <row r="150" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5412,7 +5412,7 @@
         <v>10</v>
       </c>
       <c r="J150" s="4" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="151" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5432,7 +5432,7 @@
         <v>10</v>
       </c>
       <c r="J151" s="4" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
     </row>
     <row r="152" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5452,7 +5452,7 @@
         <v>10</v>
       </c>
       <c r="J152" s="4" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
     </row>
     <row r="153" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5472,7 +5472,7 @@
         <v>10</v>
       </c>
       <c r="J153" s="4" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
     </row>
     <row r="154" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5492,7 +5492,7 @@
         <v>10</v>
       </c>
       <c r="J154" s="4" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="155" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5512,7 +5512,7 @@
         <v>10</v>
       </c>
       <c r="J155" s="4" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="156" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5532,7 +5532,7 @@
         <v>10</v>
       </c>
       <c r="J156" s="4" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
     </row>
     <row r="157" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5552,7 +5552,7 @@
         <v>10</v>
       </c>
       <c r="J157" s="4" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
     </row>
     <row r="158" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5572,7 +5572,7 @@
         <v>10</v>
       </c>
       <c r="J158" s="4" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="159" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5592,7 +5592,7 @@
         <v>10</v>
       </c>
       <c r="J159" s="4" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="160" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5612,7 +5612,7 @@
         <v>10</v>
       </c>
       <c r="J160" s="4" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="161" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5632,7 +5632,7 @@
         <v>10</v>
       </c>
       <c r="J161" s="4" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
     </row>
     <row r="162" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5652,7 +5652,7 @@
         <v>10</v>
       </c>
       <c r="J162" s="4" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="163" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5672,7 +5672,7 @@
         <v>10</v>
       </c>
       <c r="J163" s="4" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
     </row>
     <row r="164" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5692,7 +5692,7 @@
         <v>10</v>
       </c>
       <c r="J164" s="4" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="165" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5712,7 +5712,7 @@
         <v>10</v>
       </c>
       <c r="J165" s="4" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
     </row>
     <row r="166" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5732,7 +5732,7 @@
         <v>10</v>
       </c>
       <c r="J166" s="4" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="167" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5755,7 +5755,7 @@
         <v>10</v>
       </c>
       <c r="J167" s="4" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="168" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5775,7 +5775,7 @@
         <v>10</v>
       </c>
       <c r="J168" s="4" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="169" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5795,7 +5795,7 @@
         <v>10</v>
       </c>
       <c r="J169" s="4" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="170" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5815,7 +5815,7 @@
         <v>10</v>
       </c>
       <c r="J170" s="4" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
     </row>
     <row r="171" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5835,7 +5835,7 @@
         <v>10</v>
       </c>
       <c r="J171" s="4" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="172" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5855,7 +5855,7 @@
         <v>10</v>
       </c>
       <c r="J172" s="4" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
     </row>
     <row r="173" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5875,7 +5875,7 @@
         <v>10</v>
       </c>
       <c r="J173" s="4" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
     </row>
     <row r="174" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5895,7 +5895,7 @@
         <v>10</v>
       </c>
       <c r="J174" s="4" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="175" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5915,7 +5915,7 @@
         <v>10</v>
       </c>
       <c r="J175" s="4" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="176" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5935,7 +5935,7 @@
         <v>10</v>
       </c>
       <c r="J176" s="4" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="177" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5955,7 +5955,7 @@
         <v>10</v>
       </c>
       <c r="J177" s="4" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
     </row>
     <row r="178" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5975,7 +5975,7 @@
         <v>10</v>
       </c>
       <c r="J178" s="4" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
     </row>
     <row r="179" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5998,7 +5998,7 @@
         <v>10</v>
       </c>
       <c r="J179" s="4" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="180" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6021,7 +6021,7 @@
         <v>10</v>
       </c>
       <c r="J180" s="4" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
     </row>
     <row r="181" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6044,7 +6044,7 @@
         <v>10</v>
       </c>
       <c r="J181" s="4" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
     </row>
     <row r="182" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6067,7 +6067,7 @@
         <v>10</v>
       </c>
       <c r="J182" s="4" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
     </row>
     <row r="183" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6090,7 +6090,7 @@
         <v>10</v>
       </c>
       <c r="J183" s="4" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
     </row>
     <row r="184" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6110,7 +6110,7 @@
         <v>10</v>
       </c>
       <c r="J184" s="4" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
     </row>
     <row r="185" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6130,7 +6130,7 @@
         <v>10</v>
       </c>
       <c r="J185" s="4" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
     </row>
     <row r="186" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6150,7 +6150,7 @@
         <v>10</v>
       </c>
       <c r="J186" s="4" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
     </row>
     <row r="187" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6170,7 +6170,7 @@
         <v>10</v>
       </c>
       <c r="J187" s="4" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
     </row>
     <row r="188" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6190,7 +6190,7 @@
         <v>10</v>
       </c>
       <c r="J188" s="4" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
     </row>
     <row r="189" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6210,7 +6210,7 @@
         <v>10</v>
       </c>
       <c r="J189" s="4" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
     </row>
     <row r="190" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6230,7 +6230,7 @@
         <v>10</v>
       </c>
       <c r="J190" s="4" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
     </row>
     <row r="191" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6250,7 +6250,7 @@
         <v>10</v>
       </c>
       <c r="J191" s="4" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
     </row>
     <row r="192" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6270,7 +6270,7 @@
         <v>10</v>
       </c>
       <c r="J192" s="4" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="193" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6290,7 +6290,7 @@
         <v>10</v>
       </c>
       <c r="J193" s="4" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
     </row>
     <row r="194" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6310,7 +6310,7 @@
         <v>10</v>
       </c>
       <c r="J194" s="4" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
     </row>
     <row r="195" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6330,7 +6330,7 @@
         <v>10</v>
       </c>
       <c r="J195" s="4" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
     <row r="196" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6350,7 +6350,7 @@
         <v>10</v>
       </c>
       <c r="J196" s="4" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
     </row>
     <row r="197" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6370,7 +6370,7 @@
         <v>10</v>
       </c>
       <c r="J197" s="4" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
     </row>
     <row r="198" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6390,7 +6390,7 @@
         <v>10</v>
       </c>
       <c r="J198" s="4" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
     </row>
     <row r="199" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6410,7 +6410,7 @@
         <v>10</v>
       </c>
       <c r="J199" s="4" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
     </row>
     <row r="200" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6430,7 +6430,7 @@
         <v>10</v>
       </c>
       <c r="J200" s="4" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="201" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6450,7 +6450,7 @@
         <v>10</v>
       </c>
       <c r="J201" s="4" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
     </row>
     <row r="202" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6473,7 +6473,7 @@
         <v>10</v>
       </c>
       <c r="J202" s="4" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
     </row>
     <row r="203" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6496,7 +6496,7 @@
         <v>10</v>
       </c>
       <c r="J203" s="4" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
     </row>
     <row r="204" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6519,7 +6519,7 @@
         <v>10</v>
       </c>
       <c r="J204" s="4" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
     </row>
     <row r="205" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6542,7 +6542,7 @@
         <v>10</v>
       </c>
       <c r="J205" s="4" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
     </row>
     <row r="206" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6565,7 +6565,7 @@
         <v>10</v>
       </c>
       <c r="J206" s="4" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
     </row>
     <row r="207" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6588,7 +6588,7 @@
         <v>10</v>
       </c>
       <c r="J207" s="4" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
     </row>
     <row r="208" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6611,7 +6611,7 @@
         <v>10</v>
       </c>
       <c r="J208" s="4" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
     </row>
     <row r="209" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6634,7 +6634,7 @@
         <v>10</v>
       </c>
       <c r="J209" s="4" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
     </row>
     <row r="210" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6657,7 +6657,7 @@
         <v>10</v>
       </c>
       <c r="J210" s="4" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
     </row>
     <row r="211" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6680,7 +6680,7 @@
         <v>10</v>
       </c>
       <c r="J211" s="4" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
     </row>
     <row r="212" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6700,7 +6700,7 @@
         <v>10</v>
       </c>
       <c r="J212" s="4" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
     </row>
     <row r="213" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6720,7 +6720,7 @@
         <v>10</v>
       </c>
       <c r="J213" s="4" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
     </row>
     <row r="214" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6740,7 +6740,7 @@
         <v>10</v>
       </c>
       <c r="J214" s="4" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
     </row>
     <row r="215" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6763,7 +6763,7 @@
         <v>10</v>
       </c>
       <c r="J215" s="4" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
     </row>
     <row r="216" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6786,7 +6786,7 @@
         <v>10</v>
       </c>
       <c r="J216" s="4" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
     </row>
     <row r="217" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6809,7 +6809,7 @@
         <v>10</v>
       </c>
       <c r="J217" s="4" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
     </row>
     <row r="218" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6829,7 +6829,7 @@
         <v>10</v>
       </c>
       <c r="J218" s="4" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
     </row>
     <row r="219" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6849,7 +6849,7 @@
         <v>10</v>
       </c>
       <c r="J219" s="4" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
     </row>
     <row r="220" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6869,7 +6869,7 @@
         <v>10</v>
       </c>
       <c r="J220" s="4" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
     </row>
     <row r="221" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6889,7 +6889,7 @@
         <v>10</v>
       </c>
       <c r="J221" s="4" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
     </row>
     <row r="222" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6909,7 +6909,7 @@
         <v>10</v>
       </c>
       <c r="J222" s="4" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
     </row>
     <row r="223" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6929,7 +6929,7 @@
         <v>10</v>
       </c>
       <c r="J223" s="4" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
     </row>
     <row r="224" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6949,7 +6949,7 @@
         <v>10</v>
       </c>
       <c r="J224" s="4" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
     </row>
     <row r="225" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6969,7 +6969,7 @@
         <v>10</v>
       </c>
       <c r="J225" s="4" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
     </row>
     <row r="226" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6989,7 +6989,7 @@
         <v>10</v>
       </c>
       <c r="J226" s="4" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="227" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7009,7 +7009,7 @@
         <v>10</v>
       </c>
       <c r="J227" s="4" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
     </row>
     <row r="228" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7029,7 +7029,7 @@
         <v>10</v>
       </c>
       <c r="J228" s="4" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="229" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7052,7 +7052,7 @@
         <v>10</v>
       </c>
       <c r="J229" s="4" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
     </row>
     <row r="230" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7075,7 +7075,7 @@
         <v>10</v>
       </c>
       <c r="J230" s="4" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
     </row>
     <row r="231" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7098,7 +7098,7 @@
         <v>10</v>
       </c>
       <c r="J231" s="4" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
     </row>
     <row r="232" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7121,7 +7121,7 @@
         <v>10</v>
       </c>
       <c r="J232" s="4" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
     </row>
     <row r="233" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7144,7 +7144,7 @@
         <v>10</v>
       </c>
       <c r="J233" s="4" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
     </row>
     <row r="234" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7167,7 +7167,7 @@
         <v>10</v>
       </c>
       <c r="J234" s="4" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
     </row>
     <row r="235" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7190,7 +7190,7 @@
         <v>10</v>
       </c>
       <c r="J235" s="4" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
     </row>
     <row r="236" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7213,7 +7213,7 @@
         <v>10</v>
       </c>
       <c r="J236" s="4" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
     </row>
     <row r="237" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7233,7 +7233,7 @@
         <v>10</v>
       </c>
       <c r="J237" s="4" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
     </row>
     <row r="238" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7256,7 +7256,7 @@
         <v>10</v>
       </c>
       <c r="J238" s="4" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
     </row>
     <row r="239" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7276,7 +7276,7 @@
         <v>10</v>
       </c>
       <c r="J239" s="4" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
     </row>
     <row r="240" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7299,7 +7299,7 @@
         <v>10</v>
       </c>
       <c r="J240" s="4" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
     </row>
     <row r="241" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7319,7 +7319,7 @@
         <v>10</v>
       </c>
       <c r="J241" s="4" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
     </row>
     <row r="242" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7339,7 +7339,7 @@
         <v>10</v>
       </c>
       <c r="J242" s="4" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
     </row>
     <row r="243" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7356,13 +7356,13 @@
         <v>0</v>
       </c>
       <c r="F243" s="4" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="H243" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J243" s="4" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
     </row>
     <row r="244" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7382,7 +7382,7 @@
         <v>10</v>
       </c>
       <c r="J244" s="4" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
     </row>
     <row r="245" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7402,7 +7402,7 @@
         <v>10</v>
       </c>
       <c r="J245" s="4" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="246" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7422,7 +7422,7 @@
         <v>10</v>
       </c>
       <c r="J246" s="4" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
     </row>
     <row r="247" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7442,7 +7442,7 @@
         <v>10</v>
       </c>
       <c r="J247" s="4" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
     </row>
     <row r="248" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7462,7 +7462,7 @@
         <v>10</v>
       </c>
       <c r="J248" s="4" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
     <row r="249" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7482,7 +7482,7 @@
         <v>10</v>
       </c>
       <c r="J249" s="4" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
     </row>
     <row r="250" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7502,7 +7502,7 @@
         <v>10</v>
       </c>
       <c r="J250" s="4" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
     <row r="251" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7522,7 +7522,7 @@
         <v>10</v>
       </c>
       <c r="J251" s="4" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
     <row r="252" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7542,7 +7542,7 @@
         <v>10</v>
       </c>
       <c r="J252" s="4" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
     </row>
     <row r="253" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7562,7 +7562,7 @@
         <v>10</v>
       </c>
       <c r="J253" s="4" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="254" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7582,7 +7582,7 @@
         <v>10</v>
       </c>
       <c r="J254" s="4" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
     </row>
     <row r="255" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7602,7 +7602,7 @@
         <v>10</v>
       </c>
       <c r="J255" s="4" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
     </row>
     <row r="256" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7622,7 +7622,7 @@
         <v>10</v>
       </c>
       <c r="J256" s="4" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
     </row>
     <row r="257" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7642,7 +7642,7 @@
         <v>10</v>
       </c>
       <c r="J257" s="4" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="258" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7662,7 +7662,7 @@
         <v>10</v>
       </c>
       <c r="J258" s="4" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="259" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7682,7 +7682,7 @@
         <v>10</v>
       </c>
       <c r="J259" s="4" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
     </row>
     <row r="260" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7702,7 +7702,7 @@
         <v>10</v>
       </c>
       <c r="J260" s="4" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
     </row>
     <row r="261" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7722,7 +7722,7 @@
         <v>10</v>
       </c>
       <c r="J261" s="4" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="262" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7742,7 +7742,7 @@
         <v>10</v>
       </c>
       <c r="J262" s="4" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="263" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7762,7 +7762,7 @@
         <v>10</v>
       </c>
       <c r="J263" s="4" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="264" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7782,7 +7782,7 @@
         <v>10</v>
       </c>
       <c r="J264" s="4" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
     </row>
     <row r="265" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7802,7 +7802,7 @@
         <v>10</v>
       </c>
       <c r="J265" s="4" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="266" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7822,7 +7822,7 @@
         <v>10</v>
       </c>
       <c r="J266" s="4" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
     </row>
     <row r="267" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7842,7 +7842,7 @@
         <v>10</v>
       </c>
       <c r="J267" s="4" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="268" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7862,7 +7862,7 @@
         <v>10</v>
       </c>
       <c r="J268" s="4" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
     </row>
     <row r="269" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7882,7 +7882,7 @@
         <v>10</v>
       </c>
       <c r="J269" s="4" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="270" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7902,7 +7902,7 @@
         <v>10</v>
       </c>
       <c r="J270" s="4" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="271" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7922,7 +7922,7 @@
         <v>10</v>
       </c>
       <c r="J271" s="4" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="272" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7942,7 +7942,7 @@
         <v>10</v>
       </c>
       <c r="J272" s="4" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
     </row>
     <row r="273" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7962,7 +7962,7 @@
         <v>10</v>
       </c>
       <c r="J273" s="4" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="274" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7982,7 +7982,7 @@
         <v>10</v>
       </c>
       <c r="J274" s="4" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
     </row>
     <row r="275" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8002,7 +8002,7 @@
         <v>10</v>
       </c>
       <c r="J275" s="4" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="276" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8022,7 +8022,7 @@
         <v>10</v>
       </c>
       <c r="J276" s="4" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
     </row>
     <row r="277" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8042,7 +8042,7 @@
         <v>10</v>
       </c>
       <c r="J277" s="4" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="278" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8062,7 +8062,7 @@
         <v>10</v>
       </c>
       <c r="J278" s="4" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
     <row r="279" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8082,7 +8082,7 @@
         <v>10</v>
       </c>
       <c r="J279" s="4" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="280" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8102,7 +8102,7 @@
         <v>10</v>
       </c>
       <c r="J280" s="4" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
     </row>
     <row r="281" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8122,7 +8122,7 @@
         <v>10</v>
       </c>
       <c r="J281" s="4" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="282" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8142,7 +8142,7 @@
         <v>10</v>
       </c>
       <c r="J282" s="4" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
     </row>
     <row r="283" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8162,7 +8162,7 @@
         <v>10</v>
       </c>
       <c r="J283" s="4" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
     </row>
     <row r="284" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8182,7 +8182,7 @@
         <v>10</v>
       </c>
       <c r="J284" s="4" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
     </row>
     <row r="285" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8202,7 +8202,7 @@
         <v>10</v>
       </c>
       <c r="J285" s="4" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
     </row>
     <row r="286" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8222,7 +8222,7 @@
         <v>10</v>
       </c>
       <c r="J286" s="4" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
     </row>
     <row r="287" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8242,7 +8242,7 @@
         <v>10</v>
       </c>
       <c r="J287" s="4" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
     </row>
     <row r="288" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8262,7 +8262,7 @@
         <v>10</v>
       </c>
       <c r="J288" s="4" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
     </row>
     <row r="289" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8282,7 +8282,7 @@
         <v>10</v>
       </c>
       <c r="J289" s="4" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
     </row>
     <row r="290" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8302,7 +8302,7 @@
         <v>10</v>
       </c>
       <c r="J290" s="4" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
     </row>
     <row r="291" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8322,7 +8322,7 @@
         <v>10</v>
       </c>
       <c r="J291" s="4" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
     </row>
     <row r="292" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8342,7 +8342,7 @@
         <v>10</v>
       </c>
       <c r="J292" s="4" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
     </row>
     <row r="293" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8362,7 +8362,7 @@
         <v>10</v>
       </c>
       <c r="J293" s="4" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
     </row>
     <row r="294" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8382,7 +8382,7 @@
         <v>10</v>
       </c>
       <c r="J294" s="4" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="295" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8402,7 +8402,7 @@
         <v>10</v>
       </c>
       <c r="J295" s="4" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="296" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8422,7 +8422,7 @@
         <v>10</v>
       </c>
       <c r="J296" s="4" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
     </row>
     <row r="297" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8445,7 +8445,7 @@
         <v>10</v>
       </c>
       <c r="J297" s="4" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
     </row>
     <row r="298" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8468,7 +8468,7 @@
         <v>10</v>
       </c>
       <c r="J298" s="4" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
     </row>
     <row r="299" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8491,7 +8491,7 @@
         <v>10</v>
       </c>
       <c r="J299" s="4" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
     </row>
     <row r="300" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8514,7 +8514,7 @@
         <v>10</v>
       </c>
       <c r="J300" s="4" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
     </row>
     <row r="301" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8537,7 +8537,7 @@
         <v>10</v>
       </c>
       <c r="J301" s="4" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
     </row>
     <row r="302" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8560,7 +8560,7 @@
         <v>10</v>
       </c>
       <c r="J302" s="4" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
     </row>
     <row r="303" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8583,7 +8583,7 @@
         <v>10</v>
       </c>
       <c r="J303" s="4" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
     </row>
     <row r="304" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8606,7 +8606,7 @@
         <v>10</v>
       </c>
       <c r="J304" s="4" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
     </row>
     <row r="305" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8629,7 +8629,7 @@
         <v>10</v>
       </c>
       <c r="J305" s="4" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
     </row>
     <row r="306" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8652,7 +8652,7 @@
         <v>10</v>
       </c>
       <c r="J306" s="4" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="307" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8675,7 +8675,7 @@
         <v>10</v>
       </c>
       <c r="J307" s="4" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
     </row>
     <row r="308" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8698,7 +8698,7 @@
         <v>10</v>
       </c>
       <c r="J308" s="4" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
     </row>
     <row r="309" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8721,7 +8721,7 @@
         <v>10</v>
       </c>
       <c r="J309" s="4" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
     </row>
     <row r="310" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8744,7 +8744,7 @@
         <v>10</v>
       </c>
       <c r="J310" s="4" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
     </row>
     <row r="311" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8767,7 +8767,7 @@
         <v>10</v>
       </c>
       <c r="J311" s="4" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
     </row>
     <row r="312" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8790,7 +8790,7 @@
         <v>10</v>
       </c>
       <c r="J312" s="4" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
     </row>
     <row r="313" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8813,7 +8813,7 @@
         <v>10</v>
       </c>
       <c r="J313" s="4" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
     </row>
     <row r="314" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8833,7 +8833,7 @@
         <v>10</v>
       </c>
       <c r="J314" s="4" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="315" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8853,7 +8853,7 @@
         <v>10</v>
       </c>
       <c r="J315" s="4" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
     </row>
     <row r="316" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8873,7 +8873,7 @@
         <v>10</v>
       </c>
       <c r="J316" s="4" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="317" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8893,7 +8893,7 @@
         <v>10</v>
       </c>
       <c r="J317" s="4" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
     </row>
     <row r="318" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8913,7 +8913,7 @@
         <v>10</v>
       </c>
       <c r="J318" s="4" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
     </row>
     <row r="319" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8933,7 +8933,7 @@
         <v>10</v>
       </c>
       <c r="J319" s="4" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
     </row>
     <row r="320" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8953,7 +8953,7 @@
         <v>10</v>
       </c>
       <c r="J320" s="4" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
     </row>
     <row r="321" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8973,7 +8973,7 @@
         <v>10</v>
       </c>
       <c r="J321" s="4" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="322" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8993,7 +8993,7 @@
         <v>10</v>
       </c>
       <c r="J322" s="4" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="323" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9013,7 +9013,7 @@
         <v>10</v>
       </c>
       <c r="J323" s="4" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="324" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9033,7 +9033,7 @@
         <v>10</v>
       </c>
       <c r="J324" s="4" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="325" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9056,7 +9056,7 @@
         <v>10</v>
       </c>
       <c r="J325" s="4" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
     </row>
     <row r="326" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9079,7 +9079,7 @@
         <v>10</v>
       </c>
       <c r="J326" s="4" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
     </row>
     <row r="327" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9102,7 +9102,7 @@
         <v>10</v>
       </c>
       <c r="J327" s="4" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="328" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9122,7 +9122,7 @@
         <v>10</v>
       </c>
       <c r="J328" s="4" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
     </row>
     <row r="329" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9142,7 +9142,7 @@
         <v>10</v>
       </c>
       <c r="J329" s="4" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
     </row>
     <row r="330" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9162,7 +9162,7 @@
         <v>10</v>
       </c>
       <c r="J330" s="4" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
     </row>
     <row r="331" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9182,7 +9182,7 @@
         <v>10</v>
       </c>
       <c r="J331" s="4" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
     </row>
     <row r="332" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9202,7 +9202,7 @@
         <v>10</v>
       </c>
       <c r="J332" s="4" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
     </row>
     <row r="333" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9225,7 +9225,7 @@
         <v>10</v>
       </c>
       <c r="J333" s="4" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="334" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9248,7 +9248,7 @@
         <v>10</v>
       </c>
       <c r="J334" s="4" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
     </row>
     <row r="335" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9268,7 +9268,7 @@
         <v>10</v>
       </c>
       <c r="J335" s="4" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
     </row>
     <row r="336" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9288,7 +9288,7 @@
         <v>10</v>
       </c>
       <c r="J336" s="4" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
     </row>
     <row r="337" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9311,7 +9311,7 @@
         <v>10</v>
       </c>
       <c r="J337" s="4" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="338" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9334,7 +9334,7 @@
         <v>10</v>
       </c>
       <c r="J338" s="4" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
     </row>
     <row r="339" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9354,12 +9354,12 @@
         <v>10</v>
       </c>
       <c r="J339" s="4" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
     </row>
     <row r="340" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A340" s="4" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="B340" s="4" t="s">
         <v>331</v>
@@ -9371,18 +9371,18 @@
         <v>0</v>
       </c>
       <c r="F340" s="4" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="H340" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J340" s="4" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
     </row>
     <row r="341" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A341" s="4" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="B341" s="4" t="s">
         <v>332</v>
@@ -9397,12 +9397,12 @@
         <v>10</v>
       </c>
       <c r="J341" s="4" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
     </row>
     <row r="342" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A342" s="4" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="B342" s="4" t="s">
         <v>149</v>
@@ -9417,12 +9417,12 @@
         <v>10</v>
       </c>
       <c r="J342" s="4" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="343" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A343" s="4" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="B343" s="4" t="s">
         <v>31</v>
@@ -9440,7 +9440,7 @@
         <v>10</v>
       </c>
       <c r="J343" s="4" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
     </row>
   </sheetData>
@@ -9486,10 +9486,10 @@
         <v>89</v>
       </c>
       <c r="C2" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="D2" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9500,10 +9500,10 @@
         <v>51</v>
       </c>
       <c r="C3" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="E3" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9514,10 +9514,10 @@
         <v>51</v>
       </c>
       <c r="C4" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="E4" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9528,10 +9528,10 @@
         <v>51</v>
       </c>
       <c r="C5" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="E5" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9542,13 +9542,13 @@
         <v>51</v>
       </c>
       <c r="C6" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="D6" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="E6" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9559,10 +9559,10 @@
         <v>51</v>
       </c>
       <c r="C7" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="E7" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9573,10 +9573,10 @@
         <v>51</v>
       </c>
       <c r="C8" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="E8" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9587,10 +9587,10 @@
         <v>51</v>
       </c>
       <c r="C9" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="E9" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9601,10 +9601,10 @@
         <v>51</v>
       </c>
       <c r="C10" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="E10" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9615,10 +9615,10 @@
         <v>51</v>
       </c>
       <c r="C11" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="E11" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9629,10 +9629,10 @@
         <v>51</v>
       </c>
       <c r="C12" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="E12" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9643,10 +9643,10 @@
         <v>51</v>
       </c>
       <c r="C13" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="E13" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9657,10 +9657,10 @@
         <v>51</v>
       </c>
       <c r="C14" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="E14" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9671,10 +9671,10 @@
         <v>51</v>
       </c>
       <c r="C15" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="E15" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9685,10 +9685,10 @@
         <v>51</v>
       </c>
       <c r="C16" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="E16" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9699,10 +9699,10 @@
         <v>51</v>
       </c>
       <c r="C17" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="E17" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9713,10 +9713,10 @@
         <v>51</v>
       </c>
       <c r="C18" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="E18" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
     </row>
   </sheetData>
@@ -9746,10 +9746,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B2" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="C2" t="s">
         <v>21</v>
@@ -9757,7 +9757,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Update bni_golden_queries.json with correct SQL template and user intent for cash out activity
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8015EDF6-7CB3-0545-AFD1-C2D035F9EFA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{323B8465-1134-9A42-8797-5ED527459615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="660" windowWidth="33720" windowHeight="19740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="680" yWindow="660" windowWidth="33720" windowHeight="19740" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tables" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1875" uniqueCount="629">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1877" uniqueCount="630">
   <si>
     <t>Table Name</t>
   </si>
@@ -1906,13 +1906,16 @@
     <t>Wonder</t>
   </si>
   <si>
-    <t>Tampilkan cash out</t>
-  </si>
-  <si>
     <t>Nilai Transaksi / Amount</t>
   </si>
   <si>
     <t>Tanggal Transaksi Data, digunakan untuk filter tanggal, bulan, tahun</t>
+  </si>
+  <si>
+    <t>Aktivitas Cash out</t>
+  </si>
+  <si>
+    <t>SELECT * FROM dm_transaction.trxchannel WHERE destination_bankname &lt;&gt; 'BANK NEGARA INDONESIA';</t>
   </si>
 </sst>
 </file>
@@ -2440,7 +2443,7 @@
         <v>10</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2732,7 +2735,7 @@
         <v>10</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9755,9 +9758,15 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>626</v>
+        <v>628</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>629</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Update SQL query templates and descriptions for consistency and clarity
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{323B8465-1134-9A42-8797-5ED527459615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79458033-870F-9147-A2CA-A0DAE6540A85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="660" windowWidth="33720" windowHeight="19740" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="680" yWindow="660" windowWidth="33720" windowHeight="19740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tables" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1877" uniqueCount="630">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1878" uniqueCount="630">
   <si>
     <t>Table Name</t>
   </si>
@@ -1105,12 +1105,6 @@
     <t>CIF Penerima</t>
   </si>
   <si>
-    <t>No Rek Penerima</t>
-  </si>
-  <si>
-    <t>Bank Penerima</t>
-  </si>
-  <si>
     <t>Nama Penerima</t>
   </si>
   <si>
@@ -1771,9 +1765,6 @@
     <t>SELECT * FROM dm_customer.customer_icons WHERE cust_status = 'AKTIF';</t>
   </si>
   <si>
-    <t>Tampilkan nasabah aktif</t>
-  </si>
-  <si>
     <t>prd_db_sbx_ind</t>
   </si>
   <si>
@@ -1912,10 +1903,19 @@
     <t>Tanggal Transaksi Data, digunakan untuk filter tanggal, bulan, tahun</t>
   </si>
   <si>
-    <t>Aktivitas Cash out</t>
-  </si>
-  <si>
     <t>SELECT * FROM dm_transaction.trxchannel WHERE destination_bankname &lt;&gt; 'BANK NEGARA INDONESIA';</t>
+  </si>
+  <si>
+    <t>Aktivitas cashout / cash out</t>
+  </si>
+  <si>
+    <t>Nasabah aktif</t>
+  </si>
+  <si>
+    <t>Nama Bank Penerima / Nama Bank Tujuan</t>
+  </si>
+  <si>
+    <t>Nomor Rekening Penerima</t>
   </si>
 </sst>
 </file>
@@ -2332,7 +2332,7 @@
         <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -2343,7 +2343,7 @@
         <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -2354,18 +2354,18 @@
         <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="B6" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="C6" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
     </row>
   </sheetData>
@@ -2405,7 +2405,7 @@
         <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>6</v>
@@ -2443,7 +2443,7 @@
         <v>10</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2480,7 +2480,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>10</v>
@@ -2503,7 +2503,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>10</v>
@@ -2706,7 +2706,7 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>10</v>
@@ -2735,7 +2735,7 @@
         <v>10</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2752,7 +2752,7 @@
         <v>0</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
       <c r="J17" s="4" t="s">
         <v>346</v>
@@ -2992,7 +2992,7 @@
         <v>0</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="H29" s="4" t="s">
         <v>10</v>
@@ -3015,13 +3015,13 @@
         <v>0</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="H30" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J30" s="4" t="s">
-        <v>359</v>
+        <v>629</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3041,7 +3041,7 @@
         <v>10</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>360</v>
+        <v>628</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3061,7 +3061,7 @@
         <v>10</v>
       </c>
       <c r="J32" s="4" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3081,7 +3081,7 @@
         <v>10</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3101,7 +3101,7 @@
         <v>10</v>
       </c>
       <c r="J34" s="4" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3121,7 +3121,7 @@
         <v>10</v>
       </c>
       <c r="J35" s="4" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3161,7 +3161,7 @@
         <v>10</v>
       </c>
       <c r="J37" s="4" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
     </row>
     <row r="38" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3181,7 +3181,7 @@
         <v>10</v>
       </c>
       <c r="J38" s="4" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3204,7 +3204,7 @@
         <v>10</v>
       </c>
       <c r="J39" s="4" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3220,11 +3220,14 @@
       <c r="D40" s="4" t="b">
         <v>0</v>
       </c>
+      <c r="G40" s="4" t="s">
+        <v>585</v>
+      </c>
       <c r="H40" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3244,7 +3247,7 @@
         <v>10</v>
       </c>
       <c r="J41" s="4" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3284,7 +3287,7 @@
         <v>10</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3304,7 +3307,7 @@
         <v>10</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3324,7 +3327,7 @@
         <v>10</v>
       </c>
       <c r="J45" s="4" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="46" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3347,7 +3350,7 @@
         <v>10</v>
       </c>
       <c r="J46" s="4" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="47" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3367,7 +3370,7 @@
         <v>10</v>
       </c>
       <c r="J47" s="4" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="48" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3387,7 +3390,7 @@
         <v>10</v>
       </c>
       <c r="J48" s="4" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3407,7 +3410,7 @@
         <v>10</v>
       </c>
       <c r="J49" s="4" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3427,7 +3430,7 @@
         <v>10</v>
       </c>
       <c r="J50" s="4" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3447,7 +3450,7 @@
         <v>10</v>
       </c>
       <c r="J51" s="4" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="52" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3464,13 +3467,13 @@
         <v>0</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
       <c r="I52" s="4" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
       <c r="J52" s="4" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="53" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3490,7 +3493,7 @@
         <v>10</v>
       </c>
       <c r="J53" s="4" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="54" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3510,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="J54" s="4" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="55" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3530,7 +3533,7 @@
         <v>10</v>
       </c>
       <c r="J55" s="4" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="56" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3550,7 +3553,7 @@
         <v>10</v>
       </c>
       <c r="J56" s="4" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="57" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3570,7 +3573,7 @@
         <v>10</v>
       </c>
       <c r="J57" s="4" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
     </row>
     <row r="58" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3590,7 +3593,7 @@
         <v>10</v>
       </c>
       <c r="J58" s="4" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="59" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3610,7 +3613,7 @@
         <v>10</v>
       </c>
       <c r="J59" s="4" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="60" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3630,7 +3633,7 @@
         <v>10</v>
       </c>
       <c r="J60" s="4" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="61" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3650,7 +3653,7 @@
         <v>10</v>
       </c>
       <c r="J61" s="4" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="62" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3670,7 +3673,7 @@
         <v>10</v>
       </c>
       <c r="J62" s="4" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="63" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3690,7 +3693,7 @@
         <v>10</v>
       </c>
       <c r="J63" s="4" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="64" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3710,7 +3713,7 @@
         <v>10</v>
       </c>
       <c r="J64" s="4" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="65" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3730,7 +3733,7 @@
         <v>10</v>
       </c>
       <c r="J65" s="4" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="66" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3750,7 +3753,7 @@
         <v>10</v>
       </c>
       <c r="J66" s="4" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="67" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3773,7 +3776,7 @@
         <v>10</v>
       </c>
       <c r="J67" s="4" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="68" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3793,7 +3796,7 @@
         <v>10</v>
       </c>
       <c r="J68" s="4" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="69" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3813,7 +3816,7 @@
         <v>10</v>
       </c>
       <c r="J69" s="4" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="70" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3833,7 +3836,7 @@
         <v>10</v>
       </c>
       <c r="J70" s="4" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="71" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3853,7 +3856,7 @@
         <v>10</v>
       </c>
       <c r="J71" s="4" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="72" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3873,7 +3876,7 @@
         <v>10</v>
       </c>
       <c r="J72" s="4" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="73" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3893,7 +3896,7 @@
         <v>10</v>
       </c>
       <c r="J73" s="4" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="74" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3913,7 +3916,7 @@
         <v>10</v>
       </c>
       <c r="J74" s="4" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="75" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3933,7 +3936,7 @@
         <v>10</v>
       </c>
       <c r="J75" s="4" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="76" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3953,7 +3956,7 @@
         <v>10</v>
       </c>
       <c r="J76" s="4" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="77" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3973,7 +3976,7 @@
         <v>10</v>
       </c>
       <c r="J77" s="4" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="78" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3993,7 +3996,7 @@
         <v>10</v>
       </c>
       <c r="J78" s="4" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="79" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4013,7 +4016,7 @@
         <v>10</v>
       </c>
       <c r="J79" s="4" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="80" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4033,7 +4036,7 @@
         <v>10</v>
       </c>
       <c r="J80" s="4" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="81" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4053,7 +4056,7 @@
         <v>10</v>
       </c>
       <c r="J81" s="4" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="82" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4107,7 +4110,7 @@
         <v>10</v>
       </c>
       <c r="J84" s="4" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="85" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4178,7 +4181,7 @@
         <v>10</v>
       </c>
       <c r="J88" s="4" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="89" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4198,7 +4201,7 @@
         <v>10</v>
       </c>
       <c r="J89" s="4" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="90" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4218,7 +4221,7 @@
         <v>10</v>
       </c>
       <c r="J90" s="4" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="91" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4238,7 +4241,7 @@
         <v>10</v>
       </c>
       <c r="J91" s="4" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="92" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4258,7 +4261,7 @@
         <v>10</v>
       </c>
       <c r="J92" s="4" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="93" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4278,7 +4281,7 @@
         <v>10</v>
       </c>
       <c r="J93" s="4" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="94" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4298,7 +4301,7 @@
         <v>10</v>
       </c>
       <c r="J94" s="4" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="95" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4318,7 +4321,7 @@
         <v>10</v>
       </c>
       <c r="J95" s="4" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="96" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4338,7 +4341,7 @@
         <v>10</v>
       </c>
       <c r="J96" s="4" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
     </row>
     <row r="97" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4358,7 +4361,7 @@
         <v>10</v>
       </c>
       <c r="J97" s="4" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="98" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4378,7 +4381,7 @@
         <v>10</v>
       </c>
       <c r="J98" s="4" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
     <row r="99" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4398,7 +4401,7 @@
         <v>10</v>
       </c>
       <c r="J99" s="4" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="100" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4418,7 +4421,7 @@
         <v>10</v>
       </c>
       <c r="J100" s="4" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="101" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4455,7 +4458,7 @@
         <v>10</v>
       </c>
       <c r="J102" s="4" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="103" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4475,7 +4478,7 @@
         <v>10</v>
       </c>
       <c r="J103" s="4" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
     </row>
     <row r="104" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4498,7 +4501,7 @@
         <v>10</v>
       </c>
       <c r="J104" s="4" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="105" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4558,7 +4561,7 @@
         <v>10</v>
       </c>
       <c r="J107" s="4" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
     </row>
     <row r="108" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4612,7 +4615,7 @@
         <v>10</v>
       </c>
       <c r="J110" s="4" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="111" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4632,7 +4635,7 @@
         <v>10</v>
       </c>
       <c r="J111" s="4" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="112" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4652,7 +4655,7 @@
         <v>10</v>
       </c>
       <c r="J112" s="4" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="113" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4672,7 +4675,7 @@
         <v>10</v>
       </c>
       <c r="J113" s="4" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="114" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4692,7 +4695,7 @@
         <v>10</v>
       </c>
       <c r="J114" s="4" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
     </row>
     <row r="115" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4712,7 +4715,7 @@
         <v>10</v>
       </c>
       <c r="J115" s="4" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="116" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4732,7 +4735,7 @@
         <v>10</v>
       </c>
       <c r="J116" s="4" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
     <row r="117" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4752,7 +4755,7 @@
         <v>10</v>
       </c>
       <c r="J117" s="4" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
     </row>
     <row r="118" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4772,7 +4775,7 @@
         <v>10</v>
       </c>
       <c r="J118" s="4" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
     </row>
     <row r="119" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4792,7 +4795,7 @@
         <v>10</v>
       </c>
       <c r="J119" s="4" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
     </row>
     <row r="120" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4812,7 +4815,7 @@
         <v>10</v>
       </c>
       <c r="J120" s="4" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="121" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4832,7 +4835,7 @@
         <v>10</v>
       </c>
       <c r="J121" s="4" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
     </row>
     <row r="122" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4852,7 +4855,7 @@
         <v>10</v>
       </c>
       <c r="J122" s="4" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="123" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4872,7 +4875,7 @@
         <v>10</v>
       </c>
       <c r="J123" s="4" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
     </row>
     <row r="124" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4892,7 +4895,7 @@
         <v>10</v>
       </c>
       <c r="J124" s="4" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="125" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4912,7 +4915,7 @@
         <v>10</v>
       </c>
       <c r="J125" s="4" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
     </row>
     <row r="126" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4932,7 +4935,7 @@
         <v>10</v>
       </c>
       <c r="J126" s="4" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
     </row>
     <row r="127" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4952,7 +4955,7 @@
         <v>10</v>
       </c>
       <c r="J127" s="4" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
     </row>
     <row r="128" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4972,7 +4975,7 @@
         <v>10</v>
       </c>
       <c r="J128" s="4" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
     </row>
     <row r="129" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4992,7 +4995,7 @@
         <v>10</v>
       </c>
       <c r="J129" s="4" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
     </row>
     <row r="130" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5012,7 +5015,7 @@
         <v>10</v>
       </c>
       <c r="J130" s="4" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
     </row>
     <row r="131" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5032,7 +5035,7 @@
         <v>10</v>
       </c>
       <c r="J131" s="4" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
     </row>
     <row r="132" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5052,7 +5055,7 @@
         <v>10</v>
       </c>
       <c r="J132" s="4" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
     </row>
     <row r="133" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5072,7 +5075,7 @@
         <v>10</v>
       </c>
       <c r="J133" s="4" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
     </row>
     <row r="134" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5092,7 +5095,7 @@
         <v>10</v>
       </c>
       <c r="J134" s="4" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
     </row>
     <row r="135" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5112,7 +5115,7 @@
         <v>10</v>
       </c>
       <c r="J135" s="4" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
     </row>
     <row r="136" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5132,7 +5135,7 @@
         <v>10</v>
       </c>
       <c r="J136" s="4" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
     </row>
     <row r="137" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5152,7 +5155,7 @@
         <v>10</v>
       </c>
       <c r="J137" s="4" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
     </row>
     <row r="138" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5172,7 +5175,7 @@
         <v>10</v>
       </c>
       <c r="J138" s="4" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
     </row>
     <row r="139" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5192,7 +5195,7 @@
         <v>10</v>
       </c>
       <c r="J139" s="4" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
     </row>
     <row r="140" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5212,7 +5215,7 @@
         <v>10</v>
       </c>
       <c r="J140" s="4" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
     </row>
     <row r="141" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5229,13 +5232,13 @@
         <v>0</v>
       </c>
       <c r="F141" s="4" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="H141" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J141" s="4" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
     </row>
     <row r="142" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5255,7 +5258,7 @@
         <v>10</v>
       </c>
       <c r="J142" s="4" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
     </row>
     <row r="143" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5275,7 +5278,7 @@
         <v>10</v>
       </c>
       <c r="J143" s="4" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
     </row>
     <row r="144" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5295,7 +5298,7 @@
         <v>10</v>
       </c>
       <c r="J144" s="4" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="145" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5315,7 +5318,7 @@
         <v>10</v>
       </c>
       <c r="J145" s="4" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
     </row>
     <row r="146" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5335,7 +5338,7 @@
         <v>10</v>
       </c>
       <c r="J146" s="4" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
     </row>
     <row r="147" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5355,7 +5358,7 @@
         <v>10</v>
       </c>
       <c r="J147" s="4" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
     </row>
     <row r="148" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5375,7 +5378,7 @@
         <v>10</v>
       </c>
       <c r="J148" s="4" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
     </row>
     <row r="149" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5395,7 +5398,7 @@
         <v>10</v>
       </c>
       <c r="J149" s="4" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
     <row r="150" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5415,7 +5418,7 @@
         <v>10</v>
       </c>
       <c r="J150" s="4" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
     </row>
     <row r="151" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5435,7 +5438,7 @@
         <v>10</v>
       </c>
       <c r="J151" s="4" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
     </row>
     <row r="152" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5455,7 +5458,7 @@
         <v>10</v>
       </c>
       <c r="J152" s="4" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="153" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5475,7 +5478,7 @@
         <v>10</v>
       </c>
       <c r="J153" s="4" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
     </row>
     <row r="154" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5495,7 +5498,7 @@
         <v>10</v>
       </c>
       <c r="J154" s="4" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="155" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5515,7 +5518,7 @@
         <v>10</v>
       </c>
       <c r="J155" s="4" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="156" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5535,7 +5538,7 @@
         <v>10</v>
       </c>
       <c r="J156" s="4" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
     </row>
     <row r="157" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5555,7 +5558,7 @@
         <v>10</v>
       </c>
       <c r="J157" s="4" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
     </row>
     <row r="158" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5575,7 +5578,7 @@
         <v>10</v>
       </c>
       <c r="J158" s="4" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
     </row>
     <row r="159" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5595,7 +5598,7 @@
         <v>10</v>
       </c>
       <c r="J159" s="4" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="160" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5615,7 +5618,7 @@
         <v>10</v>
       </c>
       <c r="J160" s="4" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
     </row>
     <row r="161" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5635,7 +5638,7 @@
         <v>10</v>
       </c>
       <c r="J161" s="4" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="162" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5655,7 +5658,7 @@
         <v>10</v>
       </c>
       <c r="J162" s="4" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="163" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5675,7 +5678,7 @@
         <v>10</v>
       </c>
       <c r="J163" s="4" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
     </row>
     <row r="164" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5695,7 +5698,7 @@
         <v>10</v>
       </c>
       <c r="J164" s="4" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="165" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5715,7 +5718,7 @@
         <v>10</v>
       </c>
       <c r="J165" s="4" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="166" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5735,7 +5738,7 @@
         <v>10</v>
       </c>
       <c r="J166" s="4" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="167" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5758,7 +5761,7 @@
         <v>10</v>
       </c>
       <c r="J167" s="4" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="168" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5778,7 +5781,7 @@
         <v>10</v>
       </c>
       <c r="J168" s="4" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
     </row>
     <row r="169" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5798,7 +5801,7 @@
         <v>10</v>
       </c>
       <c r="J169" s="4" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
     </row>
     <row r="170" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5818,7 +5821,7 @@
         <v>10</v>
       </c>
       <c r="J170" s="4" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="171" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5838,7 +5841,7 @@
         <v>10</v>
       </c>
       <c r="J171" s="4" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="172" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5858,7 +5861,7 @@
         <v>10</v>
       </c>
       <c r="J172" s="4" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
     </row>
     <row r="173" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5878,7 +5881,7 @@
         <v>10</v>
       </c>
       <c r="J173" s="4" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="174" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5898,7 +5901,7 @@
         <v>10</v>
       </c>
       <c r="J174" s="4" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
     </row>
     <row r="175" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5918,7 +5921,7 @@
         <v>10</v>
       </c>
       <c r="J175" s="4" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
     </row>
     <row r="176" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5938,7 +5941,7 @@
         <v>10</v>
       </c>
       <c r="J176" s="4" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="177" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5958,7 +5961,7 @@
         <v>10</v>
       </c>
       <c r="J177" s="4" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="178" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5978,7 +5981,7 @@
         <v>10</v>
       </c>
       <c r="J178" s="4" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="179" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6001,7 +6004,7 @@
         <v>10</v>
       </c>
       <c r="J179" s="4" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="180" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6024,7 +6027,7 @@
         <v>10</v>
       </c>
       <c r="J180" s="4" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
     </row>
     <row r="181" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6047,7 +6050,7 @@
         <v>10</v>
       </c>
       <c r="J181" s="4" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
     </row>
     <row r="182" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6070,7 +6073,7 @@
         <v>10</v>
       </c>
       <c r="J182" s="4" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
     </row>
     <row r="183" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6093,7 +6096,7 @@
         <v>10</v>
       </c>
       <c r="J183" s="4" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
     </row>
     <row r="184" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6113,7 +6116,7 @@
         <v>10</v>
       </c>
       <c r="J184" s="4" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
     </row>
     <row r="185" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6133,7 +6136,7 @@
         <v>10</v>
       </c>
       <c r="J185" s="4" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
     </row>
     <row r="186" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6153,7 +6156,7 @@
         <v>10</v>
       </c>
       <c r="J186" s="4" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
     </row>
     <row r="187" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6173,7 +6176,7 @@
         <v>10</v>
       </c>
       <c r="J187" s="4" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
     </row>
     <row r="188" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6193,7 +6196,7 @@
         <v>10</v>
       </c>
       <c r="J188" s="4" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
     </row>
     <row r="189" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6213,7 +6216,7 @@
         <v>10</v>
       </c>
       <c r="J189" s="4" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
     </row>
     <row r="190" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6233,7 +6236,7 @@
         <v>10</v>
       </c>
       <c r="J190" s="4" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
     </row>
     <row r="191" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6253,7 +6256,7 @@
         <v>10</v>
       </c>
       <c r="J191" s="4" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
     </row>
     <row r="192" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6273,7 +6276,7 @@
         <v>10</v>
       </c>
       <c r="J192" s="4" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
     </row>
     <row r="193" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6293,7 +6296,7 @@
         <v>10</v>
       </c>
       <c r="J193" s="4" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
     </row>
     <row r="194" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6313,7 +6316,7 @@
         <v>10</v>
       </c>
       <c r="J194" s="4" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
     </row>
     <row r="195" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6333,7 +6336,7 @@
         <v>10</v>
       </c>
       <c r="J195" s="4" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
     </row>
     <row r="196" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6353,7 +6356,7 @@
         <v>10</v>
       </c>
       <c r="J196" s="4" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="197" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6373,7 +6376,7 @@
         <v>10</v>
       </c>
       <c r="J197" s="4" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="198" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6393,7 +6396,7 @@
         <v>10</v>
       </c>
       <c r="J198" s="4" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="199" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6413,7 +6416,7 @@
         <v>10</v>
       </c>
       <c r="J199" s="4" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
     </row>
     <row r="200" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6433,7 +6436,7 @@
         <v>10</v>
       </c>
       <c r="J200" s="4" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="201" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6453,7 +6456,7 @@
         <v>10</v>
       </c>
       <c r="J201" s="4" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
     </row>
     <row r="202" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6476,7 +6479,7 @@
         <v>10</v>
       </c>
       <c r="J202" s="4" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
     </row>
     <row r="203" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6499,7 +6502,7 @@
         <v>10</v>
       </c>
       <c r="J203" s="4" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
     </row>
     <row r="204" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6522,7 +6525,7 @@
         <v>10</v>
       </c>
       <c r="J204" s="4" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
     </row>
     <row r="205" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6545,7 +6548,7 @@
         <v>10</v>
       </c>
       <c r="J205" s="4" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
     </row>
     <row r="206" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6568,7 +6571,7 @@
         <v>10</v>
       </c>
       <c r="J206" s="4" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
     </row>
     <row r="207" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6591,7 +6594,7 @@
         <v>10</v>
       </c>
       <c r="J207" s="4" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
     </row>
     <row r="208" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6614,7 +6617,7 @@
         <v>10</v>
       </c>
       <c r="J208" s="4" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
     </row>
     <row r="209" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6637,7 +6640,7 @@
         <v>10</v>
       </c>
       <c r="J209" s="4" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
     </row>
     <row r="210" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6660,7 +6663,7 @@
         <v>10</v>
       </c>
       <c r="J210" s="4" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
     </row>
     <row r="211" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6683,7 +6686,7 @@
         <v>10</v>
       </c>
       <c r="J211" s="4" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
     </row>
     <row r="212" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6703,7 +6706,7 @@
         <v>10</v>
       </c>
       <c r="J212" s="4" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
     </row>
     <row r="213" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6723,7 +6726,7 @@
         <v>10</v>
       </c>
       <c r="J213" s="4" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
     </row>
     <row r="214" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6743,7 +6746,7 @@
         <v>10</v>
       </c>
       <c r="J214" s="4" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
     </row>
     <row r="215" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6766,7 +6769,7 @@
         <v>10</v>
       </c>
       <c r="J215" s="4" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
     </row>
     <row r="216" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6789,7 +6792,7 @@
         <v>10</v>
       </c>
       <c r="J216" s="4" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
     </row>
     <row r="217" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6812,7 +6815,7 @@
         <v>10</v>
       </c>
       <c r="J217" s="4" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
     </row>
     <row r="218" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6832,7 +6835,7 @@
         <v>10</v>
       </c>
       <c r="J218" s="4" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
     </row>
     <row r="219" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6852,7 +6855,7 @@
         <v>10</v>
       </c>
       <c r="J219" s="4" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
     </row>
     <row r="220" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6872,7 +6875,7 @@
         <v>10</v>
       </c>
       <c r="J220" s="4" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
     </row>
     <row r="221" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6892,7 +6895,7 @@
         <v>10</v>
       </c>
       <c r="J221" s="4" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
     </row>
     <row r="222" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6912,7 +6915,7 @@
         <v>10</v>
       </c>
       <c r="J222" s="4" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
     </row>
     <row r="223" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6932,7 +6935,7 @@
         <v>10</v>
       </c>
       <c r="J223" s="4" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
     </row>
     <row r="224" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6952,7 +6955,7 @@
         <v>10</v>
       </c>
       <c r="J224" s="4" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
     </row>
     <row r="225" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6972,7 +6975,7 @@
         <v>10</v>
       </c>
       <c r="J225" s="4" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
     </row>
     <row r="226" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6992,7 +6995,7 @@
         <v>10</v>
       </c>
       <c r="J226" s="4" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
     </row>
     <row r="227" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7012,7 +7015,7 @@
         <v>10</v>
       </c>
       <c r="J227" s="4" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
     </row>
     <row r="228" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7032,7 +7035,7 @@
         <v>10</v>
       </c>
       <c r="J228" s="4" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
     </row>
     <row r="229" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7055,7 +7058,7 @@
         <v>10</v>
       </c>
       <c r="J229" s="4" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
     </row>
     <row r="230" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7078,7 +7081,7 @@
         <v>10</v>
       </c>
       <c r="J230" s="4" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="231" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7101,7 +7104,7 @@
         <v>10</v>
       </c>
       <c r="J231" s="4" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
     </row>
     <row r="232" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7124,7 +7127,7 @@
         <v>10</v>
       </c>
       <c r="J232" s="4" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="233" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7147,7 +7150,7 @@
         <v>10</v>
       </c>
       <c r="J233" s="4" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
     </row>
     <row r="234" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7170,7 +7173,7 @@
         <v>10</v>
       </c>
       <c r="J234" s="4" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="235" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7193,7 +7196,7 @@
         <v>10</v>
       </c>
       <c r="J235" s="4" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
     </row>
     <row r="236" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7216,7 +7219,7 @@
         <v>10</v>
       </c>
       <c r="J236" s="4" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
     </row>
     <row r="237" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7236,7 +7239,7 @@
         <v>10</v>
       </c>
       <c r="J237" s="4" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
     </row>
     <row r="238" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7259,7 +7262,7 @@
         <v>10</v>
       </c>
       <c r="J238" s="4" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
     </row>
     <row r="239" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7279,7 +7282,7 @@
         <v>10</v>
       </c>
       <c r="J239" s="4" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="240" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7302,7 +7305,7 @@
         <v>10</v>
       </c>
       <c r="J240" s="4" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
     </row>
     <row r="241" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7322,7 +7325,7 @@
         <v>10</v>
       </c>
       <c r="J241" s="4" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
     </row>
     <row r="242" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7342,7 +7345,7 @@
         <v>10</v>
       </c>
       <c r="J242" s="4" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
     </row>
     <row r="243" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7359,13 +7362,13 @@
         <v>0</v>
       </c>
       <c r="F243" s="4" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="H243" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J243" s="4" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
     </row>
     <row r="244" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7385,7 +7388,7 @@
         <v>10</v>
       </c>
       <c r="J244" s="4" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
     </row>
     <row r="245" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7405,7 +7408,7 @@
         <v>10</v>
       </c>
       <c r="J245" s="4" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
     </row>
     <row r="246" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7425,7 +7428,7 @@
         <v>10</v>
       </c>
       <c r="J246" s="4" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
     </row>
     <row r="247" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7445,7 +7448,7 @@
         <v>10</v>
       </c>
       <c r="J247" s="4" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="248" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7465,7 +7468,7 @@
         <v>10</v>
       </c>
       <c r="J248" s="4" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
     </row>
     <row r="249" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7485,7 +7488,7 @@
         <v>10</v>
       </c>
       <c r="J249" s="4" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
     </row>
     <row r="250" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7505,7 +7508,7 @@
         <v>10</v>
       </c>
       <c r="J250" s="4" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
     </row>
     <row r="251" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7525,7 +7528,7 @@
         <v>10</v>
       </c>
       <c r="J251" s="4" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
     </row>
     <row r="252" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7545,7 +7548,7 @@
         <v>10</v>
       </c>
       <c r="J252" s="4" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
     <row r="253" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7565,7 +7568,7 @@
         <v>10</v>
       </c>
       <c r="J253" s="4" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
     </row>
     <row r="254" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7585,7 +7588,7 @@
         <v>10</v>
       </c>
       <c r="J254" s="4" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
     </row>
     <row r="255" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7605,7 +7608,7 @@
         <v>10</v>
       </c>
       <c r="J255" s="4" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="256" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7625,7 +7628,7 @@
         <v>10</v>
       </c>
       <c r="J256" s="4" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
     </row>
     <row r="257" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7645,7 +7648,7 @@
         <v>10</v>
       </c>
       <c r="J257" s="4" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="258" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7665,7 +7668,7 @@
         <v>10</v>
       </c>
       <c r="J258" s="4" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="259" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7685,7 +7688,7 @@
         <v>10</v>
       </c>
       <c r="J259" s="4" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
     </row>
     <row r="260" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7705,7 +7708,7 @@
         <v>10</v>
       </c>
       <c r="J260" s="4" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
     </row>
     <row r="261" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7725,7 +7728,7 @@
         <v>10</v>
       </c>
       <c r="J261" s="4" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
     </row>
     <row r="262" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7745,7 +7748,7 @@
         <v>10</v>
       </c>
       <c r="J262" s="4" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="263" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7765,7 +7768,7 @@
         <v>10</v>
       </c>
       <c r="J263" s="4" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
     </row>
     <row r="264" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7785,7 +7788,7 @@
         <v>10</v>
       </c>
       <c r="J264" s="4" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="265" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7805,7 +7808,7 @@
         <v>10</v>
       </c>
       <c r="J265" s="4" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="266" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7825,7 +7828,7 @@
         <v>10</v>
       </c>
       <c r="J266" s="4" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
     </row>
     <row r="267" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7845,7 +7848,7 @@
         <v>10</v>
       </c>
       <c r="J267" s="4" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="268" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7865,7 +7868,7 @@
         <v>10</v>
       </c>
       <c r="J268" s="4" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="269" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7885,7 +7888,7 @@
         <v>10</v>
       </c>
       <c r="J269" s="4" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="270" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7905,7 +7908,7 @@
         <v>10</v>
       </c>
       <c r="J270" s="4" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="271" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7925,7 +7928,7 @@
         <v>10</v>
       </c>
       <c r="J271" s="4" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
     </row>
     <row r="272" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7945,7 +7948,7 @@
         <v>10</v>
       </c>
       <c r="J272" s="4" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="273" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7965,7 +7968,7 @@
         <v>10</v>
       </c>
       <c r="J273" s="4" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="274" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7985,7 +7988,7 @@
         <v>10</v>
       </c>
       <c r="J274" s="4" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="275" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8005,7 +8008,7 @@
         <v>10</v>
       </c>
       <c r="J275" s="4" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
     </row>
     <row r="276" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8025,7 +8028,7 @@
         <v>10</v>
       </c>
       <c r="J276" s="4" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
     </row>
     <row r="277" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8045,7 +8048,7 @@
         <v>10</v>
       </c>
       <c r="J277" s="4" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="278" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8065,7 +8068,7 @@
         <v>10</v>
       </c>
       <c r="J278" s="4" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
     </row>
     <row r="279" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8085,7 +8088,7 @@
         <v>10</v>
       </c>
       <c r="J279" s="4" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
     </row>
     <row r="280" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8105,7 +8108,7 @@
         <v>10</v>
       </c>
       <c r="J280" s="4" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
     </row>
     <row r="281" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8125,7 +8128,7 @@
         <v>10</v>
       </c>
       <c r="J281" s="4" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="282" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8145,7 +8148,7 @@
         <v>10</v>
       </c>
       <c r="J282" s="4" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
     </row>
     <row r="283" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8165,7 +8168,7 @@
         <v>10</v>
       </c>
       <c r="J283" s="4" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="284" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8185,7 +8188,7 @@
         <v>10</v>
       </c>
       <c r="J284" s="4" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
     </row>
     <row r="285" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8205,7 +8208,7 @@
         <v>10</v>
       </c>
       <c r="J285" s="4" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
     </row>
     <row r="286" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8225,7 +8228,7 @@
         <v>10</v>
       </c>
       <c r="J286" s="4" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
     </row>
     <row r="287" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8245,7 +8248,7 @@
         <v>10</v>
       </c>
       <c r="J287" s="4" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
     </row>
     <row r="288" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8265,7 +8268,7 @@
         <v>10</v>
       </c>
       <c r="J288" s="4" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
     </row>
     <row r="289" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8285,7 +8288,7 @@
         <v>10</v>
       </c>
       <c r="J289" s="4" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
     </row>
     <row r="290" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8305,7 +8308,7 @@
         <v>10</v>
       </c>
       <c r="J290" s="4" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
     </row>
     <row r="291" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8325,7 +8328,7 @@
         <v>10</v>
       </c>
       <c r="J291" s="4" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
     </row>
     <row r="292" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8345,7 +8348,7 @@
         <v>10</v>
       </c>
       <c r="J292" s="4" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
     </row>
     <row r="293" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8365,7 +8368,7 @@
         <v>10</v>
       </c>
       <c r="J293" s="4" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="294" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8385,7 +8388,7 @@
         <v>10</v>
       </c>
       <c r="J294" s="4" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
     </row>
     <row r="295" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8405,7 +8408,7 @@
         <v>10</v>
       </c>
       <c r="J295" s="4" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="296" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8425,7 +8428,7 @@
         <v>10</v>
       </c>
       <c r="J296" s="4" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
     </row>
     <row r="297" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8448,7 +8451,7 @@
         <v>10</v>
       </c>
       <c r="J297" s="4" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
     </row>
     <row r="298" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8471,7 +8474,7 @@
         <v>10</v>
       </c>
       <c r="J298" s="4" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
     </row>
     <row r="299" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8494,7 +8497,7 @@
         <v>10</v>
       </c>
       <c r="J299" s="4" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
     </row>
     <row r="300" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8517,7 +8520,7 @@
         <v>10</v>
       </c>
       <c r="J300" s="4" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
     </row>
     <row r="301" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8540,7 +8543,7 @@
         <v>10</v>
       </c>
       <c r="J301" s="4" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
     </row>
     <row r="302" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8563,7 +8566,7 @@
         <v>10</v>
       </c>
       <c r="J302" s="4" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
     </row>
     <row r="303" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8586,7 +8589,7 @@
         <v>10</v>
       </c>
       <c r="J303" s="4" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
     </row>
     <row r="304" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8609,7 +8612,7 @@
         <v>10</v>
       </c>
       <c r="J304" s="4" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
     </row>
     <row r="305" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8632,7 +8635,7 @@
         <v>10</v>
       </c>
       <c r="J305" s="4" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
     </row>
     <row r="306" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8655,7 +8658,7 @@
         <v>10</v>
       </c>
       <c r="J306" s="4" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
     </row>
     <row r="307" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8678,7 +8681,7 @@
         <v>10</v>
       </c>
       <c r="J307" s="4" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
     </row>
     <row r="308" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8701,7 +8704,7 @@
         <v>10</v>
       </c>
       <c r="J308" s="4" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="309" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8724,7 +8727,7 @@
         <v>10</v>
       </c>
       <c r="J309" s="4" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
     </row>
     <row r="310" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8747,7 +8750,7 @@
         <v>10</v>
       </c>
       <c r="J310" s="4" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="311" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8770,7 +8773,7 @@
         <v>10</v>
       </c>
       <c r="J311" s="4" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
     </row>
     <row r="312" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8793,7 +8796,7 @@
         <v>10</v>
       </c>
       <c r="J312" s="4" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
     </row>
     <row r="313" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8816,7 +8819,7 @@
         <v>10</v>
       </c>
       <c r="J313" s="4" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
     </row>
     <row r="314" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8836,7 +8839,7 @@
         <v>10</v>
       </c>
       <c r="J314" s="4" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
     </row>
     <row r="315" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8856,7 +8859,7 @@
         <v>10</v>
       </c>
       <c r="J315" s="4" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
     </row>
     <row r="316" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8876,7 +8879,7 @@
         <v>10</v>
       </c>
       <c r="J316" s="4" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="317" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8896,7 +8899,7 @@
         <v>10</v>
       </c>
       <c r="J317" s="4" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
     </row>
     <row r="318" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8916,7 +8919,7 @@
         <v>10</v>
       </c>
       <c r="J318" s="4" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="319" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8936,7 +8939,7 @@
         <v>10</v>
       </c>
       <c r="J319" s="4" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
     </row>
     <row r="320" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8956,7 +8959,7 @@
         <v>10</v>
       </c>
       <c r="J320" s="4" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
     </row>
     <row r="321" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8976,7 +8979,7 @@
         <v>10</v>
       </c>
       <c r="J321" s="4" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
     </row>
     <row r="322" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8996,7 +8999,7 @@
         <v>10</v>
       </c>
       <c r="J322" s="4" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
     </row>
     <row r="323" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9016,7 +9019,7 @@
         <v>10</v>
       </c>
       <c r="J323" s="4" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
     </row>
     <row r="324" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9036,7 +9039,7 @@
         <v>10</v>
       </c>
       <c r="J324" s="4" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
     </row>
     <row r="325" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9059,7 +9062,7 @@
         <v>10</v>
       </c>
       <c r="J325" s="4" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
     </row>
     <row r="326" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9082,7 +9085,7 @@
         <v>10</v>
       </c>
       <c r="J326" s="4" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
     </row>
     <row r="327" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9105,7 +9108,7 @@
         <v>10</v>
       </c>
       <c r="J327" s="4" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="328" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9125,7 +9128,7 @@
         <v>10</v>
       </c>
       <c r="J328" s="4" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="329" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9145,7 +9148,7 @@
         <v>10</v>
       </c>
       <c r="J329" s="4" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="330" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9165,7 +9168,7 @@
         <v>10</v>
       </c>
       <c r="J330" s="4" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="331" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9185,7 +9188,7 @@
         <v>10</v>
       </c>
       <c r="J331" s="4" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="332" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9205,7 +9208,7 @@
         <v>10</v>
       </c>
       <c r="J332" s="4" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="333" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9228,7 +9231,7 @@
         <v>10</v>
       </c>
       <c r="J333" s="4" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="334" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9251,7 +9254,7 @@
         <v>10</v>
       </c>
       <c r="J334" s="4" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
     </row>
     <row r="335" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9271,7 +9274,7 @@
         <v>10</v>
       </c>
       <c r="J335" s="4" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
     </row>
     <row r="336" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9291,7 +9294,7 @@
         <v>10</v>
       </c>
       <c r="J336" s="4" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
     </row>
     <row r="337" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9314,7 +9317,7 @@
         <v>10</v>
       </c>
       <c r="J337" s="4" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="338" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9337,7 +9340,7 @@
         <v>10</v>
       </c>
       <c r="J338" s="4" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
     </row>
     <row r="339" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9357,12 +9360,12 @@
         <v>10</v>
       </c>
       <c r="J339" s="4" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="340" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A340" s="4" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="B340" s="4" t="s">
         <v>331</v>
@@ -9374,18 +9377,18 @@
         <v>0</v>
       </c>
       <c r="F340" s="4" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="H340" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J340" s="4" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
     </row>
     <row r="341" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A341" s="4" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="B341" s="4" t="s">
         <v>332</v>
@@ -9400,12 +9403,12 @@
         <v>10</v>
       </c>
       <c r="J341" s="4" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
     </row>
     <row r="342" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A342" s="4" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="B342" s="4" t="s">
         <v>149</v>
@@ -9420,12 +9423,12 @@
         <v>10</v>
       </c>
       <c r="J342" s="4" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="343" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A343" s="4" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="B343" s="4" t="s">
         <v>31</v>
@@ -9443,7 +9446,7 @@
         <v>10</v>
       </c>
       <c r="J343" s="4" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
     </row>
   </sheetData>
@@ -9489,10 +9492,10 @@
         <v>89</v>
       </c>
       <c r="C2" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
       <c r="D2" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9503,10 +9506,10 @@
         <v>51</v>
       </c>
       <c r="C3" t="s">
-        <v>593</v>
+        <v>590</v>
       </c>
       <c r="E3" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9517,10 +9520,10 @@
         <v>51</v>
       </c>
       <c r="C4" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
       <c r="E4" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9531,10 +9534,10 @@
         <v>51</v>
       </c>
       <c r="C5" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="E5" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9545,13 +9548,13 @@
         <v>51</v>
       </c>
       <c r="C6" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="D6" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
       <c r="E6" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9562,10 +9565,10 @@
         <v>51</v>
       </c>
       <c r="C7" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="E7" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9576,10 +9579,10 @@
         <v>51</v>
       </c>
       <c r="C8" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="E8" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9590,10 +9593,10 @@
         <v>51</v>
       </c>
       <c r="C9" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="E9" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9604,10 +9607,10 @@
         <v>51</v>
       </c>
       <c r="C10" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="E10" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9618,10 +9621,10 @@
         <v>51</v>
       </c>
       <c r="C11" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="E11" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9632,10 +9635,10 @@
         <v>51</v>
       </c>
       <c r="C12" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="E12" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9646,10 +9649,10 @@
         <v>51</v>
       </c>
       <c r="C13" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="E13" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9660,10 +9663,10 @@
         <v>51</v>
       </c>
       <c r="C14" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="E14" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9674,10 +9677,10 @@
         <v>51</v>
       </c>
       <c r="C15" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="E15" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9688,10 +9691,10 @@
         <v>51</v>
       </c>
       <c r="C16" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="E16" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9702,10 +9705,10 @@
         <v>51</v>
       </c>
       <c r="C17" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="E17" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9716,10 +9719,10 @@
         <v>51</v>
       </c>
       <c r="C18" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
       <c r="E18" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
     </row>
   </sheetData>
@@ -9749,10 +9752,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>581</v>
+        <v>627</v>
       </c>
       <c r="B2" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="C2" t="s">
         <v>21</v>
@@ -9760,10 +9763,10 @@
     </row>
     <row r="3" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>629</v>
+        <v>625</v>
       </c>
       <c r="C3" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
feat: Update transaction amount descriptions for clarity and multilingual support
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F448F407-F0F7-414C-AF7C-83BC65D9BE38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8577950B-F469-5D41-B8C7-D3F520D383FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="660" windowWidth="30680" windowHeight="19740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1390,9 +1390,6 @@
     <t>Nasabah aktif</t>
   </si>
   <si>
-    <t>Nilai Transaksi</t>
-  </si>
-  <si>
     <t>No Rek Penerima</t>
   </si>
   <si>
@@ -2138,6 +2135,9 @@
   </si>
   <si>
     <t>Tanggal snapshot customer, digunakan untuk filter tanggal, bulan, tahun</t>
+  </si>
+  <si>
+    <t>Nilai Transaksi / Transaction Amount / Amount Transaksi</t>
   </si>
 </sst>
 </file>
@@ -2612,7 +2612,7 @@
     <col min="7" max="7" width="24.33203125" style="4" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22.1640625" style="4" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="24.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="40.5" style="4" customWidth="1"/>
+    <col min="10" max="10" width="76.5" style="4" bestFit="1" customWidth="1"/>
     <col min="11" max="16384" width="8.83203125" style="4"/>
   </cols>
   <sheetData>
@@ -2711,7 +2711,7 @@
         <v>10</v>
       </c>
       <c r="J4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="32" x14ac:dyDescent="0.2">
@@ -2734,7 +2734,7 @@
         <v>10</v>
       </c>
       <c r="J5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2960,7 +2960,7 @@
         <v>10</v>
       </c>
       <c r="J16" t="s">
-        <v>454</v>
+        <v>703</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3246,7 +3246,7 @@
         <v>10</v>
       </c>
       <c r="J30" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3266,7 +3266,7 @@
         <v>10</v>
       </c>
       <c r="J31" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3452,7 +3452,7 @@
         <v>10</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3535,7 +3535,7 @@
         <v>10</v>
       </c>
       <c r="J44" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3961,7 +3961,7 @@
         <v>10</v>
       </c>
       <c r="J65" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
     </row>
     <row r="66" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3981,7 +3981,7 @@
         <v>10</v>
       </c>
       <c r="J66" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
     </row>
     <row r="67" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4001,7 +4001,7 @@
         <v>10</v>
       </c>
       <c r="J67" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="68" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4024,7 +4024,7 @@
         <v>10</v>
       </c>
       <c r="J68" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
     </row>
     <row r="69" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4044,7 +4044,7 @@
         <v>10</v>
       </c>
       <c r="J69" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
     </row>
     <row r="70" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4064,7 +4064,7 @@
         <v>10</v>
       </c>
       <c r="J70" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
     </row>
     <row r="71" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4124,7 +4124,7 @@
         <v>10</v>
       </c>
       <c r="J73" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
     </row>
     <row r="74" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4224,7 +4224,7 @@
         <v>10</v>
       </c>
       <c r="J78" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="79" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4244,7 +4244,7 @@
         <v>10</v>
       </c>
       <c r="J79" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
     </row>
     <row r="80" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4264,7 +4264,7 @@
         <v>10</v>
       </c>
       <c r="J80" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
     </row>
     <row r="81" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4284,7 +4284,7 @@
         <v>10</v>
       </c>
       <c r="J81" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
     </row>
     <row r="82" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4304,7 +4304,7 @@
         <v>10</v>
       </c>
       <c r="J82" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
     </row>
     <row r="83" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4360,7 +4360,7 @@
         <v>10</v>
       </c>
       <c r="J85" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="86" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4434,7 +4434,7 @@
         <v>10</v>
       </c>
       <c r="J89" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
     </row>
     <row r="90" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4454,7 +4454,7 @@
         <v>10</v>
       </c>
       <c r="J90" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
     </row>
     <row r="91" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4474,7 +4474,7 @@
         <v>10</v>
       </c>
       <c r="J91" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
     </row>
     <row r="92" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4494,7 +4494,7 @@
         <v>10</v>
       </c>
       <c r="J92" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
     </row>
     <row r="93" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4514,7 +4514,7 @@
         <v>10</v>
       </c>
       <c r="J93" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="94" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4534,7 +4534,7 @@
         <v>10</v>
       </c>
       <c r="J94" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
     </row>
     <row r="95" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4554,7 +4554,7 @@
         <v>10</v>
       </c>
       <c r="J95" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
     </row>
     <row r="96" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4574,7 +4574,7 @@
         <v>10</v>
       </c>
       <c r="J96" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="97" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4614,7 +4614,7 @@
         <v>10</v>
       </c>
       <c r="J98" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="99" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4634,7 +4634,7 @@
         <v>10</v>
       </c>
       <c r="J99" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="100" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4873,7 +4873,7 @@
         <v>10</v>
       </c>
       <c r="J111" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
     </row>
     <row r="112" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4893,7 +4893,7 @@
         <v>10</v>
       </c>
       <c r="J112" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
     </row>
     <row r="113" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4913,7 +4913,7 @@
         <v>10</v>
       </c>
       <c r="J113" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
     </row>
     <row r="114" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4933,7 +4933,7 @@
         <v>10</v>
       </c>
       <c r="J114" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="115" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4953,7 +4953,7 @@
         <v>10</v>
       </c>
       <c r="J115" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
     </row>
     <row r="116" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4973,7 +4973,7 @@
         <v>10</v>
       </c>
       <c r="J116" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="117" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4993,7 +4993,7 @@
         <v>10</v>
       </c>
       <c r="J117" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
     </row>
     <row r="118" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5013,7 +5013,7 @@
         <v>10</v>
       </c>
       <c r="J118" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="119" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5033,7 +5033,7 @@
         <v>10</v>
       </c>
       <c r="J119" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="120" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5053,7 +5053,7 @@
         <v>10</v>
       </c>
       <c r="J120" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
     </row>
     <row r="121" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5073,7 +5073,7 @@
         <v>10</v>
       </c>
       <c r="J121" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
     </row>
     <row r="122" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5093,7 +5093,7 @@
         <v>10</v>
       </c>
       <c r="J122" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
     </row>
     <row r="123" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5113,7 +5113,7 @@
         <v>10</v>
       </c>
       <c r="J123" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="124" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5133,7 +5133,7 @@
         <v>10</v>
       </c>
       <c r="J124" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="125" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5153,7 +5153,7 @@
         <v>10</v>
       </c>
       <c r="J125" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
     </row>
     <row r="126" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5173,7 +5173,7 @@
         <v>10</v>
       </c>
       <c r="J126" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
     </row>
     <row r="127" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5193,7 +5193,7 @@
         <v>10</v>
       </c>
       <c r="J127" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="128" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5213,7 +5213,7 @@
         <v>10</v>
       </c>
       <c r="J128" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
     <row r="129" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5233,7 +5233,7 @@
         <v>10</v>
       </c>
       <c r="J129" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
     </row>
     <row r="130" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5253,7 +5253,7 @@
         <v>10</v>
       </c>
       <c r="J130" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
     </row>
     <row r="131" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5273,7 +5273,7 @@
         <v>10</v>
       </c>
       <c r="J131" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
     </row>
     <row r="132" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5293,7 +5293,7 @@
         <v>10</v>
       </c>
       <c r="J132" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
     </row>
     <row r="133" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5313,7 +5313,7 @@
         <v>10</v>
       </c>
       <c r="J133" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
     </row>
     <row r="134" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5333,7 +5333,7 @@
         <v>10</v>
       </c>
       <c r="J134" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="135" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5353,7 +5353,7 @@
         <v>10</v>
       </c>
       <c r="J135" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
     </row>
     <row r="136" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5373,7 +5373,7 @@
         <v>10</v>
       </c>
       <c r="J136" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
     </row>
     <row r="137" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5393,7 +5393,7 @@
         <v>10</v>
       </c>
       <c r="J137" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
     </row>
     <row r="138" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5453,7 +5453,7 @@
         <v>10</v>
       </c>
       <c r="J140" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="141" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5473,7 +5473,7 @@
         <v>10</v>
       </c>
       <c r="J141" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
     </row>
     <row r="142" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5516,7 +5516,7 @@
         <v>10</v>
       </c>
       <c r="J143" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
     </row>
     <row r="144" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5536,7 +5536,7 @@
         <v>10</v>
       </c>
       <c r="J144" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
     </row>
     <row r="145" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5556,7 +5556,7 @@
         <v>10</v>
       </c>
       <c r="J145" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
     </row>
     <row r="146" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5576,7 +5576,7 @@
         <v>10</v>
       </c>
       <c r="J146" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
     </row>
     <row r="147" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5596,7 +5596,7 @@
         <v>10</v>
       </c>
       <c r="J147" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
     </row>
     <row r="148" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5616,7 +5616,7 @@
         <v>10</v>
       </c>
       <c r="J148" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
     </row>
     <row r="149" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5636,7 +5636,7 @@
         <v>10</v>
       </c>
       <c r="J149" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
     </row>
     <row r="150" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5716,7 +5716,7 @@
         <v>10</v>
       </c>
       <c r="J153" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="154" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5736,7 +5736,7 @@
         <v>10</v>
       </c>
       <c r="J154" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="155" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5756,7 +5756,7 @@
         <v>10</v>
       </c>
       <c r="J155" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
     </row>
     <row r="156" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5776,7 +5776,7 @@
         <v>10</v>
       </c>
       <c r="J156" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
     </row>
     <row r="157" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5796,7 +5796,7 @@
         <v>10</v>
       </c>
       <c r="J157" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
     </row>
     <row r="158" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5816,7 +5816,7 @@
         <v>10</v>
       </c>
       <c r="J158" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
     </row>
     <row r="159" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5836,7 +5836,7 @@
         <v>10</v>
       </c>
       <c r="J159" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
     </row>
     <row r="160" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5856,7 +5856,7 @@
         <v>10</v>
       </c>
       <c r="J160" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
     </row>
     <row r="161" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5876,7 +5876,7 @@
         <v>10</v>
       </c>
       <c r="J161" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
     </row>
     <row r="162" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5896,7 +5896,7 @@
         <v>10</v>
       </c>
       <c r="J162" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="163" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5916,7 +5916,7 @@
         <v>10</v>
       </c>
       <c r="J163" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="164" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5936,7 +5936,7 @@
         <v>10</v>
       </c>
       <c r="J164" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="165" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5956,7 +5956,7 @@
         <v>10</v>
       </c>
       <c r="J165" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="166" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5976,7 +5976,7 @@
         <v>10</v>
       </c>
       <c r="J166" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="167" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5996,7 +5996,7 @@
         <v>10</v>
       </c>
       <c r="J167" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="168" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6019,7 +6019,7 @@
         <v>10</v>
       </c>
       <c r="J168" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="169" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6039,7 +6039,7 @@
         <v>10</v>
       </c>
       <c r="J169" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="170" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6059,7 +6059,7 @@
         <v>10</v>
       </c>
       <c r="J170" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="171" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6079,7 +6079,7 @@
         <v>10</v>
       </c>
       <c r="J171" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
     </row>
     <row r="172" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6099,7 +6099,7 @@
         <v>10</v>
       </c>
       <c r="J172" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
     </row>
     <row r="173" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6119,7 +6119,7 @@
         <v>10</v>
       </c>
       <c r="J173" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
     </row>
     <row r="174" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6139,7 +6139,7 @@
         <v>10</v>
       </c>
       <c r="J174" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
     </row>
     <row r="175" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6159,7 +6159,7 @@
         <v>10</v>
       </c>
       <c r="J175" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="176" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6179,7 +6179,7 @@
         <v>10</v>
       </c>
       <c r="J176" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
     </row>
     <row r="177" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6199,7 +6199,7 @@
         <v>10</v>
       </c>
       <c r="J177" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
     </row>
     <row r="178" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6219,7 +6219,7 @@
         <v>10</v>
       </c>
       <c r="J178" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
     </row>
     <row r="179" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6239,7 +6239,7 @@
         <v>10</v>
       </c>
       <c r="J179" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
     </row>
     <row r="180" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6262,7 +6262,7 @@
         <v>10</v>
       </c>
       <c r="J180" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
     </row>
     <row r="181" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6285,7 +6285,7 @@
         <v>10</v>
       </c>
       <c r="J181" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
     </row>
     <row r="182" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6308,7 +6308,7 @@
         <v>10</v>
       </c>
       <c r="J182" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="183" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6331,7 +6331,7 @@
         <v>10</v>
       </c>
       <c r="J183" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="184" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6354,7 +6354,7 @@
         <v>10</v>
       </c>
       <c r="J184" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="185" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6374,7 +6374,7 @@
         <v>10</v>
       </c>
       <c r="J185" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="186" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6394,7 +6394,7 @@
         <v>10</v>
       </c>
       <c r="J186" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="187" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6414,7 +6414,7 @@
         <v>10</v>
       </c>
       <c r="J187" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
     </row>
     <row r="188" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6454,7 +6454,7 @@
         <v>10</v>
       </c>
       <c r="J189" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="190" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6474,7 +6474,7 @@
         <v>10</v>
       </c>
       <c r="J190" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
     </row>
     <row r="191" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6494,7 +6494,7 @@
         <v>10</v>
       </c>
       <c r="J191" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="192" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6514,7 +6514,7 @@
         <v>10</v>
       </c>
       <c r="J192" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
     </row>
     <row r="193" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6534,7 +6534,7 @@
         <v>10</v>
       </c>
       <c r="J193" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
     </row>
     <row r="194" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6554,7 +6554,7 @@
         <v>10</v>
       </c>
       <c r="J194" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="195" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6574,7 +6574,7 @@
         <v>10</v>
       </c>
       <c r="J195" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
     </row>
     <row r="196" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6594,7 +6594,7 @@
         <v>10</v>
       </c>
       <c r="J196" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
     </row>
     <row r="197" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6614,7 +6614,7 @@
         <v>10</v>
       </c>
       <c r="J197" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
     </row>
     <row r="198" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6634,7 +6634,7 @@
         <v>10</v>
       </c>
       <c r="J198" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="199" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6654,7 +6654,7 @@
         <v>10</v>
       </c>
       <c r="J199" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="200" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6674,7 +6674,7 @@
         <v>10</v>
       </c>
       <c r="J200" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="201" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6694,7 +6694,7 @@
         <v>10</v>
       </c>
       <c r="J201" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="202" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6714,7 +6714,7 @@
         <v>10</v>
       </c>
       <c r="J202" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="203" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6737,7 +6737,7 @@
         <v>10</v>
       </c>
       <c r="J203" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="204" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6760,7 +6760,7 @@
         <v>10</v>
       </c>
       <c r="J204" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
     </row>
     <row r="205" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6783,7 +6783,7 @@
         <v>10</v>
       </c>
       <c r="J205" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
     </row>
     <row r="206" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6806,7 +6806,7 @@
         <v>10</v>
       </c>
       <c r="J206" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
     </row>
     <row r="207" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6829,7 +6829,7 @@
         <v>10</v>
       </c>
       <c r="J207" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="208" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6852,10 +6852,10 @@
         <v>10</v>
       </c>
       <c r="J208" t="s">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="209" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="209" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A209" s="4" t="s">
         <v>27</v>
       </c>
@@ -6875,10 +6875,10 @@
         <v>10</v>
       </c>
       <c r="J209" s="5" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="210" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="210" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A210" s="4" t="s">
         <v>27</v>
       </c>
@@ -6898,10 +6898,10 @@
         <v>10</v>
       </c>
       <c r="J210" s="5" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="211" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="211" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A211" s="4" t="s">
         <v>27</v>
       </c>
@@ -6921,7 +6921,7 @@
         <v>10</v>
       </c>
       <c r="J211" s="5" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
     <row r="212" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6944,10 +6944,10 @@
         <v>10</v>
       </c>
       <c r="J212" s="5" t="s">
-        <v>472</v>
-      </c>
-    </row>
-    <row r="213" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="213" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A213" s="4" t="s">
         <v>27</v>
       </c>
@@ -6964,10 +6964,10 @@
         <v>10</v>
       </c>
       <c r="J213" s="5" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="214" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="214" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A214" s="4" t="s">
         <v>27</v>
       </c>
@@ -6984,7 +6984,7 @@
         <v>10</v>
       </c>
       <c r="J214" s="5" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="215" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7004,7 +7004,7 @@
         <v>10</v>
       </c>
       <c r="J215" s="5" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="216" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7027,7 +7027,7 @@
         <v>10</v>
       </c>
       <c r="J216" s="5" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="217" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7050,10 +7050,10 @@
         <v>10</v>
       </c>
       <c r="J217" s="5" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="218" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="218" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A218" s="4" t="s">
         <v>27</v>
       </c>
@@ -7073,7 +7073,7 @@
         <v>10</v>
       </c>
       <c r="J218" s="5" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="219" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7093,7 +7093,7 @@
         <v>10</v>
       </c>
       <c r="J219" s="5" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
     </row>
     <row r="220" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7113,10 +7113,10 @@
         <v>10</v>
       </c>
       <c r="J220" s="5" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="221" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="221" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A221" s="4" t="s">
         <v>27</v>
       </c>
@@ -7133,10 +7133,10 @@
         <v>10</v>
       </c>
       <c r="J221" s="5" t="s">
-        <v>481</v>
-      </c>
-    </row>
-    <row r="222" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="222" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A222" s="4" t="s">
         <v>27</v>
       </c>
@@ -7153,10 +7153,10 @@
         <v>10</v>
       </c>
       <c r="J222" s="5" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="223" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="223" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A223" s="4" t="s">
         <v>27</v>
       </c>
@@ -7173,7 +7173,7 @@
         <v>10</v>
       </c>
       <c r="J223" s="5" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
     </row>
     <row r="224" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7193,7 +7193,7 @@
         <v>10</v>
       </c>
       <c r="J224" s="5" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="225" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7213,7 +7213,7 @@
         <v>10</v>
       </c>
       <c r="J225" s="5" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
     <row r="226" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7233,7 +7233,7 @@
         <v>10</v>
       </c>
       <c r="J226" s="5" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
     </row>
     <row r="227" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7253,7 +7253,7 @@
         <v>10</v>
       </c>
       <c r="J227" s="5" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
     </row>
     <row r="228" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7273,10 +7273,10 @@
         <v>10</v>
       </c>
       <c r="J228" s="5" t="s">
-        <v>488</v>
-      </c>
-    </row>
-    <row r="229" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="229" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A229" s="4" t="s">
         <v>27</v>
       </c>
@@ -7293,7 +7293,7 @@
         <v>10</v>
       </c>
       <c r="J229" s="5" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="230" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7316,7 +7316,7 @@
         <v>10</v>
       </c>
       <c r="J230" s="5" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="231" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7339,7 +7339,7 @@
         <v>10</v>
       </c>
       <c r="J231" s="5" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="232" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7362,7 +7362,7 @@
         <v>10</v>
       </c>
       <c r="J232" s="5" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
     </row>
     <row r="233" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7385,10 +7385,10 @@
         <v>10</v>
       </c>
       <c r="J233" s="5" t="s">
-        <v>493</v>
-      </c>
-    </row>
-    <row r="234" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="234" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A234" s="4" t="s">
         <v>27</v>
       </c>
@@ -7408,7 +7408,7 @@
         <v>10</v>
       </c>
       <c r="J234" s="5" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
     </row>
     <row r="235" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7431,10 +7431,10 @@
         <v>10</v>
       </c>
       <c r="J235" s="5" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="236" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="236" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A236" s="4" t="s">
         <v>27</v>
       </c>
@@ -7454,10 +7454,10 @@
         <v>10</v>
       </c>
       <c r="J236" s="5" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="237" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="237" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A237" s="4" t="s">
         <v>27</v>
       </c>
@@ -7477,7 +7477,7 @@
         <v>10</v>
       </c>
       <c r="J237" s="5" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
     </row>
     <row r="238" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7497,10 +7497,10 @@
         <v>10</v>
       </c>
       <c r="J238" s="5" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="239" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="239" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A239" s="4" t="s">
         <v>27</v>
       </c>
@@ -7520,7 +7520,7 @@
         <v>10</v>
       </c>
       <c r="J239" s="5" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
     </row>
     <row r="240" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7540,7 +7540,7 @@
         <v>10</v>
       </c>
       <c r="J240" s="5" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="241" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7563,7 +7563,7 @@
         <v>10</v>
       </c>
       <c r="J241" s="5" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
     </row>
     <row r="242" spans="1:10" ht="32" x14ac:dyDescent="0.2">
@@ -7583,7 +7583,7 @@
         <v>10</v>
       </c>
       <c r="J242" s="5" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="243" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7603,7 +7603,7 @@
         <v>10</v>
       </c>
       <c r="J243" s="5" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="244" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7626,7 +7626,7 @@
         <v>10</v>
       </c>
       <c r="J244" s="5" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
     </row>
     <row r="245" spans="1:10" ht="32" x14ac:dyDescent="0.2">
@@ -7646,7 +7646,7 @@
         <v>10</v>
       </c>
       <c r="J245" s="5" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
     </row>
     <row r="246" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7666,7 +7666,7 @@
         <v>10</v>
       </c>
       <c r="J246" s="5" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="247" spans="1:10" ht="32" x14ac:dyDescent="0.2">
@@ -7686,7 +7686,7 @@
         <v>10</v>
       </c>
       <c r="J247" s="5" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="248" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7706,7 +7706,7 @@
         <v>10</v>
       </c>
       <c r="J248" s="5" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="249" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7726,7 +7726,7 @@
         <v>10</v>
       </c>
       <c r="J249" s="5" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
     </row>
     <row r="250" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7746,7 +7746,7 @@
         <v>10</v>
       </c>
       <c r="J250" s="5" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="251" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7766,7 +7766,7 @@
         <v>10</v>
       </c>
       <c r="J251" s="5" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="252" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7786,7 +7786,7 @@
         <v>10</v>
       </c>
       <c r="J252" s="5" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
     </row>
     <row r="253" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7806,7 +7806,7 @@
         <v>10</v>
       </c>
       <c r="J253" s="5" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
     </row>
     <row r="254" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7826,7 +7826,7 @@
         <v>10</v>
       </c>
       <c r="J254" s="5" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
     </row>
     <row r="255" spans="1:10" ht="32" x14ac:dyDescent="0.2">
@@ -7846,10 +7846,10 @@
         <v>10</v>
       </c>
       <c r="J255" s="5" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="256" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="256" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A256" s="4" t="s">
         <v>29</v>
       </c>
@@ -7866,7 +7866,7 @@
         <v>10</v>
       </c>
       <c r="J256" s="5" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
     </row>
     <row r="257" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7886,7 +7886,7 @@
         <v>10</v>
       </c>
       <c r="J257" s="5" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="258" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7906,7 +7906,7 @@
         <v>10</v>
       </c>
       <c r="J258" s="5" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="259" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7926,7 +7926,7 @@
         <v>10</v>
       </c>
       <c r="J259" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="260" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7946,7 +7946,7 @@
         <v>10</v>
       </c>
       <c r="J260" s="5" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="261" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7966,7 +7966,7 @@
         <v>10</v>
       </c>
       <c r="J261" s="5" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
     </row>
     <row r="262" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7986,10 +7986,10 @@
         <v>10</v>
       </c>
       <c r="J262" s="5" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="263" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="263" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A263" s="4" t="s">
         <v>29</v>
       </c>
@@ -8006,10 +8006,10 @@
         <v>10</v>
       </c>
       <c r="J263" s="5" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="264" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="264" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A264" s="4" t="s">
         <v>29</v>
       </c>
@@ -8026,7 +8026,7 @@
         <v>10</v>
       </c>
       <c r="J264" s="5" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="265" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8046,7 +8046,7 @@
         <v>10</v>
       </c>
       <c r="J265" s="5" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="266" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8066,7 +8066,7 @@
         <v>10</v>
       </c>
       <c r="J266" s="5" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="267" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8086,7 +8086,7 @@
         <v>10</v>
       </c>
       <c r="J267" s="5" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
     </row>
     <row r="268" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8106,7 +8106,7 @@
         <v>10</v>
       </c>
       <c r="J268" s="5" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="269" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8126,7 +8126,7 @@
         <v>10</v>
       </c>
       <c r="J269" s="5" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="270" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8146,7 +8146,7 @@
         <v>10</v>
       </c>
       <c r="J270" s="5" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
     </row>
     <row r="271" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8166,7 +8166,7 @@
         <v>10</v>
       </c>
       <c r="J271" s="5" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
     </row>
     <row r="272" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8186,10 +8186,10 @@
         <v>10</v>
       </c>
       <c r="J272" s="5" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="273" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="273" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A273" s="4" t="s">
         <v>29</v>
       </c>
@@ -8206,7 +8206,7 @@
         <v>10</v>
       </c>
       <c r="J273" s="5" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
     </row>
     <row r="274" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8226,7 +8226,7 @@
         <v>10</v>
       </c>
       <c r="J274" s="5" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
     </row>
     <row r="275" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8246,10 +8246,10 @@
         <v>10</v>
       </c>
       <c r="J275" s="5" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="276" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="276" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A276" s="4" t="s">
         <v>29</v>
       </c>
@@ -8266,7 +8266,7 @@
         <v>10</v>
       </c>
       <c r="J276" s="5" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
     </row>
     <row r="277" spans="1:10" ht="32" x14ac:dyDescent="0.2">
@@ -8286,7 +8286,7 @@
         <v>10</v>
       </c>
       <c r="J277" s="5" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
     </row>
     <row r="278" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8306,7 +8306,7 @@
         <v>10</v>
       </c>
       <c r="J278" s="5" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
     </row>
     <row r="279" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8326,10 +8326,10 @@
         <v>10</v>
       </c>
       <c r="J279" s="5" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="280" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="280" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A280" s="4" t="s">
         <v>29</v>
       </c>
@@ -8346,7 +8346,7 @@
         <v>10</v>
       </c>
       <c r="J280" s="5" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
     </row>
     <row r="281" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8366,7 +8366,7 @@
         <v>10</v>
       </c>
       <c r="J281" s="5" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
     </row>
     <row r="282" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8386,7 +8386,7 @@
         <v>10</v>
       </c>
       <c r="J282" s="5" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
     </row>
     <row r="283" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8406,7 +8406,7 @@
         <v>10</v>
       </c>
       <c r="J283" s="5" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
     </row>
     <row r="284" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8426,10 +8426,10 @@
         <v>10</v>
       </c>
       <c r="J284" s="5" t="s">
-        <v>535</v>
-      </c>
-    </row>
-    <row r="285" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="285" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A285" s="4" t="s">
         <v>29</v>
       </c>
@@ -8446,10 +8446,10 @@
         <v>10</v>
       </c>
       <c r="J285" s="5" t="s">
-        <v>536</v>
-      </c>
-    </row>
-    <row r="286" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="286" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A286" s="4" t="s">
         <v>29</v>
       </c>
@@ -8466,7 +8466,7 @@
         <v>10</v>
       </c>
       <c r="J286" s="5" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
     </row>
     <row r="287" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8486,7 +8486,7 @@
         <v>10</v>
       </c>
       <c r="J287" s="5" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="288" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8506,7 +8506,7 @@
         <v>10</v>
       </c>
       <c r="J288" s="5" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="289" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8526,7 +8526,7 @@
         <v>10</v>
       </c>
       <c r="J289" s="5" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
     </row>
     <row r="290" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8546,7 +8546,7 @@
         <v>10</v>
       </c>
       <c r="J290" s="5" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
     </row>
     <row r="291" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8566,7 +8566,7 @@
         <v>10</v>
       </c>
       <c r="J291" s="5" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
     </row>
     <row r="292" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8586,10 +8586,10 @@
         <v>10</v>
       </c>
       <c r="J292" s="5" t="s">
-        <v>543</v>
-      </c>
-    </row>
-    <row r="293" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="293" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A293" s="4" t="s">
         <v>29</v>
       </c>
@@ -8606,7 +8606,7 @@
         <v>10</v>
       </c>
       <c r="J293" s="5" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="294" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8626,7 +8626,7 @@
         <v>10</v>
       </c>
       <c r="J294" s="5" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
     </row>
     <row r="295" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8646,10 +8646,10 @@
         <v>10</v>
       </c>
       <c r="J295" s="5" t="s">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="296" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="296" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A296" s="4" t="s">
         <v>29</v>
       </c>
@@ -8666,7 +8666,7 @@
         <v>10</v>
       </c>
       <c r="J296" s="5" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
     </row>
     <row r="297" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8686,7 +8686,7 @@
         <v>10</v>
       </c>
       <c r="J297" s="5" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="298" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8709,10 +8709,10 @@
         <v>10</v>
       </c>
       <c r="J298" s="5" t="s">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="299" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="299" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A299" s="4" t="s">
         <v>29</v>
       </c>
@@ -8732,10 +8732,10 @@
         <v>10</v>
       </c>
       <c r="J299" s="5" t="s">
-        <v>549</v>
-      </c>
-    </row>
-    <row r="300" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="300" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A300" s="4" t="s">
         <v>29</v>
       </c>
@@ -8755,10 +8755,10 @@
         <v>10</v>
       </c>
       <c r="J300" s="5" t="s">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="301" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="301" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A301" s="4" t="s">
         <v>29</v>
       </c>
@@ -8778,10 +8778,10 @@
         <v>10</v>
       </c>
       <c r="J301" s="5" t="s">
-        <v>551</v>
-      </c>
-    </row>
-    <row r="302" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="302" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A302" s="4" t="s">
         <v>29</v>
       </c>
@@ -8801,10 +8801,10 @@
         <v>10</v>
       </c>
       <c r="J302" s="5" t="s">
-        <v>552</v>
-      </c>
-    </row>
-    <row r="303" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="303" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A303" s="4" t="s">
         <v>29</v>
       </c>
@@ -8824,7 +8824,7 @@
         <v>10</v>
       </c>
       <c r="J303" s="5" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
     </row>
     <row r="304" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8847,10 +8847,10 @@
         <v>10</v>
       </c>
       <c r="J304" s="5" t="s">
-        <v>554</v>
-      </c>
-    </row>
-    <row r="305" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="305" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A305" s="4" t="s">
         <v>29</v>
       </c>
@@ -8870,10 +8870,10 @@
         <v>10</v>
       </c>
       <c r="J305" s="5" t="s">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="306" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="306" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A306" s="4" t="s">
         <v>29</v>
       </c>
@@ -8893,7 +8893,7 @@
         <v>10</v>
       </c>
       <c r="J306" s="5" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
     </row>
     <row r="307" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8916,7 +8916,7 @@
         <v>10</v>
       </c>
       <c r="J307" s="5" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="308" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8939,10 +8939,10 @@
         <v>10</v>
       </c>
       <c r="J308" s="5" t="s">
-        <v>558</v>
-      </c>
-    </row>
-    <row r="309" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="309" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A309" s="4" t="s">
         <v>29</v>
       </c>
@@ -8962,7 +8962,7 @@
         <v>10</v>
       </c>
       <c r="J309" s="5" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
     </row>
     <row r="310" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8985,10 +8985,10 @@
         <v>10</v>
       </c>
       <c r="J310" s="5" t="s">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="311" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="311" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A311" s="4" t="s">
         <v>29</v>
       </c>
@@ -9008,10 +9008,10 @@
         <v>10</v>
       </c>
       <c r="J311" s="5" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="312" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="312" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A312" s="4" t="s">
         <v>29</v>
       </c>
@@ -9031,7 +9031,7 @@
         <v>10</v>
       </c>
       <c r="J312" s="5" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="313" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9054,7 +9054,7 @@
         <v>10</v>
       </c>
       <c r="J313" s="5" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="314" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9077,7 +9077,7 @@
         <v>10</v>
       </c>
       <c r="J314" s="5" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="315" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9097,7 +9097,7 @@
         <v>10</v>
       </c>
       <c r="J315" s="5" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="316" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9117,10 +9117,10 @@
         <v>10</v>
       </c>
       <c r="J316" s="5" t="s">
-        <v>566</v>
-      </c>
-    </row>
-    <row r="317" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="317" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A317" s="4" t="s">
         <v>29</v>
       </c>
@@ -9137,7 +9137,7 @@
         <v>10</v>
       </c>
       <c r="J317" s="5" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="318" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9157,7 +9157,7 @@
         <v>10</v>
       </c>
       <c r="J318" s="5" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="319" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9177,7 +9177,7 @@
         <v>10</v>
       </c>
       <c r="J319" s="5" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="320" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9197,10 +9197,10 @@
         <v>10</v>
       </c>
       <c r="J320" s="5" t="s">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="321" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="321" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A321" s="4" t="s">
         <v>29</v>
       </c>
@@ -9217,7 +9217,7 @@
         <v>10</v>
       </c>
       <c r="J321" s="5" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="322" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9237,7 +9237,7 @@
         <v>10</v>
       </c>
       <c r="J322" s="5" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
     </row>
     <row r="323" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9257,7 +9257,7 @@
         <v>10</v>
       </c>
       <c r="J323" s="5" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
     </row>
     <row r="324" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9277,7 +9277,7 @@
         <v>10</v>
       </c>
       <c r="J324" s="5" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="325" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9297,10 +9297,10 @@
         <v>10</v>
       </c>
       <c r="J325" s="5" t="s">
-        <v>575</v>
-      </c>
-    </row>
-    <row r="326" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="326" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A326" s="4" t="s">
         <v>29</v>
       </c>
@@ -9320,10 +9320,10 @@
         <v>10</v>
       </c>
       <c r="J326" s="5" t="s">
-        <v>576</v>
-      </c>
-    </row>
-    <row r="327" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="327" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A327" s="4" t="s">
         <v>29</v>
       </c>
@@ -9343,7 +9343,7 @@
         <v>10</v>
       </c>
       <c r="J327" s="5" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="328" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9366,7 +9366,7 @@
         <v>10</v>
       </c>
       <c r="J328" s="5" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="329" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9386,7 +9386,7 @@
         <v>10</v>
       </c>
       <c r="J329" s="5" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="330" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9406,7 +9406,7 @@
         <v>10</v>
       </c>
       <c r="J330" s="5" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
     <row r="331" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9426,7 +9426,7 @@
         <v>10</v>
       </c>
       <c r="J331" s="5" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="332" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9446,7 +9446,7 @@
         <v>10</v>
       </c>
       <c r="J332" s="5" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="333" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9466,7 +9466,7 @@
         <v>10</v>
       </c>
       <c r="J333" s="5" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="334" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9489,7 +9489,7 @@
         <v>10</v>
       </c>
       <c r="J334" s="5" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="335" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9512,7 +9512,7 @@
         <v>10</v>
       </c>
       <c r="J335" s="5" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="336" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9532,7 +9532,7 @@
         <v>10</v>
       </c>
       <c r="J336" s="5" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
     <row r="337" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9552,7 +9552,7 @@
         <v>10</v>
       </c>
       <c r="J337" s="5" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="338" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9575,7 +9575,7 @@
         <v>10</v>
       </c>
       <c r="J338" s="5" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="339" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9598,7 +9598,7 @@
         <v>10</v>
       </c>
       <c r="J339" s="5" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
     </row>
     <row r="340" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9618,7 +9618,7 @@
         <v>10</v>
       </c>
       <c r="J340" s="5" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
     </row>
     <row r="341" spans="1:10" ht="32" x14ac:dyDescent="0.2">
@@ -9641,7 +9641,7 @@
         <v>10</v>
       </c>
       <c r="J341" s="5" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="342" spans="1:10" ht="32" x14ac:dyDescent="0.2">
@@ -9661,7 +9661,7 @@
         <v>10</v>
       </c>
       <c r="J342" s="5" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
     </row>
     <row r="343" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9681,7 +9681,7 @@
         <v>10</v>
       </c>
       <c r="J343" s="5" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="344" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9704,7 +9704,7 @@
         <v>10</v>
       </c>
       <c r="J344" s="5" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Update aggregation time dimension from cif_open_date to as_of_date in customer_icons metrics
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8577950B-F469-5D41-B8C7-D3F520D383FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAE2D0E5-A2FC-754C-9BB6-E026923EE0B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="660" windowWidth="30680" windowHeight="19740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2648,7 +2648,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>22</v>
       </c>
@@ -3432,7 +3432,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>23</v>
       </c>
@@ -3590,9 +3590,6 @@
       </c>
       <c r="D47" s="4" t="b">
         <v>0</v>
-      </c>
-      <c r="E47" s="4" t="b">
-        <v>1</v>
       </c>
       <c r="H47" s="4" t="s">
         <v>10</v>
@@ -6855,7 +6852,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="209" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A209" s="4" t="s">
         <v>27</v>
       </c>
@@ -6878,7 +6875,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="210" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A210" s="4" t="s">
         <v>27</v>
       </c>
@@ -6901,7 +6898,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="211" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A211" s="4" t="s">
         <v>27</v>
       </c>
@@ -6947,7 +6944,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="213" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A213" s="4" t="s">
         <v>27</v>
       </c>
@@ -6967,7 +6964,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="214" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A214" s="4" t="s">
         <v>27</v>
       </c>
@@ -7053,7 +7050,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="218" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A218" s="4" t="s">
         <v>27</v>
       </c>
@@ -7116,7 +7113,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="221" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A221" s="4" t="s">
         <v>27</v>
       </c>
@@ -7136,7 +7133,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="222" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A222" s="4" t="s">
         <v>27</v>
       </c>
@@ -7156,7 +7153,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="223" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A223" s="4" t="s">
         <v>27</v>
       </c>
@@ -7276,7 +7273,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="229" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A229" s="4" t="s">
         <v>27</v>
       </c>
@@ -7388,7 +7385,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="234" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A234" s="4" t="s">
         <v>27</v>
       </c>
@@ -7434,7 +7431,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="236" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A236" s="4" t="s">
         <v>27</v>
       </c>
@@ -7457,7 +7454,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="237" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A237" s="4" t="s">
         <v>27</v>
       </c>
@@ -7500,7 +7497,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="239" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A239" s="4" t="s">
         <v>27</v>
       </c>
@@ -7566,7 +7563,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="242" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A242" s="4" t="s">
         <v>29</v>
       </c>
@@ -7629,7 +7626,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="245" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A245" s="4" t="s">
         <v>29</v>
       </c>
@@ -7669,7 +7666,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="247" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A247" s="4" t="s">
         <v>29</v>
       </c>
@@ -7829,7 +7826,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="255" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A255" s="4" t="s">
         <v>29</v>
       </c>
@@ -7849,7 +7846,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="256" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A256" s="4" t="s">
         <v>29</v>
       </c>
@@ -7989,7 +7986,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="263" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A263" s="4" t="s">
         <v>29</v>
       </c>
@@ -8009,7 +8006,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="264" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A264" s="4" t="s">
         <v>29</v>
       </c>
@@ -8189,7 +8186,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="273" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A273" s="4" t="s">
         <v>29</v>
       </c>
@@ -8249,7 +8246,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="276" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A276" s="4" t="s">
         <v>29</v>
       </c>
@@ -8269,7 +8266,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="277" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A277" s="4" t="s">
         <v>29</v>
       </c>
@@ -8329,7 +8326,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="280" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A280" s="4" t="s">
         <v>29</v>
       </c>
@@ -8429,7 +8426,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="285" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A285" s="4" t="s">
         <v>29</v>
       </c>
@@ -8449,7 +8446,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="286" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A286" s="4" t="s">
         <v>29</v>
       </c>
@@ -8589,7 +8586,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="293" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A293" s="4" t="s">
         <v>29</v>
       </c>
@@ -8649,7 +8646,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="296" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A296" s="4" t="s">
         <v>29</v>
       </c>
@@ -8712,7 +8709,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="299" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A299" s="4" t="s">
         <v>29</v>
       </c>
@@ -8735,7 +8732,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="300" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="300" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A300" s="4" t="s">
         <v>29</v>
       </c>
@@ -8758,7 +8755,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="301" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="301" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A301" s="4" t="s">
         <v>29</v>
       </c>
@@ -8781,7 +8778,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="302" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="302" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A302" s="4" t="s">
         <v>29</v>
       </c>
@@ -8804,7 +8801,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="303" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="303" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A303" s="4" t="s">
         <v>29</v>
       </c>
@@ -8850,7 +8847,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="305" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="305" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A305" s="4" t="s">
         <v>29</v>
       </c>
@@ -8873,7 +8870,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="306" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="306" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A306" s="4" t="s">
         <v>29</v>
       </c>
@@ -8942,7 +8939,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="309" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="309" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A309" s="4" t="s">
         <v>29</v>
       </c>
@@ -8988,7 +8985,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="311" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="311" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A311" s="4" t="s">
         <v>29</v>
       </c>
@@ -9011,7 +9008,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="312" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="312" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A312" s="4" t="s">
         <v>29</v>
       </c>
@@ -9120,7 +9117,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="317" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="317" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A317" s="4" t="s">
         <v>29</v>
       </c>
@@ -9200,7 +9197,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="321" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="321" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A321" s="4" t="s">
         <v>29</v>
       </c>
@@ -9300,7 +9297,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="326" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="326" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A326" s="4" t="s">
         <v>29</v>
       </c>
@@ -9323,7 +9320,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="327" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="327" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A327" s="4" t="s">
         <v>29</v>
       </c>
@@ -9621,7 +9618,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="341" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="341" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A341" s="4" t="s">
         <v>407</v>
       </c>
@@ -9644,7 +9641,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="342" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="342" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A342" s="4" t="s">
         <v>407</v>
       </c>

</xml_diff>

<commit_message>
feat: Enhance draft SQL task with default time axis and join alignment rules
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAE2D0E5-A2FC-754C-9BB6-E026923EE0B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{222849E5-03C4-9143-A1A0-2D39E2730B81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="660" windowWidth="30680" windowHeight="19740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="660" windowWidth="30680" windowHeight="19740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tables" sheetId="1" r:id="rId1"/>
@@ -19,14 +19,14 @@
     <sheet name="Golden_Queries" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Columns!$A$1:$J$344</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Columns!$A$1:$J$345</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1883" uniqueCount="704">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1888" uniqueCount="705">
   <si>
     <t>Table Name</t>
   </si>
@@ -1378,9 +1378,6 @@
     <t>Wonder</t>
   </si>
   <si>
-    <t>Tanggal Transaksi Data, digunakan untuk filter tanggal, bulan, tahun</t>
-  </si>
-  <si>
     <t>SELECT * FROM dm_transaction.trxchannel WHERE destination_bankname &lt;&gt; 'BANK NEGARA INDONESIA';</t>
   </si>
   <si>
@@ -1528,9 +1525,6 @@
     <t>Hasil mapping/mirror dari pemilik channel.</t>
   </si>
   <si>
-    <t>Tanggal posisi atau snapshot data.</t>
-  </si>
-  <si>
     <t>ID nasabah/entity pada sistem Master Data Management.</t>
   </si>
   <si>
@@ -1798,9 +1792,6 @@
     <t>Nasabah/perusahaan utama dalam satu kelompok usaha atau grup.</t>
   </si>
   <si>
-    <t>Tanggal posisi/snapshot data.</t>
-  </si>
-  <si>
     <t>CIF Key Nasabah (ID Nasabah)</t>
   </si>
   <si>
@@ -2134,10 +2125,22 @@
     <t>Divisi pemilik segmen.</t>
   </si>
   <si>
-    <t>Tanggal snapshot customer, digunakan untuk filter tanggal, bulan, tahun</t>
-  </si>
-  <si>
     <t>Nilai Transaksi / Transaction Amount / Amount Transaksi</t>
+  </si>
+  <si>
+    <t>Tanggal posisi atau snapshot data pada table funding. Digunakan untuk filter tanggal, bulan, tahun</t>
+  </si>
+  <si>
+    <t>Tanggal posisi atau snapshot data pada table lending. Digunakan untuk filter tanggal, bulan, tahun</t>
+  </si>
+  <si>
+    <t>Tanggal posisi atau snapshot data pada table mapping_group_whs. Digunakan untuk filter tanggal, bulan, tahun</t>
+  </si>
+  <si>
+    <t>Tanggal posisi atau snapshot data pada table customer / nasabah. Digunakan untuk filter tanggal, bulan, tahun</t>
+  </si>
+  <si>
+    <t>Tanggal posisi atau tanggal transaksi data, digunakan untuk filter tanggal, bulan, tahun</t>
   </si>
 </sst>
 </file>
@@ -2600,7 +2603,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J344"/>
+  <dimension ref="A1:J345"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.5" style="4" customWidth="1"/>
@@ -2668,7 +2671,7 @@
         <v>10</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>450</v>
+        <v>704</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2711,7 +2714,7 @@
         <v>10</v>
       </c>
       <c r="J4" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="32" x14ac:dyDescent="0.2">
@@ -2734,7 +2737,7 @@
         <v>10</v>
       </c>
       <c r="J5" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2960,7 +2963,7 @@
         <v>10</v>
       </c>
       <c r="J16" t="s">
-        <v>703</v>
+        <v>699</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3246,7 +3249,7 @@
         <v>10</v>
       </c>
       <c r="J30" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3266,7 +3269,7 @@
         <v>10</v>
       </c>
       <c r="J31" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3432,7 +3435,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>23</v>
       </c>
@@ -3451,8 +3454,8 @@
       <c r="H40" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J40" s="4" t="s">
-        <v>702</v>
+      <c r="J40" s="5" t="s">
+        <v>703</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3535,7 +3538,7 @@
         <v>10</v>
       </c>
       <c r="J44" t="s">
-        <v>593</v>
+        <v>590</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3958,7 +3961,7 @@
         <v>10</v>
       </c>
       <c r="J65" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
     </row>
     <row r="66" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3978,7 +3981,7 @@
         <v>10</v>
       </c>
       <c r="J66" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
     </row>
     <row r="67" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3998,7 +4001,7 @@
         <v>10</v>
       </c>
       <c r="J67" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
     </row>
     <row r="68" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4021,7 +4024,7 @@
         <v>10</v>
       </c>
       <c r="J68" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
     </row>
     <row r="69" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4041,7 +4044,7 @@
         <v>10</v>
       </c>
       <c r="J69" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
     </row>
     <row r="70" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4061,7 +4064,7 @@
         <v>10</v>
       </c>
       <c r="J70" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
     </row>
     <row r="71" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4121,7 +4124,7 @@
         <v>10</v>
       </c>
       <c r="J73" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
     </row>
     <row r="74" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4221,7 +4224,7 @@
         <v>10</v>
       </c>
       <c r="J78" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
     </row>
     <row r="79" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4241,7 +4244,7 @@
         <v>10</v>
       </c>
       <c r="J79" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
     </row>
     <row r="80" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4261,7 +4264,7 @@
         <v>10</v>
       </c>
       <c r="J80" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
     </row>
     <row r="81" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4281,7 +4284,7 @@
         <v>10</v>
       </c>
       <c r="J81" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
     </row>
     <row r="82" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4301,7 +4304,7 @@
         <v>10</v>
       </c>
       <c r="J82" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
     </row>
     <row r="83" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4357,7 +4360,7 @@
         <v>10</v>
       </c>
       <c r="J85" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
     </row>
     <row r="86" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4431,7 +4434,7 @@
         <v>10</v>
       </c>
       <c r="J89" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
     </row>
     <row r="90" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4451,7 +4454,7 @@
         <v>10</v>
       </c>
       <c r="J90" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
     </row>
     <row r="91" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4471,7 +4474,7 @@
         <v>10</v>
       </c>
       <c r="J91" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
     </row>
     <row r="92" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4491,7 +4494,7 @@
         <v>10</v>
       </c>
       <c r="J92" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
     </row>
     <row r="93" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4511,7 +4514,7 @@
         <v>10</v>
       </c>
       <c r="J93" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
     </row>
     <row r="94" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4531,7 +4534,7 @@
         <v>10</v>
       </c>
       <c r="J94" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
     </row>
     <row r="95" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4551,7 +4554,7 @@
         <v>10</v>
       </c>
       <c r="J95" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
     </row>
     <row r="96" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4571,7 +4574,7 @@
         <v>10</v>
       </c>
       <c r="J96" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
     </row>
     <row r="97" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4611,7 +4614,7 @@
         <v>10</v>
       </c>
       <c r="J98" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="99" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4631,7 +4634,7 @@
         <v>10</v>
       </c>
       <c r="J99" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
     </row>
     <row r="100" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4870,7 +4873,7 @@
         <v>10</v>
       </c>
       <c r="J111" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
     </row>
     <row r="112" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4890,7 +4893,7 @@
         <v>10</v>
       </c>
       <c r="J112" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
     </row>
     <row r="113" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4910,7 +4913,7 @@
         <v>10</v>
       </c>
       <c r="J113" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
     </row>
     <row r="114" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4930,7 +4933,7 @@
         <v>10</v>
       </c>
       <c r="J114" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
     </row>
     <row r="115" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4950,7 +4953,7 @@
         <v>10</v>
       </c>
       <c r="J115" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
     </row>
     <row r="116" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4970,7 +4973,7 @@
         <v>10</v>
       </c>
       <c r="J116" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
     </row>
     <row r="117" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4990,7 +4993,7 @@
         <v>10</v>
       </c>
       <c r="J117" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
     </row>
     <row r="118" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5010,7 +5013,7 @@
         <v>10</v>
       </c>
       <c r="J118" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
     </row>
     <row r="119" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5030,7 +5033,7 @@
         <v>10</v>
       </c>
       <c r="J119" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
     </row>
     <row r="120" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5050,7 +5053,7 @@
         <v>10</v>
       </c>
       <c r="J120" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
     </row>
     <row r="121" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5070,7 +5073,7 @@
         <v>10</v>
       </c>
       <c r="J121" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
     </row>
     <row r="122" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5090,7 +5093,7 @@
         <v>10</v>
       </c>
       <c r="J122" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
     </row>
     <row r="123" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5110,7 +5113,7 @@
         <v>10</v>
       </c>
       <c r="J123" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
     </row>
     <row r="124" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5130,7 +5133,7 @@
         <v>10</v>
       </c>
       <c r="J124" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
     </row>
     <row r="125" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5150,7 +5153,7 @@
         <v>10</v>
       </c>
       <c r="J125" t="s">
-        <v>630</v>
+        <v>627</v>
       </c>
     </row>
     <row r="126" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5170,7 +5173,7 @@
         <v>10</v>
       </c>
       <c r="J126" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
     </row>
     <row r="127" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5190,7 +5193,7 @@
         <v>10</v>
       </c>
       <c r="J127" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
     </row>
     <row r="128" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5210,7 +5213,7 @@
         <v>10</v>
       </c>
       <c r="J128" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
     </row>
     <row r="129" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5230,7 +5233,7 @@
         <v>10</v>
       </c>
       <c r="J129" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
     </row>
     <row r="130" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5250,7 +5253,7 @@
         <v>10</v>
       </c>
       <c r="J130" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
     </row>
     <row r="131" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5270,7 +5273,7 @@
         <v>10</v>
       </c>
       <c r="J131" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
     </row>
     <row r="132" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5290,7 +5293,7 @@
         <v>10</v>
       </c>
       <c r="J132" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
     </row>
     <row r="133" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5310,7 +5313,7 @@
         <v>10</v>
       </c>
       <c r="J133" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
     </row>
     <row r="134" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5330,7 +5333,7 @@
         <v>10</v>
       </c>
       <c r="J134" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
     </row>
     <row r="135" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5350,7 +5353,7 @@
         <v>10</v>
       </c>
       <c r="J135" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
     </row>
     <row r="136" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5370,7 +5373,7 @@
         <v>10</v>
       </c>
       <c r="J136" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
     </row>
     <row r="137" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5390,7 +5393,7 @@
         <v>10</v>
       </c>
       <c r="J137" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
     </row>
     <row r="138" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5450,7 +5453,7 @@
         <v>10</v>
       </c>
       <c r="J140" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
     </row>
     <row r="141" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5458,19 +5461,22 @@
         <v>27</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="C141" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D141" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E141" s="4" t="b">
         <v>1</v>
       </c>
       <c r="H141" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J141" t="s">
-        <v>651</v>
+      <c r="J141" s="5" t="s">
+        <v>700</v>
       </c>
     </row>
     <row r="142" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5478,22 +5484,19 @@
         <v>27</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="C142" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D142" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F142" s="4" t="s">
-        <v>403</v>
+        <v>1</v>
       </c>
       <c r="H142" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J142" t="s">
-        <v>402</v>
+        <v>648</v>
       </c>
     </row>
     <row r="143" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5501,19 +5504,22 @@
         <v>27</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>90</v>
+        <v>35</v>
       </c>
       <c r="C143" s="4" t="s">
-        <v>76</v>
+        <v>36</v>
       </c>
       <c r="D143" s="4" t="b">
         <v>0</v>
       </c>
+      <c r="F143" s="4" t="s">
+        <v>403</v>
+      </c>
       <c r="H143" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J143" t="s">
-        <v>653</v>
+        <v>402</v>
       </c>
     </row>
     <row r="144" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5521,10 +5527,10 @@
         <v>27</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C144" s="4" t="s">
-        <v>38</v>
+        <v>76</v>
       </c>
       <c r="D144" s="4" t="b">
         <v>0</v>
@@ -5533,7 +5539,7 @@
         <v>10</v>
       </c>
       <c r="J144" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
     </row>
     <row r="145" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5541,10 +5547,10 @@
         <v>27</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="C145" s="4" t="s">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="D145" s="4" t="b">
         <v>0</v>
@@ -5553,7 +5559,7 @@
         <v>10</v>
       </c>
       <c r="J145" t="s">
-        <v>654</v>
+        <v>649</v>
       </c>
     </row>
     <row r="146" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5561,10 +5567,10 @@
         <v>27</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C146" s="4" t="s">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="D146" s="4" t="b">
         <v>0</v>
@@ -5573,7 +5579,7 @@
         <v>10</v>
       </c>
       <c r="J146" t="s">
-        <v>655</v>
+        <v>651</v>
       </c>
     </row>
     <row r="147" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5581,10 +5587,10 @@
         <v>27</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C147" s="4" t="s">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="D147" s="4" t="b">
         <v>0</v>
@@ -5593,7 +5599,7 @@
         <v>10</v>
       </c>
       <c r="J147" t="s">
-        <v>656</v>
+        <v>652</v>
       </c>
     </row>
     <row r="148" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5601,10 +5607,10 @@
         <v>27</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C148" s="4" t="s">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="D148" s="4" t="b">
         <v>0</v>
@@ -5613,7 +5619,7 @@
         <v>10</v>
       </c>
       <c r="J148" t="s">
-        <v>658</v>
+        <v>653</v>
       </c>
     </row>
     <row r="149" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5621,10 +5627,10 @@
         <v>27</v>
       </c>
       <c r="B149" s="4" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C149" s="4" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D149" s="4" t="b">
         <v>0</v>
@@ -5633,7 +5639,7 @@
         <v>10</v>
       </c>
       <c r="J149" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
     </row>
     <row r="150" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5641,10 +5647,10 @@
         <v>27</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>179</v>
+        <v>82</v>
       </c>
       <c r="C150" s="4" t="s">
-        <v>180</v>
+        <v>32</v>
       </c>
       <c r="D150" s="4" t="b">
         <v>0</v>
@@ -5653,7 +5659,7 @@
         <v>10</v>
       </c>
       <c r="J150" t="s">
-        <v>367</v>
+        <v>654</v>
       </c>
     </row>
     <row r="151" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5661,7 +5667,7 @@
         <v>27</v>
       </c>
       <c r="B151" s="4" t="s">
-        <v>80</v>
+        <v>179</v>
       </c>
       <c r="C151" s="4" t="s">
         <v>180</v>
@@ -5673,7 +5679,7 @@
         <v>10</v>
       </c>
       <c r="J151" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="152" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5681,10 +5687,10 @@
         <v>27</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>181</v>
+        <v>80</v>
       </c>
       <c r="C152" s="4" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D152" s="4" t="b">
         <v>0</v>
@@ -5693,7 +5699,7 @@
         <v>10</v>
       </c>
       <c r="J152" t="s">
-        <v>379</v>
+        <v>368</v>
       </c>
     </row>
     <row r="153" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5701,7 +5707,7 @@
         <v>27</v>
       </c>
       <c r="B153" s="4" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C153" s="4" t="s">
         <v>182</v>
@@ -5713,7 +5719,7 @@
         <v>10</v>
       </c>
       <c r="J153" t="s">
-        <v>465</v>
+        <v>379</v>
       </c>
     </row>
     <row r="154" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5721,10 +5727,10 @@
         <v>27</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C154" s="4" t="s">
-        <v>38</v>
+        <v>182</v>
       </c>
       <c r="D154" s="4" t="b">
         <v>0</v>
@@ -5733,7 +5739,7 @@
         <v>10</v>
       </c>
       <c r="J154" t="s">
-        <v>615</v>
+        <v>464</v>
       </c>
     </row>
     <row r="155" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5741,10 +5747,10 @@
         <v>27</v>
       </c>
       <c r="B155" s="4" t="s">
-        <v>149</v>
+        <v>184</v>
       </c>
       <c r="C155" s="4" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="D155" s="4" t="b">
         <v>0</v>
@@ -5753,7 +5759,7 @@
         <v>10</v>
       </c>
       <c r="J155" t="s">
-        <v>619</v>
+        <v>612</v>
       </c>
     </row>
     <row r="156" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5761,10 +5767,10 @@
         <v>27</v>
       </c>
       <c r="B156" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C156" s="4" t="s">
-        <v>185</v>
+        <v>76</v>
       </c>
       <c r="D156" s="4" t="b">
         <v>0</v>
@@ -5773,7 +5779,7 @@
         <v>10</v>
       </c>
       <c r="J156" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="157" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5781,10 +5787,10 @@
         <v>27</v>
       </c>
       <c r="B157" s="4" t="s">
-        <v>186</v>
+        <v>150</v>
       </c>
       <c r="C157" s="4" t="s">
-        <v>76</v>
+        <v>185</v>
       </c>
       <c r="D157" s="4" t="b">
         <v>0</v>
@@ -5793,7 +5799,7 @@
         <v>10</v>
       </c>
       <c r="J157" t="s">
-        <v>638</v>
+        <v>614</v>
       </c>
     </row>
     <row r="158" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5801,7 +5807,7 @@
         <v>27</v>
       </c>
       <c r="B158" s="4" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C158" s="4" t="s">
         <v>76</v>
@@ -5813,7 +5819,7 @@
         <v>10</v>
       </c>
       <c r="J158" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
     </row>
     <row r="159" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5821,10 +5827,10 @@
         <v>27</v>
       </c>
       <c r="B159" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C159" s="4" t="s">
-        <v>38</v>
+        <v>76</v>
       </c>
       <c r="D159" s="4" t="b">
         <v>0</v>
@@ -5833,7 +5839,7 @@
         <v>10</v>
       </c>
       <c r="J159" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
     </row>
     <row r="160" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5841,10 +5847,10 @@
         <v>27</v>
       </c>
       <c r="B160" s="4" t="s">
-        <v>75</v>
+        <v>188</v>
       </c>
       <c r="C160" s="4" t="s">
-        <v>189</v>
+        <v>38</v>
       </c>
       <c r="D160" s="4" t="b">
         <v>0</v>
@@ -5853,7 +5859,7 @@
         <v>10</v>
       </c>
       <c r="J160" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
     </row>
     <row r="161" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5861,10 +5867,10 @@
         <v>27</v>
       </c>
       <c r="B161" s="4" t="s">
-        <v>190</v>
+        <v>75</v>
       </c>
       <c r="C161" s="4" t="s">
-        <v>38</v>
+        <v>189</v>
       </c>
       <c r="D161" s="4" t="b">
         <v>0</v>
@@ -5873,7 +5879,7 @@
         <v>10</v>
       </c>
       <c r="J161" t="s">
-        <v>633</v>
+        <v>629</v>
       </c>
     </row>
     <row r="162" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5881,10 +5887,10 @@
         <v>27</v>
       </c>
       <c r="B162" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C162" s="4" t="s">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="D162" s="4" t="b">
         <v>0</v>
@@ -5893,7 +5899,7 @@
         <v>10</v>
       </c>
       <c r="J162" t="s">
-        <v>456</v>
+        <v>630</v>
       </c>
     </row>
     <row r="163" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5901,10 +5907,10 @@
         <v>27</v>
       </c>
       <c r="B163" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C163" s="4" t="s">
-        <v>45</v>
+        <v>84</v>
       </c>
       <c r="D163" s="4" t="b">
         <v>0</v>
@@ -5913,7 +5919,7 @@
         <v>10</v>
       </c>
       <c r="J163" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
     </row>
     <row r="164" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5921,10 +5927,10 @@
         <v>27</v>
       </c>
       <c r="B164" s="4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C164" s="4" t="s">
-        <v>84</v>
+        <v>45</v>
       </c>
       <c r="D164" s="4" t="b">
         <v>0</v>
@@ -5933,7 +5939,7 @@
         <v>10</v>
       </c>
       <c r="J164" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
     </row>
     <row r="165" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5941,10 +5947,10 @@
         <v>27</v>
       </c>
       <c r="B165" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C165" s="4" t="s">
-        <v>195</v>
+        <v>84</v>
       </c>
       <c r="D165" s="4" t="b">
         <v>0</v>
@@ -5953,7 +5959,7 @@
         <v>10</v>
       </c>
       <c r="J165" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
     </row>
     <row r="166" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5961,10 +5967,10 @@
         <v>27</v>
       </c>
       <c r="B166" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C166" s="4" t="s">
-        <v>84</v>
+        <v>195</v>
       </c>
       <c r="D166" s="4" t="b">
         <v>0</v>
@@ -5973,7 +5979,7 @@
         <v>10</v>
       </c>
       <c r="J166" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
     </row>
     <row r="167" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5981,10 +5987,10 @@
         <v>27</v>
       </c>
       <c r="B167" s="4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C167" s="4" t="s">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="D167" s="4" t="b">
         <v>0</v>
@@ -5993,7 +5999,7 @@
         <v>10</v>
       </c>
       <c r="J167" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="168" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6001,22 +6007,19 @@
         <v>27</v>
       </c>
       <c r="B168" s="4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C168" s="4" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D168" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="E168" s="4" t="b">
-        <v>1</v>
-      </c>
       <c r="H168" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J168" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
     </row>
     <row r="169" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6024,7 +6027,7 @@
         <v>27</v>
       </c>
       <c r="B169" s="4" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C169" s="4" t="s">
         <v>32</v>
@@ -6032,11 +6035,14 @@
       <c r="D169" s="4" t="b">
         <v>0</v>
       </c>
+      <c r="E169" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="H169" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J169" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
     </row>
     <row r="170" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6044,7 +6050,7 @@
         <v>27</v>
       </c>
       <c r="B170" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C170" s="4" t="s">
         <v>32</v>
@@ -6056,7 +6062,7 @@
         <v>10</v>
       </c>
       <c r="J170" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
     <row r="171" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6064,10 +6070,10 @@
         <v>27</v>
       </c>
       <c r="B171" s="4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C171" s="4" t="s">
-        <v>84</v>
+        <v>32</v>
       </c>
       <c r="D171" s="4" t="b">
         <v>0</v>
@@ -6076,7 +6082,7 @@
         <v>10</v>
       </c>
       <c r="J171" t="s">
-        <v>634</v>
+        <v>463</v>
       </c>
     </row>
     <row r="172" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6084,10 +6090,10 @@
         <v>27</v>
       </c>
       <c r="B172" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C172" s="4" t="s">
-        <v>195</v>
+        <v>84</v>
       </c>
       <c r="D172" s="4" t="b">
         <v>0</v>
@@ -6096,7 +6102,7 @@
         <v>10</v>
       </c>
       <c r="J172" t="s">
-        <v>635</v>
+        <v>631</v>
       </c>
     </row>
     <row r="173" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6104,10 +6110,10 @@
         <v>27</v>
       </c>
       <c r="B173" s="4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C173" s="4" t="s">
-        <v>84</v>
+        <v>195</v>
       </c>
       <c r="D173" s="4" t="b">
         <v>0</v>
@@ -6116,7 +6122,7 @@
         <v>10</v>
       </c>
       <c r="J173" t="s">
-        <v>659</v>
+        <v>632</v>
       </c>
     </row>
     <row r="174" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6124,10 +6130,10 @@
         <v>27</v>
       </c>
       <c r="B174" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C174" s="4" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="D174" s="4" t="b">
         <v>0</v>
@@ -6136,7 +6142,7 @@
         <v>10</v>
       </c>
       <c r="J174" t="s">
-        <v>660</v>
+        <v>656</v>
       </c>
     </row>
     <row r="175" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6144,10 +6150,10 @@
         <v>27</v>
       </c>
       <c r="B175" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C175" s="4" t="s">
-        <v>45</v>
+        <v>76</v>
       </c>
       <c r="D175" s="4" t="b">
         <v>0</v>
@@ -6156,7 +6162,7 @@
         <v>10</v>
       </c>
       <c r="J175" t="s">
-        <v>661</v>
+        <v>657</v>
       </c>
     </row>
     <row r="176" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6164,7 +6170,7 @@
         <v>27</v>
       </c>
       <c r="B176" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C176" s="4" t="s">
         <v>45</v>
@@ -6176,7 +6182,7 @@
         <v>10</v>
       </c>
       <c r="J176" t="s">
-        <v>662</v>
+        <v>658</v>
       </c>
     </row>
     <row r="177" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6184,7 +6190,7 @@
         <v>27</v>
       </c>
       <c r="B177" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C177" s="4" t="s">
         <v>45</v>
@@ -6196,7 +6202,7 @@
         <v>10</v>
       </c>
       <c r="J177" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
     </row>
     <row r="178" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6204,10 +6210,10 @@
         <v>27</v>
       </c>
       <c r="B178" s="4" t="s">
-        <v>12</v>
+        <v>207</v>
       </c>
       <c r="C178" s="4" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="D178" s="4" t="b">
         <v>0</v>
@@ -6216,7 +6222,7 @@
         <v>10</v>
       </c>
       <c r="J178" t="s">
-        <v>663</v>
+        <v>659</v>
       </c>
     </row>
     <row r="179" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6224,10 +6230,10 @@
         <v>27</v>
       </c>
       <c r="B179" s="4" t="s">
-        <v>208</v>
+        <v>12</v>
       </c>
       <c r="C179" s="4" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="D179" s="4" t="b">
         <v>0</v>
@@ -6236,7 +6242,7 @@
         <v>10</v>
       </c>
       <c r="J179" t="s">
-        <v>664</v>
+        <v>660</v>
       </c>
     </row>
     <row r="180" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6244,22 +6250,19 @@
         <v>27</v>
       </c>
       <c r="B180" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C180" s="4" t="s">
-        <v>210</v>
+        <v>52</v>
       </c>
       <c r="D180" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="G180" s="4" t="s">
-        <v>17</v>
-      </c>
       <c r="H180" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J180" t="s">
-        <v>665</v>
+        <v>661</v>
       </c>
     </row>
     <row r="181" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6267,7 +6270,7 @@
         <v>27</v>
       </c>
       <c r="B181" s="4" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C181" s="4" t="s">
         <v>210</v>
@@ -6282,7 +6285,7 @@
         <v>10</v>
       </c>
       <c r="J181" t="s">
-        <v>666</v>
+        <v>662</v>
       </c>
     </row>
     <row r="182" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6290,7 +6293,7 @@
         <v>27</v>
       </c>
       <c r="B182" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C182" s="4" t="s">
         <v>210</v>
@@ -6305,7 +6308,7 @@
         <v>10</v>
       </c>
       <c r="J182" t="s">
-        <v>667</v>
+        <v>663</v>
       </c>
     </row>
     <row r="183" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6313,7 +6316,7 @@
         <v>27</v>
       </c>
       <c r="B183" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C183" s="4" t="s">
         <v>210</v>
@@ -6328,7 +6331,7 @@
         <v>10</v>
       </c>
       <c r="J183" t="s">
-        <v>668</v>
+        <v>664</v>
       </c>
     </row>
     <row r="184" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6336,7 +6339,7 @@
         <v>27</v>
       </c>
       <c r="B184" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C184" s="4" t="s">
         <v>210</v>
@@ -6351,7 +6354,7 @@
         <v>10</v>
       </c>
       <c r="J184" t="s">
-        <v>669</v>
+        <v>665</v>
       </c>
     </row>
     <row r="185" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6359,19 +6362,22 @@
         <v>27</v>
       </c>
       <c r="B185" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C185" s="4" t="s">
-        <v>36</v>
+        <v>210</v>
       </c>
       <c r="D185" s="4" t="b">
         <v>0</v>
       </c>
+      <c r="G185" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="H185" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J185" t="s">
-        <v>670</v>
+        <v>666</v>
       </c>
     </row>
     <row r="186" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6379,10 +6385,10 @@
         <v>27</v>
       </c>
       <c r="B186" s="4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C186" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D186" s="4" t="b">
         <v>0</v>
@@ -6391,7 +6397,7 @@
         <v>10</v>
       </c>
       <c r="J186" t="s">
-        <v>671</v>
+        <v>667</v>
       </c>
     </row>
     <row r="187" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6399,7 +6405,7 @@
         <v>27</v>
       </c>
       <c r="B187" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C187" s="4" t="s">
         <v>38</v>
@@ -6411,7 +6417,7 @@
         <v>10</v>
       </c>
       <c r="J187" t="s">
-        <v>672</v>
+        <v>668</v>
       </c>
     </row>
     <row r="188" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6419,7 +6425,7 @@
         <v>27</v>
       </c>
       <c r="B188" s="4" t="s">
-        <v>96</v>
+        <v>217</v>
       </c>
       <c r="C188" s="4" t="s">
         <v>38</v>
@@ -6431,7 +6437,7 @@
         <v>10</v>
       </c>
       <c r="J188" t="s">
-        <v>382</v>
+        <v>669</v>
       </c>
     </row>
     <row r="189" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6439,7 +6445,7 @@
         <v>27</v>
       </c>
       <c r="B189" s="4" t="s">
-        <v>218</v>
+        <v>96</v>
       </c>
       <c r="C189" s="4" t="s">
         <v>38</v>
@@ -6451,7 +6457,7 @@
         <v>10</v>
       </c>
       <c r="J189" t="s">
-        <v>465</v>
+        <v>382</v>
       </c>
     </row>
     <row r="190" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6459,7 +6465,7 @@
         <v>27</v>
       </c>
       <c r="B190" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C190" s="4" t="s">
         <v>38</v>
@@ -6471,7 +6477,7 @@
         <v>10</v>
       </c>
       <c r="J190" t="s">
-        <v>673</v>
+        <v>464</v>
       </c>
     </row>
     <row r="191" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6479,10 +6485,10 @@
         <v>27</v>
       </c>
       <c r="B191" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C191" s="4" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="D191" s="4" t="b">
         <v>0</v>
@@ -6491,7 +6497,7 @@
         <v>10</v>
       </c>
       <c r="J191" t="s">
-        <v>674</v>
+        <v>670</v>
       </c>
     </row>
     <row r="192" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6499,7 +6505,7 @@
         <v>27</v>
       </c>
       <c r="B192" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C192" s="4" t="s">
         <v>52</v>
@@ -6511,7 +6517,7 @@
         <v>10</v>
       </c>
       <c r="J192" t="s">
-        <v>675</v>
+        <v>671</v>
       </c>
     </row>
     <row r="193" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6519,10 +6525,10 @@
         <v>27</v>
       </c>
       <c r="B193" s="4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C193" s="4" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="D193" s="4" t="b">
         <v>0</v>
@@ -6531,7 +6537,7 @@
         <v>10</v>
       </c>
       <c r="J193" t="s">
-        <v>676</v>
+        <v>672</v>
       </c>
     </row>
     <row r="194" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6539,7 +6545,7 @@
         <v>27</v>
       </c>
       <c r="B194" s="4" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C194" s="4" t="s">
         <v>38</v>
@@ -6551,7 +6557,7 @@
         <v>10</v>
       </c>
       <c r="J194" t="s">
-        <v>677</v>
+        <v>673</v>
       </c>
     </row>
     <row r="195" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6559,10 +6565,10 @@
         <v>27</v>
       </c>
       <c r="B195" s="4" t="s">
-        <v>160</v>
+        <v>223</v>
       </c>
       <c r="C195" s="4" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="D195" s="4" t="b">
         <v>0</v>
@@ -6571,7 +6577,7 @@
         <v>10</v>
       </c>
       <c r="J195" t="s">
-        <v>629</v>
+        <v>674</v>
       </c>
     </row>
     <row r="196" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6579,10 +6585,10 @@
         <v>27</v>
       </c>
       <c r="B196" s="4" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="C196" s="4" t="s">
-        <v>84</v>
+        <v>45</v>
       </c>
       <c r="D196" s="4" t="b">
         <v>0</v>
@@ -6591,7 +6597,7 @@
         <v>10</v>
       </c>
       <c r="J196" t="s">
-        <v>678</v>
+        <v>626</v>
       </c>
     </row>
     <row r="197" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6599,10 +6605,10 @@
         <v>27</v>
       </c>
       <c r="B197" s="4" t="s">
-        <v>224</v>
+        <v>153</v>
       </c>
       <c r="C197" s="4" t="s">
-        <v>45</v>
+        <v>84</v>
       </c>
       <c r="D197" s="4" t="b">
         <v>0</v>
@@ -6611,7 +6617,7 @@
         <v>10</v>
       </c>
       <c r="J197" t="s">
-        <v>679</v>
+        <v>675</v>
       </c>
     </row>
     <row r="198" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6619,7 +6625,7 @@
         <v>27</v>
       </c>
       <c r="B198" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C198" s="4" t="s">
         <v>45</v>
@@ -6631,7 +6637,7 @@
         <v>10</v>
       </c>
       <c r="J198" t="s">
-        <v>680</v>
+        <v>676</v>
       </c>
     </row>
     <row r="199" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6639,7 +6645,7 @@
         <v>27</v>
       </c>
       <c r="B199" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C199" s="4" t="s">
         <v>45</v>
@@ -6651,7 +6657,7 @@
         <v>10</v>
       </c>
       <c r="J199" t="s">
-        <v>681</v>
+        <v>677</v>
       </c>
     </row>
     <row r="200" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6659,7 +6665,7 @@
         <v>27</v>
       </c>
       <c r="B200" s="4" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C200" s="4" t="s">
         <v>45</v>
@@ -6671,7 +6677,7 @@
         <v>10</v>
       </c>
       <c r="J200" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
     </row>
     <row r="201" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6679,7 +6685,7 @@
         <v>27</v>
       </c>
       <c r="B201" s="4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C201" s="4" t="s">
         <v>45</v>
@@ -6691,7 +6697,7 @@
         <v>10</v>
       </c>
       <c r="J201" t="s">
-        <v>683</v>
+        <v>679</v>
       </c>
     </row>
     <row r="202" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6699,7 +6705,7 @@
         <v>27</v>
       </c>
       <c r="B202" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C202" s="4" t="s">
         <v>45</v>
@@ -6711,7 +6717,7 @@
         <v>10</v>
       </c>
       <c r="J202" t="s">
-        <v>684</v>
+        <v>680</v>
       </c>
     </row>
     <row r="203" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6719,22 +6725,19 @@
         <v>27</v>
       </c>
       <c r="B203" s="4" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C203" s="4" t="s">
-        <v>210</v>
+        <v>45</v>
       </c>
       <c r="D203" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="G203" s="4" t="s">
-        <v>17</v>
-      </c>
       <c r="H203" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J203" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
     </row>
     <row r="204" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6742,7 +6745,7 @@
         <v>27</v>
       </c>
       <c r="B204" s="4" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C204" s="4" t="s">
         <v>210</v>
@@ -6757,7 +6760,7 @@
         <v>10</v>
       </c>
       <c r="J204" t="s">
-        <v>686</v>
+        <v>682</v>
       </c>
     </row>
     <row r="205" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6765,7 +6768,7 @@
         <v>27</v>
       </c>
       <c r="B205" s="4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C205" s="4" t="s">
         <v>210</v>
@@ -6780,7 +6783,7 @@
         <v>10</v>
       </c>
       <c r="J205" t="s">
-        <v>687</v>
+        <v>683</v>
       </c>
     </row>
     <row r="206" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6788,7 +6791,7 @@
         <v>27</v>
       </c>
       <c r="B206" s="4" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C206" s="4" t="s">
         <v>210</v>
@@ -6803,7 +6806,7 @@
         <v>10</v>
       </c>
       <c r="J206" t="s">
-        <v>688</v>
+        <v>684</v>
       </c>
     </row>
     <row r="207" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6811,7 +6814,7 @@
         <v>27</v>
       </c>
       <c r="B207" s="4" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C207" s="4" t="s">
         <v>210</v>
@@ -6826,7 +6829,7 @@
         <v>10</v>
       </c>
       <c r="J207" t="s">
-        <v>466</v>
+        <v>685</v>
       </c>
     </row>
     <row r="208" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6834,7 +6837,7 @@
         <v>27</v>
       </c>
       <c r="B208" s="4" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C208" s="4" t="s">
         <v>210</v>
@@ -6849,7 +6852,7 @@
         <v>10</v>
       </c>
       <c r="J208" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="209" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6857,7 +6860,7 @@
         <v>27</v>
       </c>
       <c r="B209" s="4" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C209" s="4" t="s">
         <v>210</v>
@@ -6871,8 +6874,8 @@
       <c r="H209" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J209" s="5" t="s">
-        <v>468</v>
+      <c r="J209" t="s">
+        <v>466</v>
       </c>
     </row>
     <row r="210" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6880,7 +6883,7 @@
         <v>27</v>
       </c>
       <c r="B210" s="4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C210" s="4" t="s">
         <v>210</v>
@@ -6895,7 +6898,7 @@
         <v>10</v>
       </c>
       <c r="J210" s="5" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
     </row>
     <row r="211" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6903,7 +6906,7 @@
         <v>27</v>
       </c>
       <c r="B211" s="4" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C211" s="4" t="s">
         <v>210</v>
@@ -6918,7 +6921,7 @@
         <v>10</v>
       </c>
       <c r="J211" s="5" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
     </row>
     <row r="212" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6926,7 +6929,7 @@
         <v>27</v>
       </c>
       <c r="B212" s="4" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C212" s="4" t="s">
         <v>210</v>
@@ -6941,7 +6944,7 @@
         <v>10</v>
       </c>
       <c r="J212" s="5" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
     </row>
     <row r="213" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6949,19 +6952,22 @@
         <v>27</v>
       </c>
       <c r="B213" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C213" s="4" t="s">
-        <v>38</v>
+        <v>210</v>
       </c>
       <c r="D213" s="4" t="b">
         <v>0</v>
       </c>
+      <c r="G213" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="H213" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J213" s="5" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
     </row>
     <row r="214" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6969,7 +6975,7 @@
         <v>27</v>
       </c>
       <c r="B214" s="4" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C214" s="4" t="s">
         <v>38</v>
@@ -6981,7 +6987,7 @@
         <v>10</v>
       </c>
       <c r="J214" s="5" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="215" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6989,7 +6995,7 @@
         <v>27</v>
       </c>
       <c r="B215" s="4" t="s">
-        <v>62</v>
+        <v>241</v>
       </c>
       <c r="C215" s="4" t="s">
         <v>38</v>
@@ -7001,7 +7007,7 @@
         <v>10</v>
       </c>
       <c r="J215" s="5" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="216" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7009,22 +7015,19 @@
         <v>27</v>
       </c>
       <c r="B216" s="4" t="s">
-        <v>242</v>
+        <v>62</v>
       </c>
       <c r="C216" s="4" t="s">
-        <v>243</v>
+        <v>38</v>
       </c>
       <c r="D216" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="G216" s="4" t="s">
-        <v>17</v>
-      </c>
       <c r="H216" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J216" s="5" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
     </row>
     <row r="217" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7032,7 +7035,7 @@
         <v>27</v>
       </c>
       <c r="B217" s="4" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C217" s="4" t="s">
         <v>243</v>
@@ -7047,7 +7050,7 @@
         <v>10</v>
       </c>
       <c r="J217" s="5" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="218" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7055,7 +7058,7 @@
         <v>27</v>
       </c>
       <c r="B218" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C218" s="4" t="s">
         <v>243</v>
@@ -7070,7 +7073,7 @@
         <v>10</v>
       </c>
       <c r="J218" s="5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
     </row>
     <row r="219" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7078,19 +7081,22 @@
         <v>27</v>
       </c>
       <c r="B219" s="4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C219" s="4" t="s">
-        <v>76</v>
+        <v>243</v>
       </c>
       <c r="D219" s="4" t="b">
         <v>0</v>
       </c>
+      <c r="G219" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="H219" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J219" s="5" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
     </row>
     <row r="220" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7098,10 +7104,10 @@
         <v>27</v>
       </c>
       <c r="B220" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C220" s="4" t="s">
-        <v>38</v>
+        <v>76</v>
       </c>
       <c r="D220" s="4" t="b">
         <v>0</v>
@@ -7110,7 +7116,7 @@
         <v>10</v>
       </c>
       <c r="J220" s="5" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="221" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7118,10 +7124,10 @@
         <v>27</v>
       </c>
       <c r="B221" s="4" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C221" s="4" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="D221" s="4" t="b">
         <v>0</v>
@@ -7130,7 +7136,7 @@
         <v>10</v>
       </c>
       <c r="J221" s="5" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="222" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7138,10 +7144,10 @@
         <v>27</v>
       </c>
       <c r="B222" s="4" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C222" s="4" t="s">
-        <v>195</v>
+        <v>52</v>
       </c>
       <c r="D222" s="4" t="b">
         <v>0</v>
@@ -7150,7 +7156,7 @@
         <v>10</v>
       </c>
       <c r="J222" s="5" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
     </row>
     <row r="223" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7158,10 +7164,10 @@
         <v>27</v>
       </c>
       <c r="B223" s="4" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C223" s="4" t="s">
-        <v>38</v>
+        <v>195</v>
       </c>
       <c r="D223" s="4" t="b">
         <v>0</v>
@@ -7170,7 +7176,7 @@
         <v>10</v>
       </c>
       <c r="J223" s="5" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="224" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7178,10 +7184,10 @@
         <v>27</v>
       </c>
       <c r="B224" s="4" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C224" s="4" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="D224" s="4" t="b">
         <v>0</v>
@@ -7190,7 +7196,7 @@
         <v>10</v>
       </c>
       <c r="J224" s="5" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
     </row>
     <row r="225" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7198,7 +7204,7 @@
         <v>27</v>
       </c>
       <c r="B225" s="4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C225" s="4" t="s">
         <v>45</v>
@@ -7210,7 +7216,7 @@
         <v>10</v>
       </c>
       <c r="J225" s="5" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
     </row>
     <row r="226" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7218,7 +7224,7 @@
         <v>27</v>
       </c>
       <c r="B226" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C226" s="4" t="s">
         <v>45</v>
@@ -7230,7 +7236,7 @@
         <v>10</v>
       </c>
       <c r="J226" s="5" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="227" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7238,10 +7244,10 @@
         <v>27</v>
       </c>
       <c r="B227" s="4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C227" s="4" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="D227" s="4" t="b">
         <v>0</v>
@@ -7250,7 +7256,7 @@
         <v>10</v>
       </c>
       <c r="J227" s="5" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="228" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7258,7 +7264,7 @@
         <v>27</v>
       </c>
       <c r="B228" s="4" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C228" s="4" t="s">
         <v>38</v>
@@ -7270,7 +7276,7 @@
         <v>10</v>
       </c>
       <c r="J228" s="5" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="229" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7278,10 +7284,10 @@
         <v>27</v>
       </c>
       <c r="B229" s="4" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C229" s="4" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="D229" s="4" t="b">
         <v>0</v>
@@ -7290,7 +7296,7 @@
         <v>10</v>
       </c>
       <c r="J229" s="5" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
     </row>
     <row r="230" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7298,22 +7304,19 @@
         <v>27</v>
       </c>
       <c r="B230" s="4" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C230" s="4" t="s">
-        <v>210</v>
+        <v>52</v>
       </c>
       <c r="D230" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="G230" s="4" t="s">
-        <v>17</v>
-      </c>
       <c r="H230" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J230" s="5" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
     </row>
     <row r="231" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7321,7 +7324,7 @@
         <v>27</v>
       </c>
       <c r="B231" s="4" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C231" s="4" t="s">
         <v>210</v>
@@ -7336,7 +7339,7 @@
         <v>10</v>
       </c>
       <c r="J231" s="5" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
     </row>
     <row r="232" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7344,7 +7347,7 @@
         <v>27</v>
       </c>
       <c r="B232" s="4" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C232" s="4" t="s">
         <v>210</v>
@@ -7359,7 +7362,7 @@
         <v>10</v>
       </c>
       <c r="J232" s="5" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
     </row>
     <row r="233" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7367,7 +7370,7 @@
         <v>27</v>
       </c>
       <c r="B233" s="4" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C233" s="4" t="s">
         <v>210</v>
@@ -7382,7 +7385,7 @@
         <v>10</v>
       </c>
       <c r="J233" s="5" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
     </row>
     <row r="234" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7390,7 +7393,7 @@
         <v>27</v>
       </c>
       <c r="B234" s="4" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C234" s="4" t="s">
         <v>210</v>
@@ -7405,7 +7408,7 @@
         <v>10</v>
       </c>
       <c r="J234" s="5" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
     </row>
     <row r="235" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7413,7 +7416,7 @@
         <v>27</v>
       </c>
       <c r="B235" s="4" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C235" s="4" t="s">
         <v>210</v>
@@ -7428,7 +7431,7 @@
         <v>10</v>
       </c>
       <c r="J235" s="5" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
     </row>
     <row r="236" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7436,7 +7439,7 @@
         <v>27</v>
       </c>
       <c r="B236" s="4" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C236" s="4" t="s">
         <v>210</v>
@@ -7451,7 +7454,7 @@
         <v>10</v>
       </c>
       <c r="J236" s="5" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
     </row>
     <row r="237" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7459,7 +7462,7 @@
         <v>27</v>
       </c>
       <c r="B237" s="4" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C237" s="4" t="s">
         <v>210</v>
@@ -7474,7 +7477,7 @@
         <v>10</v>
       </c>
       <c r="J237" s="5" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
     </row>
     <row r="238" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7482,19 +7485,22 @@
         <v>27</v>
       </c>
       <c r="B238" s="4" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C238" s="4" t="s">
-        <v>32</v>
+        <v>210</v>
       </c>
       <c r="D238" s="4" t="b">
         <v>0</v>
       </c>
+      <c r="G238" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="H238" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J238" s="5" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
     </row>
     <row r="239" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7502,22 +7508,19 @@
         <v>27</v>
       </c>
       <c r="B239" s="4" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C239" s="4" t="s">
-        <v>267</v>
+        <v>32</v>
       </c>
       <c r="D239" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="G239" s="4" t="s">
-        <v>17</v>
-      </c>
       <c r="H239" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J239" s="5" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
     </row>
     <row r="240" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7525,42 +7528,42 @@
         <v>27</v>
       </c>
       <c r="B240" s="4" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C240" s="4" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D240" s="4" t="b">
         <v>0</v>
       </c>
+      <c r="G240" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="H240" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J240" s="5" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
     </row>
     <row r="241" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A241" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B241" s="4" t="s">
-        <v>31</v>
+        <v>268</v>
       </c>
       <c r="C241" s="4" t="s">
-        <v>32</v>
+        <v>269</v>
       </c>
       <c r="D241" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="E241" s="4" t="b">
-        <v>1</v>
-      </c>
       <c r="H241" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J241" s="5" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
     </row>
     <row r="242" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7568,19 +7571,22 @@
         <v>29</v>
       </c>
       <c r="B242" s="4" t="s">
-        <v>78</v>
+        <v>31</v>
       </c>
       <c r="C242" s="4" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="D242" s="4" t="b">
         <v>0</v>
       </c>
+      <c r="E242" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="H242" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J242" s="5" t="s">
-        <v>501</v>
+        <v>701</v>
       </c>
     </row>
     <row r="243" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7588,19 +7594,19 @@
         <v>29</v>
       </c>
       <c r="B243" s="4" t="s">
-        <v>11</v>
+        <v>78</v>
       </c>
       <c r="C243" s="4" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="D243" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H243" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J243" s="5" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
     </row>
     <row r="244" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7608,22 +7614,19 @@
         <v>29</v>
       </c>
       <c r="B244" s="4" t="s">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="C244" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D244" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F244" s="4" t="s">
-        <v>403</v>
+        <v>1</v>
       </c>
       <c r="H244" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J244" s="5" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
     </row>
     <row r="245" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7631,7 +7634,7 @@
         <v>29</v>
       </c>
       <c r="B245" s="4" t="s">
-        <v>270</v>
+        <v>35</v>
       </c>
       <c r="C245" s="4" t="s">
         <v>36</v>
@@ -7639,11 +7642,14 @@
       <c r="D245" s="4" t="b">
         <v>0</v>
       </c>
+      <c r="F245" s="4" t="s">
+        <v>403</v>
+      </c>
       <c r="H245" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J245" s="5" t="s">
-        <v>689</v>
+        <v>501</v>
       </c>
     </row>
     <row r="246" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7651,10 +7657,10 @@
         <v>29</v>
       </c>
       <c r="B246" s="4" t="s">
-        <v>90</v>
+        <v>270</v>
       </c>
       <c r="C246" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D246" s="4" t="b">
         <v>0</v>
@@ -7663,7 +7669,7 @@
         <v>10</v>
       </c>
       <c r="J246" s="5" t="s">
-        <v>504</v>
+        <v>686</v>
       </c>
     </row>
     <row r="247" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7671,7 +7677,7 @@
         <v>29</v>
       </c>
       <c r="B247" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C247" s="4" t="s">
         <v>38</v>
@@ -7683,7 +7689,7 @@
         <v>10</v>
       </c>
       <c r="J247" s="5" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
     </row>
     <row r="248" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7691,10 +7697,10 @@
         <v>29</v>
       </c>
       <c r="B248" s="4" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="C248" s="4" t="s">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="D248" s="4" t="b">
         <v>0</v>
@@ -7703,7 +7709,7 @@
         <v>10</v>
       </c>
       <c r="J248" s="5" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
     </row>
     <row r="249" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7711,10 +7717,10 @@
         <v>29</v>
       </c>
       <c r="B249" s="4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C249" s="4" t="s">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="D249" s="4" t="b">
         <v>0</v>
@@ -7723,7 +7729,7 @@
         <v>10</v>
       </c>
       <c r="J249" s="5" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
     </row>
     <row r="250" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7731,10 +7737,10 @@
         <v>29</v>
       </c>
       <c r="B250" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C250" s="4" t="s">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="D250" s="4" t="b">
         <v>0</v>
@@ -7743,7 +7749,7 @@
         <v>10</v>
       </c>
       <c r="J250" s="5" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
     </row>
     <row r="251" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7751,10 +7757,10 @@
         <v>29</v>
       </c>
       <c r="B251" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C251" s="4" t="s">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="D251" s="4" t="b">
         <v>0</v>
@@ -7763,7 +7769,7 @@
         <v>10</v>
       </c>
       <c r="J251" s="5" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
     </row>
     <row r="252" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7771,10 +7777,10 @@
         <v>29</v>
       </c>
       <c r="B252" s="4" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C252" s="4" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D252" s="4" t="b">
         <v>0</v>
@@ -7783,7 +7789,7 @@
         <v>10</v>
       </c>
       <c r="J252" s="5" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
     </row>
     <row r="253" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7791,10 +7797,10 @@
         <v>29</v>
       </c>
       <c r="B253" s="4" t="s">
-        <v>179</v>
+        <v>82</v>
       </c>
       <c r="C253" s="4" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D253" s="4" t="b">
         <v>0</v>
@@ -7803,7 +7809,7 @@
         <v>10</v>
       </c>
       <c r="J253" s="5" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
     </row>
     <row r="254" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7811,7 +7817,7 @@
         <v>29</v>
       </c>
       <c r="B254" s="4" t="s">
-        <v>80</v>
+        <v>179</v>
       </c>
       <c r="C254" s="4" t="s">
         <v>38</v>
@@ -7823,7 +7829,7 @@
         <v>10</v>
       </c>
       <c r="J254" s="5" t="s">
-        <v>690</v>
+        <v>509</v>
       </c>
     </row>
     <row r="255" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7831,10 +7837,10 @@
         <v>29</v>
       </c>
       <c r="B255" s="4" t="s">
-        <v>181</v>
+        <v>80</v>
       </c>
       <c r="C255" s="4" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="D255" s="4" t="b">
         <v>0</v>
@@ -7843,7 +7849,7 @@
         <v>10</v>
       </c>
       <c r="J255" s="5" t="s">
-        <v>691</v>
+        <v>687</v>
       </c>
     </row>
     <row r="256" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7851,10 +7857,10 @@
         <v>29</v>
       </c>
       <c r="B256" s="4" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C256" s="4" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="D256" s="4" t="b">
         <v>0</v>
@@ -7863,7 +7869,7 @@
         <v>10</v>
       </c>
       <c r="J256" s="5" t="s">
-        <v>512</v>
+        <v>688</v>
       </c>
     </row>
     <row r="257" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7871,7 +7877,7 @@
         <v>29</v>
       </c>
       <c r="B257" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C257" s="4" t="s">
         <v>38</v>
@@ -7883,7 +7889,7 @@
         <v>10</v>
       </c>
       <c r="J257" s="5" t="s">
-        <v>692</v>
+        <v>510</v>
       </c>
     </row>
     <row r="258" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7891,7 +7897,7 @@
         <v>29</v>
       </c>
       <c r="B258" s="4" t="s">
-        <v>149</v>
+        <v>184</v>
       </c>
       <c r="C258" s="4" t="s">
         <v>38</v>
@@ -7903,7 +7909,7 @@
         <v>10</v>
       </c>
       <c r="J258" s="5" t="s">
-        <v>693</v>
+        <v>689</v>
       </c>
     </row>
     <row r="259" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7911,7 +7917,7 @@
         <v>29</v>
       </c>
       <c r="B259" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C259" s="4" t="s">
         <v>38</v>
@@ -7923,7 +7929,7 @@
         <v>10</v>
       </c>
       <c r="J259" s="5" t="s">
-        <v>694</v>
+        <v>690</v>
       </c>
     </row>
     <row r="260" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7931,10 +7937,10 @@
         <v>29</v>
       </c>
       <c r="B260" s="4" t="s">
-        <v>186</v>
+        <v>150</v>
       </c>
       <c r="C260" s="4" t="s">
-        <v>189</v>
+        <v>38</v>
       </c>
       <c r="D260" s="4" t="b">
         <v>0</v>
@@ -7943,7 +7949,7 @@
         <v>10</v>
       </c>
       <c r="J260" s="5" t="s">
-        <v>513</v>
+        <v>691</v>
       </c>
     </row>
     <row r="261" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7951,7 +7957,7 @@
         <v>29</v>
       </c>
       <c r="B261" s="4" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C261" s="4" t="s">
         <v>189</v>
@@ -7963,7 +7969,7 @@
         <v>10</v>
       </c>
       <c r="J261" s="5" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
     </row>
     <row r="262" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7971,10 +7977,10 @@
         <v>29</v>
       </c>
       <c r="B262" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C262" s="4" t="s">
-        <v>45</v>
+        <v>189</v>
       </c>
       <c r="D262" s="4" t="b">
         <v>0</v>
@@ -7983,7 +7989,7 @@
         <v>10</v>
       </c>
       <c r="J262" s="5" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
     </row>
     <row r="263" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7991,10 +7997,10 @@
         <v>29</v>
       </c>
       <c r="B263" s="4" t="s">
-        <v>75</v>
+        <v>188</v>
       </c>
       <c r="C263" s="4" t="s">
-        <v>189</v>
+        <v>45</v>
       </c>
       <c r="D263" s="4" t="b">
         <v>0</v>
@@ -8003,7 +8009,7 @@
         <v>10</v>
       </c>
       <c r="J263" s="5" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
     </row>
     <row r="264" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8011,10 +8017,10 @@
         <v>29</v>
       </c>
       <c r="B264" s="4" t="s">
-        <v>190</v>
+        <v>75</v>
       </c>
       <c r="C264" s="4" t="s">
-        <v>271</v>
+        <v>189</v>
       </c>
       <c r="D264" s="4" t="b">
         <v>0</v>
@@ -8023,7 +8029,7 @@
         <v>10</v>
       </c>
       <c r="J264" s="5" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
     </row>
     <row r="265" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8031,10 +8037,10 @@
         <v>29</v>
       </c>
       <c r="B265" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C265" s="4" t="s">
-        <v>84</v>
+        <v>271</v>
       </c>
       <c r="D265" s="4" t="b">
         <v>0</v>
@@ -8043,7 +8049,7 @@
         <v>10</v>
       </c>
       <c r="J265" s="5" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
     </row>
     <row r="266" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8051,10 +8057,10 @@
         <v>29</v>
       </c>
       <c r="B266" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C266" s="4" t="s">
-        <v>45</v>
+        <v>84</v>
       </c>
       <c r="D266" s="4" t="b">
         <v>0</v>
@@ -8063,7 +8069,7 @@
         <v>10</v>
       </c>
       <c r="J266" s="5" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
     </row>
     <row r="267" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8071,10 +8077,10 @@
         <v>29</v>
       </c>
       <c r="B267" s="4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C267" s="4" t="s">
-        <v>84</v>
+        <v>45</v>
       </c>
       <c r="D267" s="4" t="b">
         <v>0</v>
@@ -8083,7 +8089,7 @@
         <v>10</v>
       </c>
       <c r="J267" s="5" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
     </row>
     <row r="268" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8091,10 +8097,10 @@
         <v>29</v>
       </c>
       <c r="B268" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C268" s="4" t="s">
-        <v>272</v>
+        <v>84</v>
       </c>
       <c r="D268" s="4" t="b">
         <v>0</v>
@@ -8103,7 +8109,7 @@
         <v>10</v>
       </c>
       <c r="J268" s="5" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
     </row>
     <row r="269" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8111,10 +8117,10 @@
         <v>29</v>
       </c>
       <c r="B269" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C269" s="4" t="s">
-        <v>84</v>
+        <v>272</v>
       </c>
       <c r="D269" s="4" t="b">
         <v>0</v>
@@ -8123,7 +8129,7 @@
         <v>10</v>
       </c>
       <c r="J269" s="5" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
     </row>
     <row r="270" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8131,10 +8137,10 @@
         <v>29</v>
       </c>
       <c r="B270" s="4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C270" s="4" t="s">
-        <v>45</v>
+        <v>84</v>
       </c>
       <c r="D270" s="4" t="b">
         <v>0</v>
@@ -8143,7 +8149,7 @@
         <v>10</v>
       </c>
       <c r="J270" s="5" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
     </row>
     <row r="271" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8151,10 +8157,10 @@
         <v>29</v>
       </c>
       <c r="B271" s="4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C271" s="4" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="D271" s="4" t="b">
         <v>0</v>
@@ -8163,7 +8169,7 @@
         <v>10</v>
       </c>
       <c r="J271" s="5" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
     </row>
     <row r="272" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8171,7 +8177,7 @@
         <v>29</v>
       </c>
       <c r="B272" s="4" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C272" s="4" t="s">
         <v>32</v>
@@ -8183,7 +8189,7 @@
         <v>10</v>
       </c>
       <c r="J272" s="5" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
     </row>
     <row r="273" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8191,10 +8197,10 @@
         <v>29</v>
       </c>
       <c r="B273" s="4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C273" s="4" t="s">
-        <v>84</v>
+        <v>32</v>
       </c>
       <c r="D273" s="4" t="b">
         <v>0</v>
@@ -8203,7 +8209,7 @@
         <v>10</v>
       </c>
       <c r="J273" s="5" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
     </row>
     <row r="274" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8211,10 +8217,10 @@
         <v>29</v>
       </c>
       <c r="B274" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C274" s="4" t="s">
-        <v>273</v>
+        <v>84</v>
       </c>
       <c r="D274" s="4" t="b">
         <v>0</v>
@@ -8223,7 +8229,7 @@
         <v>10</v>
       </c>
       <c r="J274" s="5" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
     </row>
     <row r="275" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8231,10 +8237,10 @@
         <v>29</v>
       </c>
       <c r="B275" s="4" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C275" s="4" t="s">
-        <v>189</v>
+        <v>273</v>
       </c>
       <c r="D275" s="4" t="b">
         <v>0</v>
@@ -8243,7 +8249,7 @@
         <v>10</v>
       </c>
       <c r="J275" s="5" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
     </row>
     <row r="276" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8251,10 +8257,10 @@
         <v>29</v>
       </c>
       <c r="B276" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C276" s="4" t="s">
-        <v>271</v>
+        <v>189</v>
       </c>
       <c r="D276" s="4" t="b">
         <v>0</v>
@@ -8263,7 +8269,7 @@
         <v>10</v>
       </c>
       <c r="J276" s="5" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
     </row>
     <row r="277" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8271,7 +8277,7 @@
         <v>29</v>
       </c>
       <c r="B277" s="4" t="s">
-        <v>274</v>
+        <v>205</v>
       </c>
       <c r="C277" s="4" t="s">
         <v>271</v>
@@ -8283,7 +8289,7 @@
         <v>10</v>
       </c>
       <c r="J277" s="5" t="s">
-        <v>695</v>
+        <v>527</v>
       </c>
     </row>
     <row r="278" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8291,7 +8297,7 @@
         <v>29</v>
       </c>
       <c r="B278" s="4" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C278" s="4" t="s">
         <v>271</v>
@@ -8303,7 +8309,7 @@
         <v>10</v>
       </c>
       <c r="J278" s="5" t="s">
-        <v>696</v>
+        <v>692</v>
       </c>
     </row>
     <row r="279" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8311,10 +8317,10 @@
         <v>29</v>
       </c>
       <c r="B279" s="4" t="s">
-        <v>153</v>
+        <v>275</v>
       </c>
       <c r="C279" s="4" t="s">
-        <v>84</v>
+        <v>271</v>
       </c>
       <c r="D279" s="4" t="b">
         <v>0</v>
@@ -8323,7 +8329,7 @@
         <v>10</v>
       </c>
       <c r="J279" s="5" t="s">
-        <v>530</v>
+        <v>693</v>
       </c>
     </row>
     <row r="280" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8331,10 +8337,10 @@
         <v>29</v>
       </c>
       <c r="B280" s="4" t="s">
-        <v>276</v>
+        <v>153</v>
       </c>
       <c r="C280" s="4" t="s">
-        <v>271</v>
+        <v>84</v>
       </c>
       <c r="D280" s="4" t="b">
         <v>0</v>
@@ -8343,7 +8349,7 @@
         <v>10</v>
       </c>
       <c r="J280" s="5" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
     </row>
     <row r="281" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8351,10 +8357,10 @@
         <v>29</v>
       </c>
       <c r="B281" s="4" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C281" s="4" t="s">
-        <v>84</v>
+        <v>271</v>
       </c>
       <c r="D281" s="4" t="b">
         <v>0</v>
@@ -8363,7 +8369,7 @@
         <v>10</v>
       </c>
       <c r="J281" s="5" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
     </row>
     <row r="282" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8371,10 +8377,10 @@
         <v>29</v>
       </c>
       <c r="B282" s="4" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C282" s="4" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="D282" s="4" t="b">
         <v>0</v>
@@ -8383,7 +8389,7 @@
         <v>10</v>
       </c>
       <c r="J282" s="5" t="s">
-        <v>697</v>
+        <v>530</v>
       </c>
     </row>
     <row r="283" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8391,10 +8397,10 @@
         <v>29</v>
       </c>
       <c r="B283" s="4" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C283" s="4" t="s">
-        <v>32</v>
+        <v>76</v>
       </c>
       <c r="D283" s="4" t="b">
         <v>0</v>
@@ -8403,7 +8409,7 @@
         <v>10</v>
       </c>
       <c r="J283" s="5" t="s">
-        <v>533</v>
+        <v>694</v>
       </c>
     </row>
     <row r="284" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8411,7 +8417,7 @@
         <v>29</v>
       </c>
       <c r="B284" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C284" s="4" t="s">
         <v>32</v>
@@ -8423,7 +8429,7 @@
         <v>10</v>
       </c>
       <c r="J284" s="5" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
     </row>
     <row r="285" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8431,7 +8437,7 @@
         <v>29</v>
       </c>
       <c r="B285" s="4" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C285" s="4" t="s">
         <v>32</v>
@@ -8443,7 +8449,7 @@
         <v>10</v>
       </c>
       <c r="J285" s="5" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
     </row>
     <row r="286" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8451,10 +8457,10 @@
         <v>29</v>
       </c>
       <c r="B286" s="4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C286" s="4" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D286" s="4" t="b">
         <v>0</v>
@@ -8463,7 +8469,7 @@
         <v>10</v>
       </c>
       <c r="J286" s="5" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
     </row>
     <row r="287" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8471,10 +8477,10 @@
         <v>29</v>
       </c>
       <c r="B287" s="4" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C287" s="4" t="s">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="D287" s="4" t="b">
         <v>0</v>
@@ -8483,7 +8489,7 @@
         <v>10</v>
       </c>
       <c r="J287" s="5" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
     </row>
     <row r="288" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8491,10 +8497,10 @@
         <v>29</v>
       </c>
       <c r="B288" s="4" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C288" s="4" t="s">
-        <v>45</v>
+        <v>84</v>
       </c>
       <c r="D288" s="4" t="b">
         <v>0</v>
@@ -8503,7 +8509,7 @@
         <v>10</v>
       </c>
       <c r="J288" s="5" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
     </row>
     <row r="289" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8511,10 +8517,10 @@
         <v>29</v>
       </c>
       <c r="B289" s="4" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C289" s="4" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="D289" s="4" t="b">
         <v>0</v>
@@ -8523,7 +8529,7 @@
         <v>10</v>
       </c>
       <c r="J289" s="5" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
     </row>
     <row r="290" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8531,10 +8537,10 @@
         <v>29</v>
       </c>
       <c r="B290" s="4" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C290" s="4" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="D290" s="4" t="b">
         <v>0</v>
@@ -8543,7 +8549,7 @@
         <v>10</v>
       </c>
       <c r="J290" s="5" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="291" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8551,10 +8557,10 @@
         <v>29</v>
       </c>
       <c r="B291" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C291" s="4" t="s">
-        <v>189</v>
+        <v>45</v>
       </c>
       <c r="D291" s="4" t="b">
         <v>0</v>
@@ -8563,7 +8569,7 @@
         <v>10</v>
       </c>
       <c r="J291" s="5" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
     </row>
     <row r="292" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8571,10 +8577,10 @@
         <v>29</v>
       </c>
       <c r="B292" s="4" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C292" s="4" t="s">
-        <v>32</v>
+        <v>189</v>
       </c>
       <c r="D292" s="4" t="b">
         <v>0</v>
@@ -8583,7 +8589,7 @@
         <v>10</v>
       </c>
       <c r="J292" s="5" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
     </row>
     <row r="293" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8591,7 +8597,7 @@
         <v>29</v>
       </c>
       <c r="B293" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C293" s="4" t="s">
         <v>32</v>
@@ -8603,7 +8609,7 @@
         <v>10</v>
       </c>
       <c r="J293" s="5" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
     </row>
     <row r="294" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8611,7 +8617,7 @@
         <v>29</v>
       </c>
       <c r="B294" s="4" t="s">
-        <v>12</v>
+        <v>289</v>
       </c>
       <c r="C294" s="4" t="s">
         <v>32</v>
@@ -8623,7 +8629,7 @@
         <v>10</v>
       </c>
       <c r="J294" s="5" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
     </row>
     <row r="295" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8631,10 +8637,10 @@
         <v>29</v>
       </c>
       <c r="B295" s="4" t="s">
-        <v>206</v>
+        <v>12</v>
       </c>
       <c r="C295" s="4" t="s">
-        <v>84</v>
+        <v>32</v>
       </c>
       <c r="D295" s="4" t="b">
         <v>0</v>
@@ -8643,7 +8649,7 @@
         <v>10</v>
       </c>
       <c r="J295" s="5" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
     </row>
     <row r="296" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8651,10 +8657,10 @@
         <v>29</v>
       </c>
       <c r="B296" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C296" s="4" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="D296" s="4" t="b">
         <v>0</v>
@@ -8663,7 +8669,7 @@
         <v>10</v>
       </c>
       <c r="J296" s="5" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
     </row>
     <row r="297" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8671,10 +8677,10 @@
         <v>29</v>
       </c>
       <c r="B297" s="4" t="s">
-        <v>290</v>
+        <v>207</v>
       </c>
       <c r="C297" s="4" t="s">
-        <v>38</v>
+        <v>76</v>
       </c>
       <c r="D297" s="4" t="b">
         <v>0</v>
@@ -8683,7 +8689,7 @@
         <v>10</v>
       </c>
       <c r="J297" s="5" t="s">
-        <v>698</v>
+        <v>544</v>
       </c>
     </row>
     <row r="298" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8691,22 +8697,19 @@
         <v>29</v>
       </c>
       <c r="B298" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C298" s="4" t="s">
-        <v>143</v>
+        <v>38</v>
       </c>
       <c r="D298" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="G298" s="4" t="s">
-        <v>17</v>
-      </c>
       <c r="H298" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J298" s="5" t="s">
-        <v>547</v>
+        <v>695</v>
       </c>
     </row>
     <row r="299" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8714,10 +8717,10 @@
         <v>29</v>
       </c>
       <c r="B299" s="4" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C299" s="4" t="s">
-        <v>210</v>
+        <v>143</v>
       </c>
       <c r="D299" s="4" t="b">
         <v>0</v>
@@ -8729,7 +8732,7 @@
         <v>10</v>
       </c>
       <c r="J299" s="5" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
     </row>
     <row r="300" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8737,7 +8740,7 @@
         <v>29</v>
       </c>
       <c r="B300" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C300" s="4" t="s">
         <v>210</v>
@@ -8752,7 +8755,7 @@
         <v>10</v>
       </c>
       <c r="J300" s="5" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
     </row>
     <row r="301" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8760,7 +8763,7 @@
         <v>29</v>
       </c>
       <c r="B301" s="4" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C301" s="4" t="s">
         <v>210</v>
@@ -8775,7 +8778,7 @@
         <v>10</v>
       </c>
       <c r="J301" s="5" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
     </row>
     <row r="302" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8783,7 +8786,7 @@
         <v>29</v>
       </c>
       <c r="B302" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C302" s="4" t="s">
         <v>210</v>
@@ -8798,7 +8801,7 @@
         <v>10</v>
       </c>
       <c r="J302" s="5" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
     </row>
     <row r="303" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8806,7 +8809,7 @@
         <v>29</v>
       </c>
       <c r="B303" s="4" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C303" s="4" t="s">
         <v>210</v>
@@ -8821,7 +8824,7 @@
         <v>10</v>
       </c>
       <c r="J303" s="5" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
     </row>
     <row r="304" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8829,7 +8832,7 @@
         <v>29</v>
       </c>
       <c r="B304" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C304" s="4" t="s">
         <v>210</v>
@@ -8844,7 +8847,7 @@
         <v>10</v>
       </c>
       <c r="J304" s="5" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
     </row>
     <row r="305" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8852,7 +8855,7 @@
         <v>29</v>
       </c>
       <c r="B305" s="4" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C305" s="4" t="s">
         <v>210</v>
@@ -8867,7 +8870,7 @@
         <v>10</v>
       </c>
       <c r="J305" s="5" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
     </row>
     <row r="306" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8875,7 +8878,7 @@
         <v>29</v>
       </c>
       <c r="B306" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C306" s="4" t="s">
         <v>210</v>
@@ -8890,7 +8893,7 @@
         <v>10</v>
       </c>
       <c r="J306" s="5" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
     </row>
     <row r="307" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8898,7 +8901,7 @@
         <v>29</v>
       </c>
       <c r="B307" s="4" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C307" s="4" t="s">
         <v>210</v>
@@ -8913,7 +8916,7 @@
         <v>10</v>
       </c>
       <c r="J307" s="5" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
     </row>
     <row r="308" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8921,7 +8924,7 @@
         <v>29</v>
       </c>
       <c r="B308" s="4" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C308" s="4" t="s">
         <v>210</v>
@@ -8936,7 +8939,7 @@
         <v>10</v>
       </c>
       <c r="J308" s="5" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
     </row>
     <row r="309" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8944,7 +8947,7 @@
         <v>29</v>
       </c>
       <c r="B309" s="4" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C309" s="4" t="s">
         <v>210</v>
@@ -8959,7 +8962,7 @@
         <v>10</v>
       </c>
       <c r="J309" s="5" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
     </row>
     <row r="310" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8967,7 +8970,7 @@
         <v>29</v>
       </c>
       <c r="B310" s="4" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C310" s="4" t="s">
         <v>210</v>
@@ -8982,7 +8985,7 @@
         <v>10</v>
       </c>
       <c r="J310" s="5" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
     </row>
     <row r="311" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8990,7 +8993,7 @@
         <v>29</v>
       </c>
       <c r="B311" s="4" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C311" s="4" t="s">
         <v>210</v>
@@ -9005,7 +9008,7 @@
         <v>10</v>
       </c>
       <c r="J311" s="5" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
     </row>
     <row r="312" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9013,7 +9016,7 @@
         <v>29</v>
       </c>
       <c r="B312" s="4" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C312" s="4" t="s">
         <v>210</v>
@@ -9028,7 +9031,7 @@
         <v>10</v>
       </c>
       <c r="J312" s="5" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
     </row>
     <row r="313" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9036,7 +9039,7 @@
         <v>29</v>
       </c>
       <c r="B313" s="4" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C313" s="4" t="s">
         <v>210</v>
@@ -9051,7 +9054,7 @@
         <v>10</v>
       </c>
       <c r="J313" s="5" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
     </row>
     <row r="314" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9059,7 +9062,7 @@
         <v>29</v>
       </c>
       <c r="B314" s="4" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C314" s="4" t="s">
         <v>210</v>
@@ -9074,7 +9077,7 @@
         <v>10</v>
       </c>
       <c r="J314" s="5" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
     </row>
     <row r="315" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9082,19 +9085,22 @@
         <v>29</v>
       </c>
       <c r="B315" s="4" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C315" s="4" t="s">
-        <v>84</v>
+        <v>210</v>
       </c>
       <c r="D315" s="4" t="b">
         <v>0</v>
       </c>
+      <c r="G315" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="H315" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J315" s="5" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
     </row>
     <row r="316" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9102,10 +9108,10 @@
         <v>29</v>
       </c>
       <c r="B316" s="4" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C316" s="4" t="s">
-        <v>32</v>
+        <v>84</v>
       </c>
       <c r="D316" s="4" t="b">
         <v>0</v>
@@ -9114,7 +9120,7 @@
         <v>10</v>
       </c>
       <c r="J316" s="5" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
     </row>
     <row r="317" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9122,10 +9128,10 @@
         <v>29</v>
       </c>
       <c r="B317" s="4" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C317" s="4" t="s">
-        <v>189</v>
+        <v>32</v>
       </c>
       <c r="D317" s="4" t="b">
         <v>0</v>
@@ -9134,7 +9140,7 @@
         <v>10</v>
       </c>
       <c r="J317" s="5" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
     </row>
     <row r="318" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9142,7 +9148,7 @@
         <v>29</v>
       </c>
       <c r="B318" s="4" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C318" s="4" t="s">
         <v>189</v>
@@ -9154,7 +9160,7 @@
         <v>10</v>
       </c>
       <c r="J318" s="5" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
     </row>
     <row r="319" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9162,10 +9168,10 @@
         <v>29</v>
       </c>
       <c r="B319" s="4" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C319" s="4" t="s">
-        <v>32</v>
+        <v>189</v>
       </c>
       <c r="D319" s="4" t="b">
         <v>0</v>
@@ -9174,7 +9180,7 @@
         <v>10</v>
       </c>
       <c r="J319" s="5" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
     </row>
     <row r="320" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9182,10 +9188,10 @@
         <v>29</v>
       </c>
       <c r="B320" s="4" t="s">
-        <v>227</v>
+        <v>312</v>
       </c>
       <c r="C320" s="4" t="s">
-        <v>271</v>
+        <v>32</v>
       </c>
       <c r="D320" s="4" t="b">
         <v>0</v>
@@ -9194,7 +9200,7 @@
         <v>10</v>
       </c>
       <c r="J320" s="5" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
     </row>
     <row r="321" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9202,7 +9208,7 @@
         <v>29</v>
       </c>
       <c r="B321" s="4" t="s">
-        <v>313</v>
+        <v>227</v>
       </c>
       <c r="C321" s="4" t="s">
         <v>271</v>
@@ -9214,7 +9220,7 @@
         <v>10</v>
       </c>
       <c r="J321" s="5" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
     </row>
     <row r="322" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9222,7 +9228,7 @@
         <v>29</v>
       </c>
       <c r="B322" s="4" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C322" s="4" t="s">
         <v>271</v>
@@ -9234,7 +9240,7 @@
         <v>10</v>
       </c>
       <c r="J322" s="5" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
     </row>
     <row r="323" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9242,7 +9248,7 @@
         <v>29</v>
       </c>
       <c r="B323" s="4" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C323" s="4" t="s">
         <v>271</v>
@@ -9254,7 +9260,7 @@
         <v>10</v>
       </c>
       <c r="J323" s="5" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="324" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9262,7 +9268,7 @@
         <v>29</v>
       </c>
       <c r="B324" s="4" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C324" s="4" t="s">
         <v>271</v>
@@ -9274,7 +9280,7 @@
         <v>10</v>
       </c>
       <c r="J324" s="5" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
     </row>
     <row r="325" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9282,10 +9288,10 @@
         <v>29</v>
       </c>
       <c r="B325" s="4" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C325" s="4" t="s">
-        <v>84</v>
+        <v>271</v>
       </c>
       <c r="D325" s="4" t="b">
         <v>0</v>
@@ -9294,7 +9300,7 @@
         <v>10</v>
       </c>
       <c r="J325" s="5" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
     </row>
     <row r="326" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9302,22 +9308,19 @@
         <v>29</v>
       </c>
       <c r="B326" s="4" t="s">
-        <v>212</v>
+        <v>317</v>
       </c>
       <c r="C326" s="4" t="s">
-        <v>210</v>
+        <v>84</v>
       </c>
       <c r="D326" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="G326" s="4" t="s">
-        <v>17</v>
-      </c>
       <c r="H326" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J326" s="5" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
     </row>
     <row r="327" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9325,7 +9328,7 @@
         <v>29</v>
       </c>
       <c r="B327" s="4" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C327" s="4" t="s">
         <v>210</v>
@@ -9340,7 +9343,7 @@
         <v>10</v>
       </c>
       <c r="J327" s="5" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
     </row>
     <row r="328" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9348,7 +9351,7 @@
         <v>29</v>
       </c>
       <c r="B328" s="4" t="s">
-        <v>318</v>
+        <v>211</v>
       </c>
       <c r="C328" s="4" t="s">
         <v>210</v>
@@ -9363,7 +9366,7 @@
         <v>10</v>
       </c>
       <c r="J328" s="5" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
     </row>
     <row r="329" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9371,19 +9374,22 @@
         <v>29</v>
       </c>
       <c r="B329" s="4" t="s">
-        <v>224</v>
+        <v>318</v>
       </c>
       <c r="C329" s="4" t="s">
-        <v>273</v>
+        <v>210</v>
       </c>
       <c r="D329" s="4" t="b">
         <v>0</v>
       </c>
+      <c r="G329" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="H329" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J329" s="5" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
     </row>
     <row r="330" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9391,7 +9397,7 @@
         <v>29</v>
       </c>
       <c r="B330" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C330" s="4" t="s">
         <v>273</v>
@@ -9403,7 +9409,7 @@
         <v>10</v>
       </c>
       <c r="J330" s="5" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
     </row>
     <row r="331" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9411,7 +9417,7 @@
         <v>29</v>
       </c>
       <c r="B331" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C331" s="4" t="s">
         <v>273</v>
@@ -9423,7 +9429,7 @@
         <v>10</v>
       </c>
       <c r="J331" s="5" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
     </row>
     <row r="332" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9431,7 +9437,7 @@
         <v>29</v>
       </c>
       <c r="B332" s="4" t="s">
-        <v>268</v>
+        <v>226</v>
       </c>
       <c r="C332" s="4" t="s">
         <v>273</v>
@@ -9443,7 +9449,7 @@
         <v>10</v>
       </c>
       <c r="J332" s="5" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
     </row>
     <row r="333" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9451,7 +9457,7 @@
         <v>29</v>
       </c>
       <c r="B333" s="4" t="s">
-        <v>319</v>
+        <v>268</v>
       </c>
       <c r="C333" s="4" t="s">
         <v>273</v>
@@ -9463,7 +9469,7 @@
         <v>10</v>
       </c>
       <c r="J333" s="5" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
     </row>
     <row r="334" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9471,22 +9477,19 @@
         <v>29</v>
       </c>
       <c r="B334" s="4" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C334" s="4" t="s">
-        <v>321</v>
+        <v>273</v>
       </c>
       <c r="D334" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="G334" s="4" t="s">
-        <v>17</v>
-      </c>
       <c r="H334" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J334" s="5" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
     </row>
     <row r="335" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9494,7 +9497,7 @@
         <v>29</v>
       </c>
       <c r="B335" s="4" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="C335" s="4" t="s">
         <v>321</v>
@@ -9509,7 +9512,7 @@
         <v>10</v>
       </c>
       <c r="J335" s="5" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
     </row>
     <row r="336" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9517,19 +9520,22 @@
         <v>29</v>
       </c>
       <c r="B336" s="4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C336" s="4" t="s">
-        <v>52</v>
+        <v>321</v>
       </c>
       <c r="D336" s="4" t="b">
         <v>0</v>
       </c>
+      <c r="G336" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="H336" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J336" s="5" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
     </row>
     <row r="337" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9537,7 +9543,7 @@
         <v>29</v>
       </c>
       <c r="B337" s="4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C337" s="4" t="s">
         <v>52</v>
@@ -9549,7 +9555,7 @@
         <v>10</v>
       </c>
       <c r="J337" s="5" t="s">
-        <v>699</v>
+        <v>583</v>
       </c>
     </row>
     <row r="338" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9557,22 +9563,19 @@
         <v>29</v>
       </c>
       <c r="B338" s="4" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C338" s="4" t="s">
-        <v>326</v>
+        <v>52</v>
       </c>
       <c r="D338" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="G338" s="4" t="s">
-        <v>17</v>
-      </c>
       <c r="H338" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J338" s="5" t="s">
-        <v>586</v>
+        <v>696</v>
       </c>
     </row>
     <row r="339" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9580,10 +9583,10 @@
         <v>29</v>
       </c>
       <c r="B339" s="4" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C339" s="4" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D339" s="4" t="b">
         <v>0</v>
@@ -9595,7 +9598,7 @@
         <v>10</v>
       </c>
       <c r="J339" s="5" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
     </row>
     <row r="340" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9603,42 +9606,42 @@
         <v>29</v>
       </c>
       <c r="B340" s="4" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C340" s="4" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="D340" s="4" t="b">
         <v>0</v>
       </c>
+      <c r="G340" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="H340" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J340" s="5" t="s">
-        <v>700</v>
+        <v>585</v>
       </c>
     </row>
     <row r="341" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A341" s="4" t="s">
-        <v>407</v>
+        <v>29</v>
       </c>
       <c r="B341" s="4" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C341" s="4" t="s">
-        <v>36</v>
+        <v>330</v>
       </c>
       <c r="D341" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="F341" s="4" t="s">
-        <v>403</v>
-      </c>
       <c r="H341" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J341" s="5" t="s">
-        <v>588</v>
+        <v>697</v>
       </c>
     </row>
     <row r="342" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9646,19 +9649,22 @@
         <v>407</v>
       </c>
       <c r="B342" s="4" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C342" s="4" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="D342" s="4" t="b">
         <v>0</v>
       </c>
+      <c r="F342" s="4" t="s">
+        <v>403</v>
+      </c>
       <c r="H342" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J342" s="5" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
     </row>
     <row r="343" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9666,10 +9672,10 @@
         <v>407</v>
       </c>
       <c r="B343" s="4" t="s">
-        <v>149</v>
+        <v>332</v>
       </c>
       <c r="C343" s="4" t="s">
-        <v>76</v>
+        <v>52</v>
       </c>
       <c r="D343" s="4" t="b">
         <v>0</v>
@@ -9678,7 +9684,7 @@
         <v>10</v>
       </c>
       <c r="J343" s="5" t="s">
-        <v>701</v>
+        <v>587</v>
       </c>
     </row>
     <row r="344" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9686,26 +9692,46 @@
         <v>407</v>
       </c>
       <c r="B344" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="C344" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D344" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H344" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J344" s="5" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="345" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+      <c r="A345" s="4" t="s">
+        <v>407</v>
+      </c>
+      <c r="B345" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C344" s="4" t="s">
+      <c r="C345" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D344" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E344" s="4" t="b">
+      <c r="D345" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E345" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="H344" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="J344" s="5" t="s">
-        <v>590</v>
+      <c r="H345" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J345" s="5" t="s">
+        <v>702</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J344" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <autoFilter ref="A1:J345" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10007,7 +10033,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B2" t="s">
         <v>405</v>
@@ -10018,10 +10044,10 @@
     </row>
     <row r="3" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C3" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
feat: Update descriptions in schema and dbt files for clarity and consistency
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A63F2F6C-EAFA-704C-80B3-981C26B3FB85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEBE6C08-B2A1-C24B-8DCE-3A0DDC38E841}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="660" windowWidth="30680" windowHeight="19740" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="660" windowWidth="30680" windowHeight="19740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tables" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1888" uniqueCount="705">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1890" uniqueCount="702">
   <si>
     <t>Table Name</t>
   </si>
@@ -1126,12 +1126,6 @@
     <t>MDM ID</t>
   </si>
   <si>
-    <t>CIF ID Nasabah</t>
-  </si>
-  <si>
-    <t>Nama Nasabah</t>
-  </si>
-  <si>
     <t>Nama Perusahaan</t>
   </si>
   <si>
@@ -1153,15 +1147,6 @@
     <t>Source Status</t>
   </si>
   <si>
-    <t>Status Customer</t>
-  </si>
-  <si>
-    <t>Kode Type</t>
-  </si>
-  <si>
-    <t>Tipe Customer</t>
-  </si>
-  <si>
     <t>Flag Pemerintah</t>
   </si>
   <si>
@@ -1228,15 +1213,6 @@
     <t>Channel Pembuka CIF</t>
   </si>
   <si>
-    <t>Channel Nasabah ( Consentisi Pemegang Nasabah)</t>
-  </si>
-  <si>
-    <t>Channel Nasabah ( Consent_Nameisi Pemegang Nasabah)</t>
-  </si>
-  <si>
-    <t>Cif Key Nasabah</t>
-  </si>
-  <si>
     <t>customer_icons.cif_key</t>
   </si>
   <si>
@@ -1489,9 +1465,6 @@
     <t>Channel yang digunakan untuk membuka rekening.</t>
   </si>
   <si>
-    <t>Jenis atau bentuk badan hukum nasabah/perusahaan.</t>
-  </si>
-  <si>
     <t>Saldo akhir untuk periode Month-to-Date.</t>
   </si>
   <si>
@@ -1525,21 +1498,12 @@
     <t>Hasil mapping/mirror dari pemilik channel.</t>
   </si>
   <si>
-    <t>ID nasabah/entity pada sistem Master Data Management.</t>
-  </si>
-  <si>
     <t>Nomor rekening.</t>
   </si>
   <si>
     <t>Kunci/identifier Customer Information File (CIF).</t>
   </si>
   <si>
-    <t>Kode jenis nasabah.</t>
-  </si>
-  <si>
-    <t>Deskripsi jenis nasabah, misalnya individu atau badan usaha.</t>
-  </si>
-  <si>
     <t>Kode region tempat CIF dibuka.</t>
   </si>
   <si>
@@ -1555,9 +1519,6 @@
     <t>Tanggal CIF dibuat atau dibuka.</t>
   </si>
   <si>
-    <t>Nama nasabah.</t>
-  </si>
-  <si>
     <t>Penanda apakah CIF terkait proses/produk Burekol atau buka rekening kolektif.</t>
   </si>
   <si>
@@ -1786,12 +1747,6 @@
     <t>Interest Income atau pendapatan bunga bulanan.</t>
   </si>
   <si>
-    <t>CIF utama/principal apabila nasabah memiliki beberapa CIF terkait.</t>
-  </si>
-  <si>
-    <t>Nasabah/perusahaan utama dalam satu kelompok usaha atau grup.</t>
-  </si>
-  <si>
     <t>CIF Key Nasabah (ID Nasabah)</t>
   </si>
   <si>
@@ -1975,12 +1930,6 @@
     <t>Account Number / Nomor Akun</t>
   </si>
   <si>
-    <t>Tipe nasabah</t>
-  </si>
-  <si>
-    <t>Kode tipe nasabah</t>
-  </si>
-  <si>
     <t>Kode Region pembukaan CIF</t>
   </si>
   <si>
@@ -2101,9 +2050,6 @@
     <t>Divisi yang menjadi pemilik segmen.</t>
   </si>
   <si>
-    <t>Sub segmen nasabah.</t>
-  </si>
-  <si>
     <t>Nama sentra atau unit bisnis yang menangani rekening</t>
   </si>
   <si>
@@ -2141,6 +2087,51 @@
   </si>
   <si>
     <t>Tanggal posisi atau tanggal transaksi data, digunakan untuk filter tanggal, bulan, tahun</t>
+  </si>
+  <si>
+    <t>CIF utama/principal apabila memiliki beberapa CIF terkait.</t>
+  </si>
+  <si>
+    <t>Consent Channel</t>
+  </si>
+  <si>
+    <t>Consent Channel Sebelum (Previous)</t>
+  </si>
+  <si>
+    <t>Cif Key</t>
+  </si>
+  <si>
+    <t>Nama</t>
+  </si>
+  <si>
+    <t>Jenis atau bentuk badan hukum</t>
+  </si>
+  <si>
+    <t>ID MDM / Global pada sistem Master Data Management.</t>
+  </si>
+  <si>
+    <t>Sub segment</t>
+  </si>
+  <si>
+    <t>Entity utama dalam satu kelompok usaha atau grup.</t>
+  </si>
+  <si>
+    <t>Kode tipe customer/nasabah</t>
+  </si>
+  <si>
+    <t>CIF Nasabah</t>
+  </si>
+  <si>
+    <t>Status Customer/nasabah</t>
+  </si>
+  <si>
+    <t>Tipe Customer/nasabah</t>
+  </si>
+  <si>
+    <t>Pendapatan Lain</t>
+  </si>
+  <si>
+    <t>Pendapatan Sewa</t>
   </si>
 </sst>
 </file>
@@ -2560,7 +2551,7 @@
         <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>408</v>
+        <v>400</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -2571,7 +2562,7 @@
         <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>410</v>
+        <v>402</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -2582,18 +2573,18 @@
         <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>409</v>
+        <v>401</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>406</v>
+        <v>398</v>
       </c>
       <c r="B6" t="s">
-        <v>407</v>
+        <v>399</v>
       </c>
       <c r="C6" t="s">
-        <v>411</v>
+        <v>403</v>
       </c>
     </row>
   </sheetData>
@@ -2633,7 +2624,7 @@
         <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>416</v>
+        <v>408</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>6</v>
@@ -2671,7 +2662,7 @@
         <v>10</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>704</v>
+        <v>686</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2708,13 +2699,13 @@
         <v>0</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>403</v>
+        <v>395</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J4" t="s">
-        <v>588</v>
+        <v>573</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="32" x14ac:dyDescent="0.2">
@@ -2731,13 +2722,13 @@
         <v>0</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>404</v>
+        <v>396</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J5" t="s">
-        <v>589</v>
+        <v>574</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2934,7 +2925,7 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>412</v>
+        <v>404</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>10</v>
@@ -2963,7 +2954,7 @@
         <v>10</v>
       </c>
       <c r="J16" t="s">
-        <v>699</v>
+        <v>681</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -2980,7 +2971,7 @@
         <v>0</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>415</v>
+        <v>407</v>
       </c>
       <c r="J17" t="s">
         <v>344</v>
@@ -3220,7 +3211,7 @@
         <v>0</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>403</v>
+        <v>395</v>
       </c>
       <c r="H29" s="4" t="s">
         <v>10</v>
@@ -3243,13 +3234,13 @@
         <v>0</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>404</v>
+        <v>396</v>
       </c>
       <c r="H30" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J30" t="s">
-        <v>453</v>
+        <v>445</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3269,7 +3260,7 @@
         <v>10</v>
       </c>
       <c r="J31" t="s">
-        <v>454</v>
+        <v>446</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3455,7 +3446,7 @@
         <v>10</v>
       </c>
       <c r="J40" s="5" t="s">
-        <v>703</v>
+        <v>685</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3472,7 +3463,7 @@
         <v>0</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>412</v>
+        <v>404</v>
       </c>
       <c r="H41" s="4" t="s">
         <v>10</v>
@@ -3498,7 +3489,7 @@
         <v>10</v>
       </c>
       <c r="J42" t="s">
-        <v>366</v>
+        <v>697</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3538,7 +3529,7 @@
         <v>10</v>
       </c>
       <c r="J44" t="s">
-        <v>590</v>
+        <v>575</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3558,7 +3549,7 @@
         <v>10</v>
       </c>
       <c r="J45" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="46" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3578,7 +3569,7 @@
         <v>10</v>
       </c>
       <c r="J46" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="47" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3598,7 +3589,7 @@
         <v>10</v>
       </c>
       <c r="J47" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
     </row>
     <row r="48" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3618,7 +3609,7 @@
         <v>10</v>
       </c>
       <c r="J48" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3638,7 +3629,7 @@
         <v>10</v>
       </c>
       <c r="J49" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3658,7 +3649,7 @@
         <v>10</v>
       </c>
       <c r="J50" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3678,7 +3669,7 @@
         <v>10</v>
       </c>
       <c r="J51" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="52" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3698,7 +3689,7 @@
         <v>10</v>
       </c>
       <c r="J52" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="53" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3715,13 +3706,13 @@
         <v>0</v>
       </c>
       <c r="H53" s="4" t="s">
-        <v>415</v>
+        <v>407</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>414</v>
+        <v>406</v>
       </c>
       <c r="J53" t="s">
-        <v>375</v>
+        <v>698</v>
       </c>
     </row>
     <row r="54" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3741,7 +3732,7 @@
         <v>10</v>
       </c>
       <c r="J54" t="s">
-        <v>376</v>
+        <v>696</v>
       </c>
     </row>
     <row r="55" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3761,7 +3752,7 @@
         <v>10</v>
       </c>
       <c r="J55" t="s">
-        <v>377</v>
+        <v>699</v>
       </c>
     </row>
     <row r="56" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3781,7 +3772,7 @@
         <v>10</v>
       </c>
       <c r="J56" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
     </row>
     <row r="57" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3801,7 +3792,7 @@
         <v>10</v>
       </c>
       <c r="J57" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
     </row>
     <row r="58" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3821,7 +3812,7 @@
         <v>10</v>
       </c>
       <c r="J58" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
     </row>
     <row r="59" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3841,7 +3832,7 @@
         <v>10</v>
       </c>
       <c r="J59" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
     </row>
     <row r="60" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3861,7 +3852,7 @@
         <v>10</v>
       </c>
       <c r="J60" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
     </row>
     <row r="61" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3881,7 +3872,7 @@
         <v>10</v>
       </c>
       <c r="J61" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
     </row>
     <row r="62" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3901,7 +3892,7 @@
         <v>10</v>
       </c>
       <c r="J62" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
     </row>
     <row r="63" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3921,7 +3912,7 @@
         <v>10</v>
       </c>
       <c r="J63" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
     </row>
     <row r="64" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3941,7 +3932,7 @@
         <v>10</v>
       </c>
       <c r="J64" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
     </row>
     <row r="65" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3961,7 +3952,7 @@
         <v>10</v>
       </c>
       <c r="J65" t="s">
-        <v>591</v>
+        <v>576</v>
       </c>
     </row>
     <row r="66" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3981,7 +3972,7 @@
         <v>10</v>
       </c>
       <c r="J66" t="s">
-        <v>592</v>
+        <v>577</v>
       </c>
     </row>
     <row r="67" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4001,7 +3992,7 @@
         <v>10</v>
       </c>
       <c r="J67" t="s">
-        <v>593</v>
+        <v>578</v>
       </c>
     </row>
     <row r="68" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4024,7 +4015,7 @@
         <v>10</v>
       </c>
       <c r="J68" t="s">
-        <v>594</v>
+        <v>579</v>
       </c>
     </row>
     <row r="69" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4044,7 +4035,7 @@
         <v>10</v>
       </c>
       <c r="J69" t="s">
-        <v>595</v>
+        <v>580</v>
       </c>
     </row>
     <row r="70" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4064,7 +4055,7 @@
         <v>10</v>
       </c>
       <c r="J70" t="s">
-        <v>596</v>
+        <v>581</v>
       </c>
     </row>
     <row r="71" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4084,7 +4075,7 @@
         <v>10</v>
       </c>
       <c r="J71" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
     </row>
     <row r="72" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4104,7 +4095,7 @@
         <v>10</v>
       </c>
       <c r="J72" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
     </row>
     <row r="73" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4124,7 +4115,7 @@
         <v>10</v>
       </c>
       <c r="J73" t="s">
-        <v>597</v>
+        <v>582</v>
       </c>
     </row>
     <row r="74" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4144,7 +4135,7 @@
         <v>10</v>
       </c>
       <c r="J74" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
     </row>
     <row r="75" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4164,7 +4155,7 @@
         <v>10</v>
       </c>
       <c r="J75" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
     </row>
     <row r="76" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4184,7 +4175,7 @@
         <v>10</v>
       </c>
       <c r="J76" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
     </row>
     <row r="77" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4204,7 +4195,7 @@
         <v>10</v>
       </c>
       <c r="J77" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
     </row>
     <row r="78" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4224,7 +4215,7 @@
         <v>10</v>
       </c>
       <c r="J78" t="s">
-        <v>598</v>
+        <v>583</v>
       </c>
     </row>
     <row r="79" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4244,7 +4235,7 @@
         <v>10</v>
       </c>
       <c r="J79" t="s">
-        <v>599</v>
+        <v>584</v>
       </c>
     </row>
     <row r="80" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4264,7 +4255,7 @@
         <v>10</v>
       </c>
       <c r="J80" t="s">
-        <v>601</v>
+        <v>586</v>
       </c>
     </row>
     <row r="81" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4284,7 +4275,7 @@
         <v>10</v>
       </c>
       <c r="J81" t="s">
-        <v>600</v>
+        <v>585</v>
       </c>
     </row>
     <row r="82" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4304,7 +4295,7 @@
         <v>10</v>
       </c>
       <c r="J82" t="s">
-        <v>602</v>
+        <v>587</v>
       </c>
     </row>
     <row r="83" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4360,7 +4351,7 @@
         <v>10</v>
       </c>
       <c r="J85" t="s">
-        <v>603</v>
+        <v>588</v>
       </c>
     </row>
     <row r="86" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4434,7 +4425,7 @@
         <v>10</v>
       </c>
       <c r="J89" t="s">
-        <v>604</v>
+        <v>589</v>
       </c>
     </row>
     <row r="90" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4454,7 +4445,7 @@
         <v>10</v>
       </c>
       <c r="J90" t="s">
-        <v>605</v>
+        <v>590</v>
       </c>
     </row>
     <row r="91" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4474,7 +4465,7 @@
         <v>10</v>
       </c>
       <c r="J91" t="s">
-        <v>606</v>
+        <v>591</v>
       </c>
     </row>
     <row r="92" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4494,7 +4485,7 @@
         <v>10</v>
       </c>
       <c r="J92" t="s">
-        <v>607</v>
+        <v>592</v>
       </c>
     </row>
     <row r="93" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4514,7 +4505,7 @@
         <v>10</v>
       </c>
       <c r="J93" t="s">
-        <v>608</v>
+        <v>593</v>
       </c>
     </row>
     <row r="94" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4534,7 +4525,7 @@
         <v>10</v>
       </c>
       <c r="J94" t="s">
-        <v>609</v>
+        <v>594</v>
       </c>
     </row>
     <row r="95" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4554,7 +4545,7 @@
         <v>10</v>
       </c>
       <c r="J95" t="s">
-        <v>610</v>
+        <v>595</v>
       </c>
     </row>
     <row r="96" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4574,7 +4565,7 @@
         <v>10</v>
       </c>
       <c r="J96" t="s">
-        <v>611</v>
+        <v>596</v>
       </c>
     </row>
     <row r="97" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4594,7 +4585,7 @@
         <v>10</v>
       </c>
       <c r="J97" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
     </row>
     <row r="98" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4614,7 +4605,7 @@
         <v>10</v>
       </c>
       <c r="J98" t="s">
-        <v>612</v>
+        <v>597</v>
       </c>
     </row>
     <row r="99" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4634,7 +4625,7 @@
         <v>10</v>
       </c>
       <c r="J99" t="s">
-        <v>613</v>
+        <v>598</v>
       </c>
     </row>
     <row r="100" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4654,7 +4645,7 @@
         <v>10</v>
       </c>
       <c r="J100" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
     </row>
     <row r="101" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4674,7 +4665,7 @@
         <v>10</v>
       </c>
       <c r="J101" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
     </row>
     <row r="102" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4712,7 +4703,7 @@
         <v>10</v>
       </c>
       <c r="J103" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
     </row>
     <row r="104" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4732,7 +4723,7 @@
         <v>10</v>
       </c>
       <c r="J104" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
     </row>
     <row r="105" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4755,7 +4746,7 @@
         <v>10</v>
       </c>
       <c r="J105" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
     </row>
     <row r="106" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4777,7 +4768,9 @@
       <c r="H106" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J106"/>
+      <c r="J106" t="s">
+        <v>701</v>
+      </c>
     </row>
     <row r="107" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A107" s="4" t="s">
@@ -4798,7 +4791,9 @@
       <c r="H107" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J107"/>
+      <c r="J107" t="s">
+        <v>700</v>
+      </c>
     </row>
     <row r="108" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A108" s="4" t="s">
@@ -4817,7 +4812,7 @@
         <v>10</v>
       </c>
       <c r="J108" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
     </row>
     <row r="109" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4873,7 +4868,7 @@
         <v>10</v>
       </c>
       <c r="J111" t="s">
-        <v>616</v>
+        <v>601</v>
       </c>
     </row>
     <row r="112" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4893,7 +4888,7 @@
         <v>10</v>
       </c>
       <c r="J112" t="s">
-        <v>614</v>
+        <v>599</v>
       </c>
     </row>
     <row r="113" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4913,7 +4908,7 @@
         <v>10</v>
       </c>
       <c r="J113" t="s">
-        <v>615</v>
+        <v>600</v>
       </c>
     </row>
     <row r="114" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4933,7 +4928,7 @@
         <v>10</v>
       </c>
       <c r="J114" t="s">
-        <v>598</v>
+        <v>583</v>
       </c>
     </row>
     <row r="115" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4953,7 +4948,7 @@
         <v>10</v>
       </c>
       <c r="J115" t="s">
-        <v>617</v>
+        <v>602</v>
       </c>
     </row>
     <row r="116" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4973,7 +4968,7 @@
         <v>10</v>
       </c>
       <c r="J116" t="s">
-        <v>618</v>
+        <v>603</v>
       </c>
     </row>
     <row r="117" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4993,7 +4988,7 @@
         <v>10</v>
       </c>
       <c r="J117" t="s">
-        <v>619</v>
+        <v>604</v>
       </c>
     </row>
     <row r="118" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5013,7 +5008,7 @@
         <v>10</v>
       </c>
       <c r="J118" t="s">
-        <v>620</v>
+        <v>605</v>
       </c>
     </row>
     <row r="119" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5033,7 +5028,7 @@
         <v>10</v>
       </c>
       <c r="J119" t="s">
-        <v>621</v>
+        <v>606</v>
       </c>
     </row>
     <row r="120" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5053,7 +5048,7 @@
         <v>10</v>
       </c>
       <c r="J120" t="s">
-        <v>622</v>
+        <v>607</v>
       </c>
     </row>
     <row r="121" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5073,7 +5068,7 @@
         <v>10</v>
       </c>
       <c r="J121" t="s">
-        <v>623</v>
+        <v>608</v>
       </c>
     </row>
     <row r="122" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5093,7 +5088,7 @@
         <v>10</v>
       </c>
       <c r="J122" t="s">
-        <v>626</v>
+        <v>611</v>
       </c>
     </row>
     <row r="123" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5113,7 +5108,7 @@
         <v>10</v>
       </c>
       <c r="J123" t="s">
-        <v>625</v>
+        <v>610</v>
       </c>
     </row>
     <row r="124" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5133,7 +5128,7 @@
         <v>10</v>
       </c>
       <c r="J124" t="s">
-        <v>624</v>
+        <v>609</v>
       </c>
     </row>
     <row r="125" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5153,7 +5148,7 @@
         <v>10</v>
       </c>
       <c r="J125" t="s">
-        <v>627</v>
+        <v>612</v>
       </c>
     </row>
     <row r="126" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5173,7 +5168,7 @@
         <v>10</v>
       </c>
       <c r="J126" t="s">
-        <v>628</v>
+        <v>613</v>
       </c>
     </row>
     <row r="127" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5193,7 +5188,7 @@
         <v>10</v>
       </c>
       <c r="J127" t="s">
-        <v>636</v>
+        <v>621</v>
       </c>
     </row>
     <row r="128" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5213,7 +5208,7 @@
         <v>10</v>
       </c>
       <c r="J128" t="s">
-        <v>637</v>
+        <v>622</v>
       </c>
     </row>
     <row r="129" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5233,7 +5228,7 @@
         <v>10</v>
       </c>
       <c r="J129" t="s">
-        <v>638</v>
+        <v>623</v>
       </c>
     </row>
     <row r="130" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5253,7 +5248,7 @@
         <v>10</v>
       </c>
       <c r="J130" t="s">
-        <v>639</v>
+        <v>624</v>
       </c>
     </row>
     <row r="131" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5273,7 +5268,7 @@
         <v>10</v>
       </c>
       <c r="J131" t="s">
-        <v>640</v>
+        <v>625</v>
       </c>
     </row>
     <row r="132" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5293,7 +5288,7 @@
         <v>10</v>
       </c>
       <c r="J132" t="s">
-        <v>641</v>
+        <v>626</v>
       </c>
     </row>
     <row r="133" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5313,7 +5308,7 @@
         <v>10</v>
       </c>
       <c r="J133" t="s">
-        <v>642</v>
+        <v>627</v>
       </c>
     </row>
     <row r="134" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5333,7 +5328,7 @@
         <v>10</v>
       </c>
       <c r="J134" t="s">
-        <v>643</v>
+        <v>628</v>
       </c>
     </row>
     <row r="135" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5353,7 +5348,7 @@
         <v>10</v>
       </c>
       <c r="J135" t="s">
-        <v>644</v>
+        <v>629</v>
       </c>
     </row>
     <row r="136" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5373,7 +5368,7 @@
         <v>10</v>
       </c>
       <c r="J136" t="s">
-        <v>646</v>
+        <v>631</v>
       </c>
     </row>
     <row r="137" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5393,7 +5388,7 @@
         <v>10</v>
       </c>
       <c r="J137" t="s">
-        <v>645</v>
+        <v>630</v>
       </c>
     </row>
     <row r="138" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5413,7 +5408,7 @@
         <v>10</v>
       </c>
       <c r="J138" t="s">
-        <v>400</v>
+        <v>688</v>
       </c>
     </row>
     <row r="139" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5433,7 +5428,7 @@
         <v>10</v>
       </c>
       <c r="J139" t="s">
-        <v>401</v>
+        <v>689</v>
       </c>
     </row>
     <row r="140" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5453,7 +5448,7 @@
         <v>10</v>
       </c>
       <c r="J140" t="s">
-        <v>647</v>
+        <v>632</v>
       </c>
     </row>
     <row r="141" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5476,7 +5471,7 @@
         <v>10</v>
       </c>
       <c r="J141" s="5" t="s">
-        <v>700</v>
+        <v>682</v>
       </c>
     </row>
     <row r="142" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5496,7 +5491,7 @@
         <v>10</v>
       </c>
       <c r="J142" t="s">
-        <v>648</v>
+        <v>633</v>
       </c>
     </row>
     <row r="143" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5513,13 +5508,13 @@
         <v>0</v>
       </c>
       <c r="F143" s="4" t="s">
-        <v>403</v>
+        <v>395</v>
       </c>
       <c r="H143" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J143" t="s">
-        <v>402</v>
+        <v>690</v>
       </c>
     </row>
     <row r="144" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5539,7 +5534,7 @@
         <v>10</v>
       </c>
       <c r="J144" t="s">
-        <v>650</v>
+        <v>696</v>
       </c>
     </row>
     <row r="145" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5559,7 +5554,7 @@
         <v>10</v>
       </c>
       <c r="J145" t="s">
-        <v>649</v>
+        <v>699</v>
       </c>
     </row>
     <row r="146" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5579,7 +5574,7 @@
         <v>10</v>
       </c>
       <c r="J146" t="s">
-        <v>651</v>
+        <v>634</v>
       </c>
     </row>
     <row r="147" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5599,7 +5594,7 @@
         <v>10</v>
       </c>
       <c r="J147" t="s">
-        <v>652</v>
+        <v>635</v>
       </c>
     </row>
     <row r="148" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5619,7 +5614,7 @@
         <v>10</v>
       </c>
       <c r="J148" t="s">
-        <v>653</v>
+        <v>636</v>
       </c>
     </row>
     <row r="149" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5639,7 +5634,7 @@
         <v>10</v>
       </c>
       <c r="J149" t="s">
-        <v>655</v>
+        <v>638</v>
       </c>
     </row>
     <row r="150" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5659,7 +5654,7 @@
         <v>10</v>
       </c>
       <c r="J150" t="s">
-        <v>654</v>
+        <v>637</v>
       </c>
     </row>
     <row r="151" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5679,7 +5674,7 @@
         <v>10</v>
       </c>
       <c r="J151" t="s">
-        <v>367</v>
+        <v>691</v>
       </c>
     </row>
     <row r="152" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5699,7 +5694,7 @@
         <v>10</v>
       </c>
       <c r="J152" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="153" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5719,7 +5714,7 @@
         <v>10</v>
       </c>
       <c r="J153" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
     </row>
     <row r="154" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5739,7 +5734,7 @@
         <v>10</v>
       </c>
       <c r="J154" t="s">
-        <v>464</v>
+        <v>456</v>
       </c>
     </row>
     <row r="155" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5759,7 +5754,7 @@
         <v>10</v>
       </c>
       <c r="J155" t="s">
-        <v>612</v>
+        <v>597</v>
       </c>
     </row>
     <row r="156" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5779,7 +5774,7 @@
         <v>10</v>
       </c>
       <c r="J156" t="s">
-        <v>616</v>
+        <v>601</v>
       </c>
     </row>
     <row r="157" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5799,7 +5794,7 @@
         <v>10</v>
       </c>
       <c r="J157" t="s">
-        <v>614</v>
+        <v>599</v>
       </c>
     </row>
     <row r="158" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5819,7 +5814,7 @@
         <v>10</v>
       </c>
       <c r="J158" t="s">
-        <v>635</v>
+        <v>620</v>
       </c>
     </row>
     <row r="159" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5839,7 +5834,7 @@
         <v>10</v>
       </c>
       <c r="J159" t="s">
-        <v>634</v>
+        <v>619</v>
       </c>
     </row>
     <row r="160" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5859,7 +5854,7 @@
         <v>10</v>
       </c>
       <c r="J160" t="s">
-        <v>633</v>
+        <v>618</v>
       </c>
     </row>
     <row r="161" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5879,7 +5874,7 @@
         <v>10</v>
       </c>
       <c r="J161" t="s">
-        <v>629</v>
+        <v>614</v>
       </c>
     </row>
     <row r="162" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5899,7 +5894,7 @@
         <v>10</v>
       </c>
       <c r="J162" t="s">
-        <v>630</v>
+        <v>615</v>
       </c>
     </row>
     <row r="163" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5919,7 +5914,7 @@
         <v>10</v>
       </c>
       <c r="J163" t="s">
-        <v>455</v>
+        <v>447</v>
       </c>
     </row>
     <row r="164" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5939,7 +5934,7 @@
         <v>10</v>
       </c>
       <c r="J164" t="s">
-        <v>456</v>
+        <v>448</v>
       </c>
     </row>
     <row r="165" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5959,7 +5954,7 @@
         <v>10</v>
       </c>
       <c r="J165" t="s">
-        <v>457</v>
+        <v>449</v>
       </c>
     </row>
     <row r="166" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5979,7 +5974,7 @@
         <v>10</v>
       </c>
       <c r="J166" t="s">
-        <v>458</v>
+        <v>450</v>
       </c>
     </row>
     <row r="167" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -5999,7 +5994,7 @@
         <v>10</v>
       </c>
       <c r="J167" t="s">
-        <v>459</v>
+        <v>451</v>
       </c>
     </row>
     <row r="168" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6019,7 +6014,7 @@
         <v>10</v>
       </c>
       <c r="J168" t="s">
-        <v>460</v>
+        <v>452</v>
       </c>
     </row>
     <row r="169" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6042,7 +6037,7 @@
         <v>10</v>
       </c>
       <c r="J169" t="s">
-        <v>461</v>
+        <v>453</v>
       </c>
     </row>
     <row r="170" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6062,7 +6057,7 @@
         <v>10</v>
       </c>
       <c r="J170" t="s">
-        <v>462</v>
+        <v>454</v>
       </c>
     </row>
     <row r="171" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6082,7 +6077,7 @@
         <v>10</v>
       </c>
       <c r="J171" t="s">
-        <v>463</v>
+        <v>455</v>
       </c>
     </row>
     <row r="172" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6102,7 +6097,7 @@
         <v>10</v>
       </c>
       <c r="J172" t="s">
-        <v>631</v>
+        <v>616</v>
       </c>
     </row>
     <row r="173" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6122,7 +6117,7 @@
         <v>10</v>
       </c>
       <c r="J173" t="s">
-        <v>632</v>
+        <v>617</v>
       </c>
     </row>
     <row r="174" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6142,7 +6137,7 @@
         <v>10</v>
       </c>
       <c r="J174" t="s">
-        <v>656</v>
+        <v>639</v>
       </c>
     </row>
     <row r="175" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6162,7 +6157,7 @@
         <v>10</v>
       </c>
       <c r="J175" t="s">
-        <v>657</v>
+        <v>640</v>
       </c>
     </row>
     <row r="176" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6182,7 +6177,7 @@
         <v>10</v>
       </c>
       <c r="J176" t="s">
-        <v>658</v>
+        <v>641</v>
       </c>
     </row>
     <row r="177" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6202,7 +6197,7 @@
         <v>10</v>
       </c>
       <c r="J177" t="s">
-        <v>659</v>
+        <v>642</v>
       </c>
     </row>
     <row r="178" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6222,7 +6217,7 @@
         <v>10</v>
       </c>
       <c r="J178" t="s">
-        <v>659</v>
+        <v>642</v>
       </c>
     </row>
     <row r="179" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6242,7 +6237,7 @@
         <v>10</v>
       </c>
       <c r="J179" t="s">
-        <v>660</v>
+        <v>643</v>
       </c>
     </row>
     <row r="180" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6262,7 +6257,7 @@
         <v>10</v>
       </c>
       <c r="J180" t="s">
-        <v>661</v>
+        <v>644</v>
       </c>
     </row>
     <row r="181" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6285,7 +6280,7 @@
         <v>10</v>
       </c>
       <c r="J181" t="s">
-        <v>662</v>
+        <v>645</v>
       </c>
     </row>
     <row r="182" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6308,7 +6303,7 @@
         <v>10</v>
       </c>
       <c r="J182" t="s">
-        <v>663</v>
+        <v>646</v>
       </c>
     </row>
     <row r="183" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6331,7 +6326,7 @@
         <v>10</v>
       </c>
       <c r="J183" t="s">
-        <v>664</v>
+        <v>647</v>
       </c>
     </row>
     <row r="184" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6354,7 +6349,7 @@
         <v>10</v>
       </c>
       <c r="J184" t="s">
-        <v>665</v>
+        <v>648</v>
       </c>
     </row>
     <row r="185" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6377,7 +6372,7 @@
         <v>10</v>
       </c>
       <c r="J185" t="s">
-        <v>666</v>
+        <v>649</v>
       </c>
     </row>
     <row r="186" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6397,7 +6392,7 @@
         <v>10</v>
       </c>
       <c r="J186" t="s">
-        <v>667</v>
+        <v>650</v>
       </c>
     </row>
     <row r="187" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6417,7 +6412,7 @@
         <v>10</v>
       </c>
       <c r="J187" t="s">
-        <v>668</v>
+        <v>651</v>
       </c>
     </row>
     <row r="188" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6437,7 +6432,7 @@
         <v>10</v>
       </c>
       <c r="J188" t="s">
-        <v>669</v>
+        <v>652</v>
       </c>
     </row>
     <row r="189" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6457,7 +6452,7 @@
         <v>10</v>
       </c>
       <c r="J189" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
     </row>
     <row r="190" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6477,7 +6472,7 @@
         <v>10</v>
       </c>
       <c r="J190" t="s">
-        <v>464</v>
+        <v>456</v>
       </c>
     </row>
     <row r="191" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6497,7 +6492,7 @@
         <v>10</v>
       </c>
       <c r="J191" t="s">
-        <v>670</v>
+        <v>653</v>
       </c>
     </row>
     <row r="192" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6517,7 +6512,7 @@
         <v>10</v>
       </c>
       <c r="J192" t="s">
-        <v>671</v>
+        <v>654</v>
       </c>
     </row>
     <row r="193" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6537,7 +6532,7 @@
         <v>10</v>
       </c>
       <c r="J193" t="s">
-        <v>672</v>
+        <v>655</v>
       </c>
     </row>
     <row r="194" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6557,7 +6552,7 @@
         <v>10</v>
       </c>
       <c r="J194" t="s">
-        <v>673</v>
+        <v>656</v>
       </c>
     </row>
     <row r="195" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6577,7 +6572,7 @@
         <v>10</v>
       </c>
       <c r="J195" t="s">
-        <v>674</v>
+        <v>657</v>
       </c>
     </row>
     <row r="196" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6597,7 +6592,7 @@
         <v>10</v>
       </c>
       <c r="J196" t="s">
-        <v>626</v>
+        <v>611</v>
       </c>
     </row>
     <row r="197" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6617,7 +6612,7 @@
         <v>10</v>
       </c>
       <c r="J197" t="s">
-        <v>675</v>
+        <v>658</v>
       </c>
     </row>
     <row r="198" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6637,7 +6632,7 @@
         <v>10</v>
       </c>
       <c r="J198" t="s">
-        <v>676</v>
+        <v>659</v>
       </c>
     </row>
     <row r="199" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6657,7 +6652,7 @@
         <v>10</v>
       </c>
       <c r="J199" t="s">
-        <v>677</v>
+        <v>660</v>
       </c>
     </row>
     <row r="200" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6677,7 +6672,7 @@
         <v>10</v>
       </c>
       <c r="J200" t="s">
-        <v>678</v>
+        <v>661</v>
       </c>
     </row>
     <row r="201" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6697,7 +6692,7 @@
         <v>10</v>
       </c>
       <c r="J201" t="s">
-        <v>679</v>
+        <v>662</v>
       </c>
     </row>
     <row r="202" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6717,7 +6712,7 @@
         <v>10</v>
       </c>
       <c r="J202" t="s">
-        <v>680</v>
+        <v>663</v>
       </c>
     </row>
     <row r="203" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6737,7 +6732,7 @@
         <v>10</v>
       </c>
       <c r="J203" t="s">
-        <v>681</v>
+        <v>664</v>
       </c>
     </row>
     <row r="204" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6760,7 +6755,7 @@
         <v>10</v>
       </c>
       <c r="J204" t="s">
-        <v>682</v>
+        <v>665</v>
       </c>
     </row>
     <row r="205" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6783,7 +6778,7 @@
         <v>10</v>
       </c>
       <c r="J205" t="s">
-        <v>683</v>
+        <v>666</v>
       </c>
     </row>
     <row r="206" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6806,7 +6801,7 @@
         <v>10</v>
       </c>
       <c r="J206" t="s">
-        <v>684</v>
+        <v>667</v>
       </c>
     </row>
     <row r="207" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6829,7 +6824,7 @@
         <v>10</v>
       </c>
       <c r="J207" t="s">
-        <v>685</v>
+        <v>668</v>
       </c>
     </row>
     <row r="208" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6852,7 +6847,7 @@
         <v>10</v>
       </c>
       <c r="J208" t="s">
-        <v>465</v>
+        <v>457</v>
       </c>
     </row>
     <row r="209" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6875,7 +6870,7 @@
         <v>10</v>
       </c>
       <c r="J209" t="s">
-        <v>466</v>
+        <v>458</v>
       </c>
     </row>
     <row r="210" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6898,7 +6893,7 @@
         <v>10</v>
       </c>
       <c r="J210" s="5" t="s">
-        <v>467</v>
+        <v>459</v>
       </c>
     </row>
     <row r="211" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6921,7 +6916,7 @@
         <v>10</v>
       </c>
       <c r="J211" s="5" t="s">
-        <v>468</v>
+        <v>460</v>
       </c>
     </row>
     <row r="212" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6944,7 +6939,7 @@
         <v>10</v>
       </c>
       <c r="J212" s="5" t="s">
-        <v>469</v>
+        <v>461</v>
       </c>
     </row>
     <row r="213" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6967,7 +6962,7 @@
         <v>10</v>
       </c>
       <c r="J213" s="5" t="s">
-        <v>470</v>
+        <v>462</v>
       </c>
     </row>
     <row r="214" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6987,7 +6982,7 @@
         <v>10</v>
       </c>
       <c r="J214" s="5" t="s">
-        <v>471</v>
+        <v>463</v>
       </c>
     </row>
     <row r="215" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7007,7 +7002,7 @@
         <v>10</v>
       </c>
       <c r="J215" s="5" t="s">
-        <v>472</v>
+        <v>464</v>
       </c>
     </row>
     <row r="216" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7027,7 +7022,7 @@
         <v>10</v>
       </c>
       <c r="J216" s="5" t="s">
-        <v>473</v>
+        <v>465</v>
       </c>
     </row>
     <row r="217" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7050,7 +7045,7 @@
         <v>10</v>
       </c>
       <c r="J217" s="5" t="s">
-        <v>474</v>
+        <v>466</v>
       </c>
     </row>
     <row r="218" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7073,7 +7068,7 @@
         <v>10</v>
       </c>
       <c r="J218" s="5" t="s">
-        <v>475</v>
+        <v>467</v>
       </c>
     </row>
     <row r="219" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7096,7 +7091,7 @@
         <v>10</v>
       </c>
       <c r="J219" s="5" t="s">
-        <v>476</v>
+        <v>468</v>
       </c>
     </row>
     <row r="220" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7116,7 +7111,7 @@
         <v>10</v>
       </c>
       <c r="J220" s="5" t="s">
-        <v>477</v>
+        <v>469</v>
       </c>
     </row>
     <row r="221" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7136,7 +7131,7 @@
         <v>10</v>
       </c>
       <c r="J221" s="5" t="s">
-        <v>478</v>
+        <v>470</v>
       </c>
     </row>
     <row r="222" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7156,7 +7151,7 @@
         <v>10</v>
       </c>
       <c r="J222" s="5" t="s">
-        <v>479</v>
+        <v>471</v>
       </c>
     </row>
     <row r="223" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7176,7 +7171,7 @@
         <v>10</v>
       </c>
       <c r="J223" s="5" t="s">
-        <v>480</v>
+        <v>472</v>
       </c>
     </row>
     <row r="224" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7196,7 +7191,7 @@
         <v>10</v>
       </c>
       <c r="J224" s="5" t="s">
-        <v>481</v>
+        <v>473</v>
       </c>
     </row>
     <row r="225" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7216,7 +7211,7 @@
         <v>10</v>
       </c>
       <c r="J225" s="5" t="s">
-        <v>482</v>
+        <v>474</v>
       </c>
     </row>
     <row r="226" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7236,7 +7231,7 @@
         <v>10</v>
       </c>
       <c r="J226" s="5" t="s">
-        <v>483</v>
+        <v>475</v>
       </c>
     </row>
     <row r="227" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7256,7 +7251,7 @@
         <v>10</v>
       </c>
       <c r="J227" s="5" t="s">
-        <v>484</v>
+        <v>476</v>
       </c>
     </row>
     <row r="228" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7276,7 +7271,7 @@
         <v>10</v>
       </c>
       <c r="J228" s="5" t="s">
-        <v>485</v>
+        <v>477</v>
       </c>
     </row>
     <row r="229" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7296,7 +7291,7 @@
         <v>10</v>
       </c>
       <c r="J229" s="5" t="s">
-        <v>486</v>
+        <v>478</v>
       </c>
     </row>
     <row r="230" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7316,7 +7311,7 @@
         <v>10</v>
       </c>
       <c r="J230" s="5" t="s">
-        <v>487</v>
+        <v>692</v>
       </c>
     </row>
     <row r="231" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7339,7 +7334,7 @@
         <v>10</v>
       </c>
       <c r="J231" s="5" t="s">
-        <v>488</v>
+        <v>479</v>
       </c>
     </row>
     <row r="232" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7362,7 +7357,7 @@
         <v>10</v>
       </c>
       <c r="J232" s="5" t="s">
-        <v>489</v>
+        <v>480</v>
       </c>
     </row>
     <row r="233" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7385,7 +7380,7 @@
         <v>10</v>
       </c>
       <c r="J233" s="5" t="s">
-        <v>490</v>
+        <v>481</v>
       </c>
     </row>
     <row r="234" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7408,7 +7403,7 @@
         <v>10</v>
       </c>
       <c r="J234" s="5" t="s">
-        <v>491</v>
+        <v>482</v>
       </c>
     </row>
     <row r="235" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7431,7 +7426,7 @@
         <v>10</v>
       </c>
       <c r="J235" s="5" t="s">
-        <v>492</v>
+        <v>483</v>
       </c>
     </row>
     <row r="236" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7454,7 +7449,7 @@
         <v>10</v>
       </c>
       <c r="J236" s="5" t="s">
-        <v>493</v>
+        <v>484</v>
       </c>
     </row>
     <row r="237" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7477,7 +7472,7 @@
         <v>10</v>
       </c>
       <c r="J237" s="5" t="s">
-        <v>494</v>
+        <v>485</v>
       </c>
     </row>
     <row r="238" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7500,7 +7495,7 @@
         <v>10</v>
       </c>
       <c r="J238" s="5" t="s">
-        <v>495</v>
+        <v>486</v>
       </c>
     </row>
     <row r="239" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7520,7 +7515,7 @@
         <v>10</v>
       </c>
       <c r="J239" s="5" t="s">
-        <v>496</v>
+        <v>487</v>
       </c>
     </row>
     <row r="240" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7543,7 +7538,7 @@
         <v>10</v>
       </c>
       <c r="J240" s="5" t="s">
-        <v>497</v>
+        <v>488</v>
       </c>
     </row>
     <row r="241" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7563,7 +7558,7 @@
         <v>10</v>
       </c>
       <c r="J241" s="5" t="s">
-        <v>498</v>
+        <v>489</v>
       </c>
     </row>
     <row r="242" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7586,7 +7581,7 @@
         <v>10</v>
       </c>
       <c r="J242" s="5" t="s">
-        <v>701</v>
+        <v>683</v>
       </c>
     </row>
     <row r="243" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7606,7 +7601,7 @@
         <v>10</v>
       </c>
       <c r="J243" s="5" t="s">
-        <v>499</v>
+        <v>693</v>
       </c>
     </row>
     <row r="244" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7626,7 +7621,7 @@
         <v>10</v>
       </c>
       <c r="J244" s="5" t="s">
-        <v>500</v>
+        <v>490</v>
       </c>
     </row>
     <row r="245" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7643,13 +7638,13 @@
         <v>0</v>
       </c>
       <c r="F245" s="4" t="s">
-        <v>403</v>
+        <v>395</v>
       </c>
       <c r="H245" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J245" s="5" t="s">
-        <v>501</v>
+        <v>491</v>
       </c>
     </row>
     <row r="246" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7669,7 +7664,7 @@
         <v>10</v>
       </c>
       <c r="J246" s="5" t="s">
-        <v>686</v>
+        <v>669</v>
       </c>
     </row>
     <row r="247" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7688,8 +7683,8 @@
       <c r="H247" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J247" s="5" t="s">
-        <v>502</v>
+      <c r="J247" t="s">
+        <v>696</v>
       </c>
     </row>
     <row r="248" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7708,8 +7703,8 @@
       <c r="H248" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J248" s="5" t="s">
-        <v>503</v>
+      <c r="J248" t="s">
+        <v>699</v>
       </c>
     </row>
     <row r="249" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7729,7 +7724,7 @@
         <v>10</v>
       </c>
       <c r="J249" s="5" t="s">
-        <v>504</v>
+        <v>492</v>
       </c>
     </row>
     <row r="250" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7749,7 +7744,7 @@
         <v>10</v>
       </c>
       <c r="J250" s="5" t="s">
-        <v>505</v>
+        <v>493</v>
       </c>
     </row>
     <row r="251" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7769,7 +7764,7 @@
         <v>10</v>
       </c>
       <c r="J251" s="5" t="s">
-        <v>506</v>
+        <v>494</v>
       </c>
     </row>
     <row r="252" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7789,7 +7784,7 @@
         <v>10</v>
       </c>
       <c r="J252" s="5" t="s">
-        <v>507</v>
+        <v>495</v>
       </c>
     </row>
     <row r="253" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7809,7 +7804,7 @@
         <v>10</v>
       </c>
       <c r="J253" s="5" t="s">
-        <v>508</v>
+        <v>496</v>
       </c>
     </row>
     <row r="254" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7829,7 +7824,7 @@
         <v>10</v>
       </c>
       <c r="J254" s="5" t="s">
-        <v>509</v>
+        <v>691</v>
       </c>
     </row>
     <row r="255" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7849,7 +7844,7 @@
         <v>10</v>
       </c>
       <c r="J255" s="5" t="s">
-        <v>687</v>
+        <v>670</v>
       </c>
     </row>
     <row r="256" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7869,7 +7864,7 @@
         <v>10</v>
       </c>
       <c r="J256" s="5" t="s">
-        <v>688</v>
+        <v>671</v>
       </c>
     </row>
     <row r="257" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7889,7 +7884,7 @@
         <v>10</v>
       </c>
       <c r="J257" s="5" t="s">
-        <v>510</v>
+        <v>497</v>
       </c>
     </row>
     <row r="258" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7909,7 +7904,7 @@
         <v>10</v>
       </c>
       <c r="J258" s="5" t="s">
-        <v>689</v>
+        <v>672</v>
       </c>
     </row>
     <row r="259" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7929,7 +7924,7 @@
         <v>10</v>
       </c>
       <c r="J259" s="5" t="s">
-        <v>690</v>
+        <v>673</v>
       </c>
     </row>
     <row r="260" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7949,7 +7944,7 @@
         <v>10</v>
       </c>
       <c r="J260" s="5" t="s">
-        <v>691</v>
+        <v>694</v>
       </c>
     </row>
     <row r="261" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7969,7 +7964,7 @@
         <v>10</v>
       </c>
       <c r="J261" s="5" t="s">
-        <v>511</v>
+        <v>498</v>
       </c>
     </row>
     <row r="262" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7989,7 +7984,7 @@
         <v>10</v>
       </c>
       <c r="J262" s="5" t="s">
-        <v>512</v>
+        <v>499</v>
       </c>
     </row>
     <row r="263" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8009,7 +8004,7 @@
         <v>10</v>
       </c>
       <c r="J263" s="5" t="s">
-        <v>513</v>
+        <v>500</v>
       </c>
     </row>
     <row r="264" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8029,7 +8024,7 @@
         <v>10</v>
       </c>
       <c r="J264" s="5" t="s">
-        <v>514</v>
+        <v>501</v>
       </c>
     </row>
     <row r="265" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8049,7 +8044,7 @@
         <v>10</v>
       </c>
       <c r="J265" s="5" t="s">
-        <v>515</v>
+        <v>502</v>
       </c>
     </row>
     <row r="266" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8069,7 +8064,7 @@
         <v>10</v>
       </c>
       <c r="J266" s="5" t="s">
-        <v>516</v>
+        <v>503</v>
       </c>
     </row>
     <row r="267" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8089,7 +8084,7 @@
         <v>10</v>
       </c>
       <c r="J267" s="5" t="s">
-        <v>517</v>
+        <v>504</v>
       </c>
     </row>
     <row r="268" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8109,7 +8104,7 @@
         <v>10</v>
       </c>
       <c r="J268" s="5" t="s">
-        <v>518</v>
+        <v>505</v>
       </c>
     </row>
     <row r="269" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8129,7 +8124,7 @@
         <v>10</v>
       </c>
       <c r="J269" s="5" t="s">
-        <v>519</v>
+        <v>506</v>
       </c>
     </row>
     <row r="270" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8149,7 +8144,7 @@
         <v>10</v>
       </c>
       <c r="J270" s="5" t="s">
-        <v>520</v>
+        <v>507</v>
       </c>
     </row>
     <row r="271" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8169,7 +8164,7 @@
         <v>10</v>
       </c>
       <c r="J271" s="5" t="s">
-        <v>521</v>
+        <v>508</v>
       </c>
     </row>
     <row r="272" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8189,7 +8184,7 @@
         <v>10</v>
       </c>
       <c r="J272" s="5" t="s">
-        <v>522</v>
+        <v>509</v>
       </c>
     </row>
     <row r="273" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8209,7 +8204,7 @@
         <v>10</v>
       </c>
       <c r="J273" s="5" t="s">
-        <v>523</v>
+        <v>510</v>
       </c>
     </row>
     <row r="274" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8229,7 +8224,7 @@
         <v>10</v>
       </c>
       <c r="J274" s="5" t="s">
-        <v>524</v>
+        <v>511</v>
       </c>
     </row>
     <row r="275" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8249,7 +8244,7 @@
         <v>10</v>
       </c>
       <c r="J275" s="5" t="s">
-        <v>525</v>
+        <v>512</v>
       </c>
     </row>
     <row r="276" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8269,7 +8264,7 @@
         <v>10</v>
       </c>
       <c r="J276" s="5" t="s">
-        <v>526</v>
+        <v>513</v>
       </c>
     </row>
     <row r="277" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8289,7 +8284,7 @@
         <v>10</v>
       </c>
       <c r="J277" s="5" t="s">
-        <v>527</v>
+        <v>514</v>
       </c>
     </row>
     <row r="278" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8309,7 +8304,7 @@
         <v>10</v>
       </c>
       <c r="J278" s="5" t="s">
-        <v>692</v>
+        <v>674</v>
       </c>
     </row>
     <row r="279" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8329,7 +8324,7 @@
         <v>10</v>
       </c>
       <c r="J279" s="5" t="s">
-        <v>693</v>
+        <v>675</v>
       </c>
     </row>
     <row r="280" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8349,7 +8344,7 @@
         <v>10</v>
       </c>
       <c r="J280" s="5" t="s">
-        <v>528</v>
+        <v>515</v>
       </c>
     </row>
     <row r="281" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8369,7 +8364,7 @@
         <v>10</v>
       </c>
       <c r="J281" s="5" t="s">
-        <v>529</v>
+        <v>516</v>
       </c>
     </row>
     <row r="282" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8389,7 +8384,7 @@
         <v>10</v>
       </c>
       <c r="J282" s="5" t="s">
-        <v>530</v>
+        <v>517</v>
       </c>
     </row>
     <row r="283" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8409,7 +8404,7 @@
         <v>10</v>
       </c>
       <c r="J283" s="5" t="s">
-        <v>694</v>
+        <v>676</v>
       </c>
     </row>
     <row r="284" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8429,7 +8424,7 @@
         <v>10</v>
       </c>
       <c r="J284" s="5" t="s">
-        <v>531</v>
+        <v>518</v>
       </c>
     </row>
     <row r="285" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8449,7 +8444,7 @@
         <v>10</v>
       </c>
       <c r="J285" s="5" t="s">
-        <v>532</v>
+        <v>519</v>
       </c>
     </row>
     <row r="286" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8469,7 +8464,7 @@
         <v>10</v>
       </c>
       <c r="J286" s="5" t="s">
-        <v>533</v>
+        <v>520</v>
       </c>
     </row>
     <row r="287" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8489,7 +8484,7 @@
         <v>10</v>
       </c>
       <c r="J287" s="5" t="s">
-        <v>534</v>
+        <v>521</v>
       </c>
     </row>
     <row r="288" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8509,7 +8504,7 @@
         <v>10</v>
       </c>
       <c r="J288" s="5" t="s">
-        <v>535</v>
+        <v>522</v>
       </c>
     </row>
     <row r="289" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8529,7 +8524,7 @@
         <v>10</v>
       </c>
       <c r="J289" s="5" t="s">
-        <v>536</v>
+        <v>523</v>
       </c>
     </row>
     <row r="290" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8549,7 +8544,7 @@
         <v>10</v>
       </c>
       <c r="J290" s="5" t="s">
-        <v>537</v>
+        <v>524</v>
       </c>
     </row>
     <row r="291" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8569,7 +8564,7 @@
         <v>10</v>
       </c>
       <c r="J291" s="5" t="s">
-        <v>538</v>
+        <v>525</v>
       </c>
     </row>
     <row r="292" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8589,7 +8584,7 @@
         <v>10</v>
       </c>
       <c r="J292" s="5" t="s">
-        <v>539</v>
+        <v>526</v>
       </c>
     </row>
     <row r="293" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8609,7 +8604,7 @@
         <v>10</v>
       </c>
       <c r="J293" s="5" t="s">
-        <v>540</v>
+        <v>527</v>
       </c>
     </row>
     <row r="294" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8629,7 +8624,7 @@
         <v>10</v>
       </c>
       <c r="J294" s="5" t="s">
-        <v>541</v>
+        <v>528</v>
       </c>
     </row>
     <row r="295" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8649,7 +8644,7 @@
         <v>10</v>
       </c>
       <c r="J295" s="5" t="s">
-        <v>542</v>
+        <v>529</v>
       </c>
     </row>
     <row r="296" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8669,7 +8664,7 @@
         <v>10</v>
       </c>
       <c r="J296" s="5" t="s">
-        <v>543</v>
+        <v>530</v>
       </c>
     </row>
     <row r="297" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8689,7 +8684,7 @@
         <v>10</v>
       </c>
       <c r="J297" s="5" t="s">
-        <v>544</v>
+        <v>531</v>
       </c>
     </row>
     <row r="298" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8709,7 +8704,7 @@
         <v>10</v>
       </c>
       <c r="J298" s="5" t="s">
-        <v>695</v>
+        <v>677</v>
       </c>
     </row>
     <row r="299" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8732,7 +8727,7 @@
         <v>10</v>
       </c>
       <c r="J299" s="5" t="s">
-        <v>545</v>
+        <v>532</v>
       </c>
     </row>
     <row r="300" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8755,7 +8750,7 @@
         <v>10</v>
       </c>
       <c r="J300" s="5" t="s">
-        <v>546</v>
+        <v>533</v>
       </c>
     </row>
     <row r="301" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8778,7 +8773,7 @@
         <v>10</v>
       </c>
       <c r="J301" s="5" t="s">
-        <v>547</v>
+        <v>534</v>
       </c>
     </row>
     <row r="302" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8801,7 +8796,7 @@
         <v>10</v>
       </c>
       <c r="J302" s="5" t="s">
-        <v>548</v>
+        <v>535</v>
       </c>
     </row>
     <row r="303" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8824,7 +8819,7 @@
         <v>10</v>
       </c>
       <c r="J303" s="5" t="s">
-        <v>549</v>
+        <v>536</v>
       </c>
     </row>
     <row r="304" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8847,7 +8842,7 @@
         <v>10</v>
       </c>
       <c r="J304" s="5" t="s">
-        <v>550</v>
+        <v>537</v>
       </c>
     </row>
     <row r="305" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8870,7 +8865,7 @@
         <v>10</v>
       </c>
       <c r="J305" s="5" t="s">
-        <v>551</v>
+        <v>538</v>
       </c>
     </row>
     <row r="306" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8893,7 +8888,7 @@
         <v>10</v>
       </c>
       <c r="J306" s="5" t="s">
-        <v>552</v>
+        <v>539</v>
       </c>
     </row>
     <row r="307" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8916,7 +8911,7 @@
         <v>10</v>
       </c>
       <c r="J307" s="5" t="s">
-        <v>553</v>
+        <v>540</v>
       </c>
     </row>
     <row r="308" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8939,7 +8934,7 @@
         <v>10</v>
       </c>
       <c r="J308" s="5" t="s">
-        <v>554</v>
+        <v>541</v>
       </c>
     </row>
     <row r="309" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8962,7 +8957,7 @@
         <v>10</v>
       </c>
       <c r="J309" s="5" t="s">
-        <v>555</v>
+        <v>542</v>
       </c>
     </row>
     <row r="310" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8985,7 +8980,7 @@
         <v>10</v>
       </c>
       <c r="J310" s="5" t="s">
-        <v>556</v>
+        <v>543</v>
       </c>
     </row>
     <row r="311" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9008,7 +9003,7 @@
         <v>10</v>
       </c>
       <c r="J311" s="5" t="s">
-        <v>557</v>
+        <v>544</v>
       </c>
     </row>
     <row r="312" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9031,7 +9026,7 @@
         <v>10</v>
       </c>
       <c r="J312" s="5" t="s">
-        <v>558</v>
+        <v>545</v>
       </c>
     </row>
     <row r="313" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9054,7 +9049,7 @@
         <v>10</v>
       </c>
       <c r="J313" s="5" t="s">
-        <v>559</v>
+        <v>546</v>
       </c>
     </row>
     <row r="314" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9077,7 +9072,7 @@
         <v>10</v>
       </c>
       <c r="J314" s="5" t="s">
-        <v>560</v>
+        <v>547</v>
       </c>
     </row>
     <row r="315" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9100,7 +9095,7 @@
         <v>10</v>
       </c>
       <c r="J315" s="5" t="s">
-        <v>561</v>
+        <v>548</v>
       </c>
     </row>
     <row r="316" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9120,7 +9115,7 @@
         <v>10</v>
       </c>
       <c r="J316" s="5" t="s">
-        <v>562</v>
+        <v>549</v>
       </c>
     </row>
     <row r="317" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9140,7 +9135,7 @@
         <v>10</v>
       </c>
       <c r="J317" s="5" t="s">
-        <v>563</v>
+        <v>550</v>
       </c>
     </row>
     <row r="318" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9160,7 +9155,7 @@
         <v>10</v>
       </c>
       <c r="J318" s="5" t="s">
-        <v>564</v>
+        <v>551</v>
       </c>
     </row>
     <row r="319" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9180,7 +9175,7 @@
         <v>10</v>
       </c>
       <c r="J319" s="5" t="s">
-        <v>565</v>
+        <v>552</v>
       </c>
     </row>
     <row r="320" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9200,7 +9195,7 @@
         <v>10</v>
       </c>
       <c r="J320" s="5" t="s">
-        <v>566</v>
+        <v>553</v>
       </c>
     </row>
     <row r="321" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9220,7 +9215,7 @@
         <v>10</v>
       </c>
       <c r="J321" s="5" t="s">
-        <v>567</v>
+        <v>554</v>
       </c>
     </row>
     <row r="322" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9240,7 +9235,7 @@
         <v>10</v>
       </c>
       <c r="J322" s="5" t="s">
-        <v>568</v>
+        <v>555</v>
       </c>
     </row>
     <row r="323" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9260,7 +9255,7 @@
         <v>10</v>
       </c>
       <c r="J323" s="5" t="s">
-        <v>569</v>
+        <v>556</v>
       </c>
     </row>
     <row r="324" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9280,7 +9275,7 @@
         <v>10</v>
       </c>
       <c r="J324" s="5" t="s">
-        <v>570</v>
+        <v>557</v>
       </c>
     </row>
     <row r="325" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9300,7 +9295,7 @@
         <v>10</v>
       </c>
       <c r="J325" s="5" t="s">
-        <v>571</v>
+        <v>558</v>
       </c>
     </row>
     <row r="326" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9320,7 +9315,7 @@
         <v>10</v>
       </c>
       <c r="J326" s="5" t="s">
-        <v>572</v>
+        <v>559</v>
       </c>
     </row>
     <row r="327" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9343,7 +9338,7 @@
         <v>10</v>
       </c>
       <c r="J327" s="5" t="s">
-        <v>573</v>
+        <v>560</v>
       </c>
     </row>
     <row r="328" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9366,7 +9361,7 @@
         <v>10</v>
       </c>
       <c r="J328" s="5" t="s">
-        <v>574</v>
+        <v>561</v>
       </c>
     </row>
     <row r="329" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9389,7 +9384,7 @@
         <v>10</v>
       </c>
       <c r="J329" s="5" t="s">
-        <v>575</v>
+        <v>562</v>
       </c>
     </row>
     <row r="330" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9409,7 +9404,7 @@
         <v>10</v>
       </c>
       <c r="J330" s="5" t="s">
-        <v>576</v>
+        <v>563</v>
       </c>
     </row>
     <row r="331" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9429,7 +9424,7 @@
         <v>10</v>
       </c>
       <c r="J331" s="5" t="s">
-        <v>577</v>
+        <v>564</v>
       </c>
     </row>
     <row r="332" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9449,7 +9444,7 @@
         <v>10</v>
       </c>
       <c r="J332" s="5" t="s">
-        <v>578</v>
+        <v>565</v>
       </c>
     </row>
     <row r="333" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9469,7 +9464,7 @@
         <v>10</v>
       </c>
       <c r="J333" s="5" t="s">
-        <v>579</v>
+        <v>566</v>
       </c>
     </row>
     <row r="334" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9489,7 +9484,7 @@
         <v>10</v>
       </c>
       <c r="J334" s="5" t="s">
-        <v>580</v>
+        <v>567</v>
       </c>
     </row>
     <row r="335" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9512,7 +9507,7 @@
         <v>10</v>
       </c>
       <c r="J335" s="5" t="s">
-        <v>581</v>
+        <v>568</v>
       </c>
     </row>
     <row r="336" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9535,7 +9530,7 @@
         <v>10</v>
       </c>
       <c r="J336" s="5" t="s">
-        <v>582</v>
+        <v>569</v>
       </c>
     </row>
     <row r="337" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9555,7 +9550,7 @@
         <v>10</v>
       </c>
       <c r="J337" s="5" t="s">
-        <v>583</v>
+        <v>570</v>
       </c>
     </row>
     <row r="338" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9575,7 +9570,7 @@
         <v>10</v>
       </c>
       <c r="J338" s="5" t="s">
-        <v>696</v>
+        <v>678</v>
       </c>
     </row>
     <row r="339" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9598,7 +9593,7 @@
         <v>10</v>
       </c>
       <c r="J339" s="5" t="s">
-        <v>584</v>
+        <v>571</v>
       </c>
     </row>
     <row r="340" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9621,7 +9616,7 @@
         <v>10</v>
       </c>
       <c r="J340" s="5" t="s">
-        <v>585</v>
+        <v>572</v>
       </c>
     </row>
     <row r="341" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9641,12 +9636,12 @@
         <v>10</v>
       </c>
       <c r="J341" s="5" t="s">
-        <v>697</v>
+        <v>679</v>
       </c>
     </row>
     <row r="342" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A342" s="4" t="s">
-        <v>407</v>
+        <v>399</v>
       </c>
       <c r="B342" s="4" t="s">
         <v>331</v>
@@ -9658,18 +9653,18 @@
         <v>0</v>
       </c>
       <c r="F342" s="4" t="s">
-        <v>403</v>
+        <v>395</v>
       </c>
       <c r="H342" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J342" s="5" t="s">
-        <v>586</v>
+        <v>687</v>
       </c>
     </row>
     <row r="343" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A343" s="4" t="s">
-        <v>407</v>
+        <v>399</v>
       </c>
       <c r="B343" s="4" t="s">
         <v>332</v>
@@ -9684,12 +9679,12 @@
         <v>10</v>
       </c>
       <c r="J343" s="5" t="s">
-        <v>587</v>
+        <v>695</v>
       </c>
     </row>
     <row r="344" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A344" s="4" t="s">
-        <v>407</v>
+        <v>399</v>
       </c>
       <c r="B344" s="4" t="s">
         <v>149</v>
@@ -9704,12 +9699,12 @@
         <v>10</v>
       </c>
       <c r="J344" s="5" t="s">
-        <v>698</v>
+        <v>680</v>
       </c>
     </row>
     <row r="345" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A345" s="4" t="s">
-        <v>407</v>
+        <v>399</v>
       </c>
       <c r="B345" s="4" t="s">
         <v>31</v>
@@ -9727,7 +9722,7 @@
         <v>10</v>
       </c>
       <c r="J345" s="5" t="s">
-        <v>702</v>
+        <v>684</v>
       </c>
     </row>
   </sheetData>
@@ -9773,10 +9768,10 @@
         <v>89</v>
       </c>
       <c r="C2" t="s">
-        <v>413</v>
+        <v>405</v>
       </c>
       <c r="D2" t="s">
-        <v>414</v>
+        <v>406</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9787,10 +9782,10 @@
         <v>51</v>
       </c>
       <c r="C3" t="s">
-        <v>417</v>
+        <v>409</v>
       </c>
       <c r="E3" t="s">
-        <v>444</v>
+        <v>436</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9801,10 +9796,10 @@
         <v>51</v>
       </c>
       <c r="C4" t="s">
-        <v>418</v>
+        <v>410</v>
       </c>
       <c r="E4" t="s">
-        <v>445</v>
+        <v>437</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9815,10 +9810,10 @@
         <v>51</v>
       </c>
       <c r="C5" t="s">
-        <v>419</v>
+        <v>411</v>
       </c>
       <c r="E5" t="s">
-        <v>446</v>
+        <v>438</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9829,13 +9824,13 @@
         <v>51</v>
       </c>
       <c r="C6" t="s">
-        <v>420</v>
+        <v>412</v>
       </c>
       <c r="D6" t="s">
-        <v>449</v>
+        <v>441</v>
       </c>
       <c r="E6" t="s">
-        <v>434</v>
+        <v>426</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9846,10 +9841,10 @@
         <v>51</v>
       </c>
       <c r="C7" t="s">
-        <v>421</v>
+        <v>413</v>
       </c>
       <c r="E7" t="s">
-        <v>433</v>
+        <v>425</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9860,10 +9855,10 @@
         <v>51</v>
       </c>
       <c r="C8" t="s">
-        <v>422</v>
+        <v>414</v>
       </c>
       <c r="E8" t="s">
-        <v>435</v>
+        <v>427</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9874,10 +9869,10 @@
         <v>51</v>
       </c>
       <c r="C9" t="s">
-        <v>423</v>
+        <v>415</v>
       </c>
       <c r="E9" t="s">
-        <v>436</v>
+        <v>428</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9888,10 +9883,10 @@
         <v>51</v>
       </c>
       <c r="C10" t="s">
-        <v>424</v>
+        <v>416</v>
       </c>
       <c r="E10" t="s">
-        <v>447</v>
+        <v>439</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9902,10 +9897,10 @@
         <v>51</v>
       </c>
       <c r="C11" t="s">
-        <v>425</v>
+        <v>417</v>
       </c>
       <c r="E11" t="s">
-        <v>437</v>
+        <v>429</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9916,10 +9911,10 @@
         <v>51</v>
       </c>
       <c r="C12" t="s">
-        <v>426</v>
+        <v>418</v>
       </c>
       <c r="E12" t="s">
-        <v>438</v>
+        <v>430</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9930,10 +9925,10 @@
         <v>51</v>
       </c>
       <c r="C13" t="s">
-        <v>427</v>
+        <v>419</v>
       </c>
       <c r="E13" t="s">
-        <v>448</v>
+        <v>440</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9944,10 +9939,10 @@
         <v>51</v>
       </c>
       <c r="C14" t="s">
-        <v>428</v>
+        <v>420</v>
       </c>
       <c r="E14" t="s">
-        <v>439</v>
+        <v>431</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9958,10 +9953,10 @@
         <v>51</v>
       </c>
       <c r="C15" t="s">
-        <v>429</v>
+        <v>421</v>
       </c>
       <c r="E15" t="s">
-        <v>440</v>
+        <v>432</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9972,10 +9967,10 @@
         <v>51</v>
       </c>
       <c r="C16" t="s">
-        <v>430</v>
+        <v>422</v>
       </c>
       <c r="E16" t="s">
-        <v>441</v>
+        <v>433</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -9986,10 +9981,10 @@
         <v>51</v>
       </c>
       <c r="C17" t="s">
-        <v>432</v>
+        <v>424</v>
       </c>
       <c r="E17" t="s">
-        <v>442</v>
+        <v>434</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -10000,10 +9995,10 @@
         <v>51</v>
       </c>
       <c r="C18" t="s">
-        <v>431</v>
+        <v>423</v>
       </c>
       <c r="E18" t="s">
-        <v>443</v>
+        <v>435</v>
       </c>
     </row>
   </sheetData>
@@ -10033,10 +10028,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>452</v>
+        <v>444</v>
       </c>
       <c r="B2" t="s">
-        <v>405</v>
+        <v>397</v>
       </c>
       <c r="C2" t="s">
         <v>21</v>
@@ -10044,10 +10039,10 @@
     </row>
     <row r="3" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>451</v>
+        <v>443</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>450</v>
+        <v>442</v>
       </c>
       <c r="C3" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
feat: Add Indonesian stop words filtering to search query processing
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEBE6C08-B2A1-C24B-8DCE-3A0DDC38E841}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CF3AF11-B869-654D-B77E-085C29D3DBFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="660" windowWidth="30680" windowHeight="19740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1492,9 +1492,6 @@
     <t>Tanggal transaksi terakhir (last transaction date).</t>
   </si>
   <si>
-    <t>Nilai saldo yang diblokir atau tidak dapat digunakan.</t>
-  </si>
-  <si>
     <t>Hasil mapping/mirror dari pemilik channel.</t>
   </si>
   <si>
@@ -1624,18 +1621,6 @@
     <t>Satuan atau multiplier yang digunakan pada original term, misalnya hari/bulan/tahun.</t>
   </si>
   <si>
-    <t>Nilai pokok pinjaman dalam Rupiah.</t>
-  </si>
-  <si>
-    <t>Saldo pokok kredit yang masih terutang/outstanding.</t>
-  </si>
-  <si>
-    <t>Nilai penyesuaian PSAK dengan kategori/komponen DMA sesuai definisi internal.</t>
-  </si>
-  <si>
-    <t>Nilai penyesuaian PSAK dengan kategori/komponen ACC sesuai definisi internal.</t>
-  </si>
-  <si>
     <t>Rata-rata pokok pinjaman berdasarkan PSAK untuk periode Month-to-Date.</t>
   </si>
   <si>
@@ -2132,6 +2117,21 @@
   </si>
   <si>
     <t>Pendapatan Sewa</t>
+  </si>
+  <si>
+    <t>Nilai saldo diblokir atau tidak dapat digunakan.</t>
+  </si>
+  <si>
+    <t>Nilai pokok pinjaman Rupiah.</t>
+  </si>
+  <si>
+    <t>Saldo pokok kredit masih terutang/outstanding.</t>
+  </si>
+  <si>
+    <t>Nilai penyesuaian PSAK kategori/komponen DMA sesuai definisi internal.</t>
+  </si>
+  <si>
+    <t>Nilai penyesuaian PSAK kategori/komponen ACC sesuai definisi internal.</t>
   </si>
 </sst>
 </file>
@@ -2594,6 +2594,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:J345"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2642,7 +2643,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>22</v>
       </c>
@@ -2662,10 +2663,10 @@
         <v>10</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>686</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>22</v>
       </c>
@@ -2685,7 +2686,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>22</v>
       </c>
@@ -2705,10 +2706,10 @@
         <v>10</v>
       </c>
       <c r="J4" t="s">
-        <v>573</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>22</v>
       </c>
@@ -2728,10 +2729,10 @@
         <v>10</v>
       </c>
       <c r="J5" t="s">
-        <v>574</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>22</v>
       </c>
@@ -2751,7 +2752,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>22</v>
       </c>
@@ -2771,7 +2772,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>22</v>
       </c>
@@ -2791,7 +2792,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>22</v>
       </c>
@@ -2811,7 +2812,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>22</v>
       </c>
@@ -2831,7 +2832,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>22</v>
       </c>
@@ -2851,7 +2852,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>22</v>
       </c>
@@ -2871,7 +2872,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>22</v>
       </c>
@@ -2891,7 +2892,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>22</v>
       </c>
@@ -2954,10 +2955,10 @@
         <v>10</v>
       </c>
       <c r="J16" t="s">
-        <v>681</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>22</v>
       </c>
@@ -2977,7 +2978,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>22</v>
       </c>
@@ -2997,7 +2998,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>22</v>
       </c>
@@ -3017,7 +3018,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>22</v>
       </c>
@@ -3037,7 +3038,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>22</v>
       </c>
@@ -3057,7 +3058,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>22</v>
       </c>
@@ -3077,7 +3078,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>22</v>
       </c>
@@ -3097,7 +3098,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>22</v>
       </c>
@@ -3117,7 +3118,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
         <v>22</v>
       </c>
@@ -3137,7 +3138,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>22</v>
       </c>
@@ -3157,7 +3158,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>22</v>
       </c>
@@ -3177,7 +3178,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>22</v>
       </c>
@@ -3197,7 +3198,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>22</v>
       </c>
@@ -3220,7 +3221,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>22</v>
       </c>
@@ -3243,7 +3244,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>22</v>
       </c>
@@ -3263,7 +3264,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>22</v>
       </c>
@@ -3283,7 +3284,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
         <v>22</v>
       </c>
@@ -3303,7 +3304,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
         <v>22</v>
       </c>
@@ -3323,7 +3324,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
         <v>22</v>
       </c>
@@ -3343,7 +3344,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
         <v>22</v>
       </c>
@@ -3363,7 +3364,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
         <v>22</v>
       </c>
@@ -3383,7 +3384,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
         <v>22</v>
       </c>
@@ -3426,7 +3427,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:10" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>23</v>
       </c>
@@ -3446,7 +3447,7 @@
         <v>10</v>
       </c>
       <c r="J40" s="5" t="s">
-        <v>685</v>
+        <v>680</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -3472,7 +3473,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
         <v>23</v>
       </c>
@@ -3489,10 +3490,10 @@
         <v>10</v>
       </c>
       <c r="J42" t="s">
-        <v>697</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
         <v>23</v>
       </c>
@@ -3512,7 +3513,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
         <v>23</v>
       </c>
@@ -3529,10 +3530,10 @@
         <v>10</v>
       </c>
       <c r="J44" t="s">
-        <v>575</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
         <v>23</v>
       </c>
@@ -3552,7 +3553,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
         <v>23</v>
       </c>
@@ -3572,7 +3573,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
         <v>23</v>
       </c>
@@ -3592,7 +3593,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
         <v>23</v>
       </c>
@@ -3612,7 +3613,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
         <v>23</v>
       </c>
@@ -3632,7 +3633,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
         <v>23</v>
       </c>
@@ -3652,7 +3653,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
         <v>23</v>
       </c>
@@ -3672,7 +3673,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
         <v>23</v>
       </c>
@@ -3692,7 +3693,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
         <v>23</v>
       </c>
@@ -3712,10 +3713,10 @@
         <v>406</v>
       </c>
       <c r="J53" t="s">
-        <v>698</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
         <v>23</v>
       </c>
@@ -3732,10 +3733,10 @@
         <v>10</v>
       </c>
       <c r="J54" t="s">
-        <v>696</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
         <v>23</v>
       </c>
@@ -3752,10 +3753,10 @@
         <v>10</v>
       </c>
       <c r="J55" t="s">
-        <v>699</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
         <v>23</v>
       </c>
@@ -3775,7 +3776,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
         <v>23</v>
       </c>
@@ -3795,7 +3796,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" s="4" t="s">
         <v>23</v>
       </c>
@@ -3815,7 +3816,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" s="4" t="s">
         <v>23</v>
       </c>
@@ -3835,7 +3836,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60" s="4" t="s">
         <v>23</v>
       </c>
@@ -3855,7 +3856,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
         <v>23</v>
       </c>
@@ -3875,7 +3876,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" s="4" t="s">
         <v>23</v>
       </c>
@@ -3895,7 +3896,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="63" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" s="4" t="s">
         <v>23</v>
       </c>
@@ -3915,7 +3916,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="64" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" s="4" t="s">
         <v>23</v>
       </c>
@@ -3935,7 +3936,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" s="4" t="s">
         <v>23</v>
       </c>
@@ -3952,10 +3953,10 @@
         <v>10</v>
       </c>
       <c r="J65" t="s">
-        <v>576</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" s="4" t="s">
         <v>23</v>
       </c>
@@ -3972,10 +3973,10 @@
         <v>10</v>
       </c>
       <c r="J66" t="s">
-        <v>577</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" s="4" t="s">
         <v>23</v>
       </c>
@@ -3992,7 +3993,7 @@
         <v>10</v>
       </c>
       <c r="J67" t="s">
-        <v>578</v>
+        <v>573</v>
       </c>
     </row>
     <row r="68" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4015,10 +4016,10 @@
         <v>10</v>
       </c>
       <c r="J68" t="s">
-        <v>579</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69" s="4" t="s">
         <v>23</v>
       </c>
@@ -4035,10 +4036,10 @@
         <v>10</v>
       </c>
       <c r="J69" t="s">
-        <v>580</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A70" s="4" t="s">
         <v>23</v>
       </c>
@@ -4055,10 +4056,10 @@
         <v>10</v>
       </c>
       <c r="J70" t="s">
-        <v>581</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71" s="4" t="s">
         <v>23</v>
       </c>
@@ -4078,7 +4079,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="72" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" s="4" t="s">
         <v>23</v>
       </c>
@@ -4098,7 +4099,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="73" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73" s="4" t="s">
         <v>23</v>
       </c>
@@ -4115,10 +4116,10 @@
         <v>10</v>
       </c>
       <c r="J73" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="74" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A74" s="4" t="s">
         <v>23</v>
       </c>
@@ -4138,7 +4139,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="75" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A75" s="4" t="s">
         <v>23</v>
       </c>
@@ -4158,7 +4159,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="76" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76" s="4" t="s">
         <v>23</v>
       </c>
@@ -4178,7 +4179,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="77" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A77" s="4" t="s">
         <v>23</v>
       </c>
@@ -4198,7 +4199,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="78" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A78" s="4" t="s">
         <v>23</v>
       </c>
@@ -4215,10 +4216,10 @@
         <v>10</v>
       </c>
       <c r="J78" t="s">
-        <v>583</v>
-      </c>
-    </row>
-    <row r="79" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A79" s="4" t="s">
         <v>23</v>
       </c>
@@ -4235,10 +4236,10 @@
         <v>10</v>
       </c>
       <c r="J79" t="s">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="80" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A80" s="4" t="s">
         <v>23</v>
       </c>
@@ -4255,10 +4256,10 @@
         <v>10</v>
       </c>
       <c r="J80" t="s">
-        <v>586</v>
-      </c>
-    </row>
-    <row r="81" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A81" s="4" t="s">
         <v>23</v>
       </c>
@@ -4275,10 +4276,10 @@
         <v>10</v>
       </c>
       <c r="J81" t="s">
-        <v>585</v>
-      </c>
-    </row>
-    <row r="82" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A82" s="4" t="s">
         <v>23</v>
       </c>
@@ -4295,10 +4296,10 @@
         <v>10</v>
       </c>
       <c r="J82" t="s">
-        <v>587</v>
-      </c>
-    </row>
-    <row r="83" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A83" s="4" t="s">
         <v>23</v>
       </c>
@@ -4316,7 +4317,7 @@
       </c>
       <c r="J83"/>
     </row>
-    <row r="84" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84" s="4" t="s">
         <v>23</v>
       </c>
@@ -4334,7 +4335,7 @@
       </c>
       <c r="J84"/>
     </row>
-    <row r="85" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A85" s="4" t="s">
         <v>23</v>
       </c>
@@ -4351,10 +4352,10 @@
         <v>10</v>
       </c>
       <c r="J85" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="86" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A86" s="4" t="s">
         <v>23</v>
       </c>
@@ -4372,7 +4373,7 @@
       </c>
       <c r="J86"/>
     </row>
-    <row r="87" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A87" s="4" t="s">
         <v>23</v>
       </c>
@@ -4390,7 +4391,7 @@
       </c>
       <c r="J87"/>
     </row>
-    <row r="88" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A88" s="4" t="s">
         <v>23</v>
       </c>
@@ -4408,7 +4409,7 @@
       </c>
       <c r="J88"/>
     </row>
-    <row r="89" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A89" s="4" t="s">
         <v>23</v>
       </c>
@@ -4425,10 +4426,10 @@
         <v>10</v>
       </c>
       <c r="J89" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="90" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A90" s="4" t="s">
         <v>23</v>
       </c>
@@ -4445,10 +4446,10 @@
         <v>10</v>
       </c>
       <c r="J90" t="s">
-        <v>590</v>
-      </c>
-    </row>
-    <row r="91" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A91" s="4" t="s">
         <v>23</v>
       </c>
@@ -4465,10 +4466,10 @@
         <v>10</v>
       </c>
       <c r="J91" t="s">
-        <v>591</v>
-      </c>
-    </row>
-    <row r="92" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A92" s="4" t="s">
         <v>23</v>
       </c>
@@ -4485,10 +4486,10 @@
         <v>10</v>
       </c>
       <c r="J92" t="s">
-        <v>592</v>
-      </c>
-    </row>
-    <row r="93" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A93" s="4" t="s">
         <v>23</v>
       </c>
@@ -4505,10 +4506,10 @@
         <v>10</v>
       </c>
       <c r="J93" t="s">
-        <v>593</v>
-      </c>
-    </row>
-    <row r="94" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A94" s="4" t="s">
         <v>23</v>
       </c>
@@ -4525,10 +4526,10 @@
         <v>10</v>
       </c>
       <c r="J94" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="95" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A95" s="4" t="s">
         <v>23</v>
       </c>
@@ -4545,10 +4546,10 @@
         <v>10</v>
       </c>
       <c r="J95" t="s">
-        <v>595</v>
-      </c>
-    </row>
-    <row r="96" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A96" s="4" t="s">
         <v>23</v>
       </c>
@@ -4565,10 +4566,10 @@
         <v>10</v>
       </c>
       <c r="J96" t="s">
-        <v>596</v>
-      </c>
-    </row>
-    <row r="97" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A97" s="4" t="s">
         <v>23</v>
       </c>
@@ -4588,7 +4589,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="98" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A98" s="4" t="s">
         <v>23</v>
       </c>
@@ -4605,10 +4606,10 @@
         <v>10</v>
       </c>
       <c r="J98" t="s">
-        <v>597</v>
-      </c>
-    </row>
-    <row r="99" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A99" s="4" t="s">
         <v>23</v>
       </c>
@@ -4625,10 +4626,10 @@
         <v>10</v>
       </c>
       <c r="J99" t="s">
-        <v>598</v>
-      </c>
-    </row>
-    <row r="100" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A100" s="4" t="s">
         <v>23</v>
       </c>
@@ -4648,7 +4649,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="101" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A101" s="4" t="s">
         <v>23</v>
       </c>
@@ -4668,7 +4669,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="102" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A102" s="4" t="s">
         <v>23</v>
       </c>
@@ -4686,7 +4687,7 @@
       </c>
       <c r="J102"/>
     </row>
-    <row r="103" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A103" s="4" t="s">
         <v>23</v>
       </c>
@@ -4706,7 +4707,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="104" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A104" s="4" t="s">
         <v>23</v>
       </c>
@@ -4769,7 +4770,7 @@
         <v>10</v>
       </c>
       <c r="J106" t="s">
-        <v>701</v>
+        <v>696</v>
       </c>
     </row>
     <row r="107" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -4792,10 +4793,10 @@
         <v>10</v>
       </c>
       <c r="J107" t="s">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="108" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A108" s="4" t="s">
         <v>23</v>
       </c>
@@ -4815,7 +4816,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="109" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A109" s="4" t="s">
         <v>23</v>
       </c>
@@ -4833,7 +4834,7 @@
       </c>
       <c r="J109"/>
     </row>
-    <row r="110" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A110" s="4" t="s">
         <v>23</v>
       </c>
@@ -4851,7 +4852,7 @@
       </c>
       <c r="J110"/>
     </row>
-    <row r="111" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A111" s="4" t="s">
         <v>23</v>
       </c>
@@ -4868,10 +4869,10 @@
         <v>10</v>
       </c>
       <c r="J111" t="s">
-        <v>601</v>
-      </c>
-    </row>
-    <row r="112" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A112" s="4" t="s">
         <v>23</v>
       </c>
@@ -4888,10 +4889,10 @@
         <v>10</v>
       </c>
       <c r="J112" t="s">
-        <v>599</v>
-      </c>
-    </row>
-    <row r="113" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A113" s="4" t="s">
         <v>23</v>
       </c>
@@ -4908,10 +4909,10 @@
         <v>10</v>
       </c>
       <c r="J113" t="s">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="114" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A114" s="4" t="s">
         <v>23</v>
       </c>
@@ -4928,10 +4929,10 @@
         <v>10</v>
       </c>
       <c r="J114" t="s">
-        <v>583</v>
-      </c>
-    </row>
-    <row r="115" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A115" s="4" t="s">
         <v>23</v>
       </c>
@@ -4948,10 +4949,10 @@
         <v>10</v>
       </c>
       <c r="J115" t="s">
-        <v>602</v>
-      </c>
-    </row>
-    <row r="116" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A116" s="4" t="s">
         <v>23</v>
       </c>
@@ -4968,10 +4969,10 @@
         <v>10</v>
       </c>
       <c r="J116" t="s">
-        <v>603</v>
-      </c>
-    </row>
-    <row r="117" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="117" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A117" s="4" t="s">
         <v>23</v>
       </c>
@@ -4988,10 +4989,10 @@
         <v>10</v>
       </c>
       <c r="J117" t="s">
-        <v>604</v>
-      </c>
-    </row>
-    <row r="118" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="118" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A118" s="4" t="s">
         <v>23</v>
       </c>
@@ -5008,10 +5009,10 @@
         <v>10</v>
       </c>
       <c r="J118" t="s">
-        <v>605</v>
-      </c>
-    </row>
-    <row r="119" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A119" s="4" t="s">
         <v>23</v>
       </c>
@@ -5028,10 +5029,10 @@
         <v>10</v>
       </c>
       <c r="J119" t="s">
-        <v>606</v>
-      </c>
-    </row>
-    <row r="120" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A120" s="4" t="s">
         <v>23</v>
       </c>
@@ -5048,10 +5049,10 @@
         <v>10</v>
       </c>
       <c r="J120" t="s">
-        <v>607</v>
-      </c>
-    </row>
-    <row r="121" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A121" s="4" t="s">
         <v>23</v>
       </c>
@@ -5068,10 +5069,10 @@
         <v>10</v>
       </c>
       <c r="J121" t="s">
-        <v>608</v>
-      </c>
-    </row>
-    <row r="122" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A122" s="4" t="s">
         <v>23</v>
       </c>
@@ -5088,10 +5089,10 @@
         <v>10</v>
       </c>
       <c r="J122" t="s">
-        <v>611</v>
-      </c>
-    </row>
-    <row r="123" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A123" s="4" t="s">
         <v>23</v>
       </c>
@@ -5108,10 +5109,10 @@
         <v>10</v>
       </c>
       <c r="J123" t="s">
-        <v>610</v>
-      </c>
-    </row>
-    <row r="124" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A124" s="4" t="s">
         <v>23</v>
       </c>
@@ -5128,10 +5129,10 @@
         <v>10</v>
       </c>
       <c r="J124" t="s">
-        <v>609</v>
-      </c>
-    </row>
-    <row r="125" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A125" s="4" t="s">
         <v>23</v>
       </c>
@@ -5148,10 +5149,10 @@
         <v>10</v>
       </c>
       <c r="J125" t="s">
-        <v>612</v>
-      </c>
-    </row>
-    <row r="126" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A126" s="4" t="s">
         <v>23</v>
       </c>
@@ -5168,10 +5169,10 @@
         <v>10</v>
       </c>
       <c r="J126" t="s">
-        <v>613</v>
-      </c>
-    </row>
-    <row r="127" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A127" s="4" t="s">
         <v>23</v>
       </c>
@@ -5188,10 +5189,10 @@
         <v>10</v>
       </c>
       <c r="J127" t="s">
-        <v>621</v>
-      </c>
-    </row>
-    <row r="128" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A128" s="4" t="s">
         <v>23</v>
       </c>
@@ -5208,10 +5209,10 @@
         <v>10</v>
       </c>
       <c r="J128" t="s">
-        <v>622</v>
-      </c>
-    </row>
-    <row r="129" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="129" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A129" s="4" t="s">
         <v>23</v>
       </c>
@@ -5228,10 +5229,10 @@
         <v>10</v>
       </c>
       <c r="J129" t="s">
-        <v>623</v>
-      </c>
-    </row>
-    <row r="130" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A130" s="4" t="s">
         <v>23</v>
       </c>
@@ -5248,10 +5249,10 @@
         <v>10</v>
       </c>
       <c r="J130" t="s">
-        <v>624</v>
-      </c>
-    </row>
-    <row r="131" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="131" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A131" s="4" t="s">
         <v>23</v>
       </c>
@@ -5268,10 +5269,10 @@
         <v>10</v>
       </c>
       <c r="J131" t="s">
-        <v>625</v>
-      </c>
-    </row>
-    <row r="132" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="132" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A132" s="4" t="s">
         <v>23</v>
       </c>
@@ -5288,10 +5289,10 @@
         <v>10</v>
       </c>
       <c r="J132" t="s">
-        <v>626</v>
-      </c>
-    </row>
-    <row r="133" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="133" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A133" s="4" t="s">
         <v>23</v>
       </c>
@@ -5308,10 +5309,10 @@
         <v>10</v>
       </c>
       <c r="J133" t="s">
-        <v>627</v>
-      </c>
-    </row>
-    <row r="134" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="134" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A134" s="4" t="s">
         <v>23</v>
       </c>
@@ -5328,10 +5329,10 @@
         <v>10</v>
       </c>
       <c r="J134" t="s">
-        <v>628</v>
-      </c>
-    </row>
-    <row r="135" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="135" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A135" s="4" t="s">
         <v>23</v>
       </c>
@@ -5348,10 +5349,10 @@
         <v>10</v>
       </c>
       <c r="J135" t="s">
-        <v>629</v>
-      </c>
-    </row>
-    <row r="136" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="136" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A136" s="4" t="s">
         <v>23</v>
       </c>
@@ -5368,10 +5369,10 @@
         <v>10</v>
       </c>
       <c r="J136" t="s">
-        <v>631</v>
-      </c>
-    </row>
-    <row r="137" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="137" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A137" s="4" t="s">
         <v>23</v>
       </c>
@@ -5388,10 +5389,10 @@
         <v>10</v>
       </c>
       <c r="J137" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="138" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="138" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A138" s="4" t="s">
         <v>23</v>
       </c>
@@ -5408,10 +5409,10 @@
         <v>10</v>
       </c>
       <c r="J138" t="s">
-        <v>688</v>
-      </c>
-    </row>
-    <row r="139" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="139" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A139" s="4" t="s">
         <v>23</v>
       </c>
@@ -5428,10 +5429,10 @@
         <v>10</v>
       </c>
       <c r="J139" t="s">
-        <v>689</v>
-      </c>
-    </row>
-    <row r="140" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="140" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A140" s="4" t="s">
         <v>23</v>
       </c>
@@ -5448,10 +5449,10 @@
         <v>10</v>
       </c>
       <c r="J140" t="s">
-        <v>632</v>
-      </c>
-    </row>
-    <row r="141" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="141" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A141" s="4" t="s">
         <v>27</v>
       </c>
@@ -5471,10 +5472,10 @@
         <v>10</v>
       </c>
       <c r="J141" s="5" t="s">
-        <v>682</v>
-      </c>
-    </row>
-    <row r="142" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="142" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A142" s="4" t="s">
         <v>27</v>
       </c>
@@ -5491,10 +5492,10 @@
         <v>10</v>
       </c>
       <c r="J142" t="s">
-        <v>633</v>
-      </c>
-    </row>
-    <row r="143" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="143" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A143" s="4" t="s">
         <v>27</v>
       </c>
@@ -5514,10 +5515,10 @@
         <v>10</v>
       </c>
       <c r="J143" t="s">
-        <v>690</v>
-      </c>
-    </row>
-    <row r="144" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="144" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A144" s="4" t="s">
         <v>27</v>
       </c>
@@ -5534,10 +5535,10 @@
         <v>10</v>
       </c>
       <c r="J144" t="s">
-        <v>696</v>
-      </c>
-    </row>
-    <row r="145" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="145" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A145" s="4" t="s">
         <v>27</v>
       </c>
@@ -5554,10 +5555,10 @@
         <v>10</v>
       </c>
       <c r="J145" t="s">
-        <v>699</v>
-      </c>
-    </row>
-    <row r="146" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="146" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A146" s="4" t="s">
         <v>27</v>
       </c>
@@ -5574,10 +5575,10 @@
         <v>10</v>
       </c>
       <c r="J146" t="s">
-        <v>634</v>
-      </c>
-    </row>
-    <row r="147" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="147" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A147" s="4" t="s">
         <v>27</v>
       </c>
@@ -5594,10 +5595,10 @@
         <v>10</v>
       </c>
       <c r="J147" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="148" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="148" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A148" s="4" t="s">
         <v>27</v>
       </c>
@@ -5614,10 +5615,10 @@
         <v>10</v>
       </c>
       <c r="J148" t="s">
-        <v>636</v>
-      </c>
-    </row>
-    <row r="149" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="149" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A149" s="4" t="s">
         <v>27</v>
       </c>
@@ -5634,10 +5635,10 @@
         <v>10</v>
       </c>
       <c r="J149" t="s">
-        <v>638</v>
-      </c>
-    </row>
-    <row r="150" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="150" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A150" s="4" t="s">
         <v>27</v>
       </c>
@@ -5654,10 +5655,10 @@
         <v>10</v>
       </c>
       <c r="J150" t="s">
-        <v>637</v>
-      </c>
-    </row>
-    <row r="151" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="151" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A151" s="4" t="s">
         <v>27</v>
       </c>
@@ -5674,10 +5675,10 @@
         <v>10</v>
       </c>
       <c r="J151" t="s">
-        <v>691</v>
-      </c>
-    </row>
-    <row r="152" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="152" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A152" s="4" t="s">
         <v>27</v>
       </c>
@@ -5697,7 +5698,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="153" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A153" s="4" t="s">
         <v>27</v>
       </c>
@@ -5717,7 +5718,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="154" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A154" s="4" t="s">
         <v>27</v>
       </c>
@@ -5737,7 +5738,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="155" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A155" s="4" t="s">
         <v>27</v>
       </c>
@@ -5754,10 +5755,10 @@
         <v>10</v>
       </c>
       <c r="J155" t="s">
-        <v>597</v>
-      </c>
-    </row>
-    <row r="156" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="156" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A156" s="4" t="s">
         <v>27</v>
       </c>
@@ -5774,10 +5775,10 @@
         <v>10</v>
       </c>
       <c r="J156" t="s">
-        <v>601</v>
-      </c>
-    </row>
-    <row r="157" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="157" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A157" s="4" t="s">
         <v>27</v>
       </c>
@@ -5794,10 +5795,10 @@
         <v>10</v>
       </c>
       <c r="J157" t="s">
-        <v>599</v>
-      </c>
-    </row>
-    <row r="158" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="158" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A158" s="4" t="s">
         <v>27</v>
       </c>
@@ -5814,10 +5815,10 @@
         <v>10</v>
       </c>
       <c r="J158" t="s">
-        <v>620</v>
-      </c>
-    </row>
-    <row r="159" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="159" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A159" s="4" t="s">
         <v>27</v>
       </c>
@@ -5834,10 +5835,10 @@
         <v>10</v>
       </c>
       <c r="J159" t="s">
-        <v>619</v>
-      </c>
-    </row>
-    <row r="160" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="160" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A160" s="4" t="s">
         <v>27</v>
       </c>
@@ -5854,10 +5855,10 @@
         <v>10</v>
       </c>
       <c r="J160" t="s">
-        <v>618</v>
-      </c>
-    </row>
-    <row r="161" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="161" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A161" s="4" t="s">
         <v>27</v>
       </c>
@@ -5874,10 +5875,10 @@
         <v>10</v>
       </c>
       <c r="J161" t="s">
-        <v>614</v>
-      </c>
-    </row>
-    <row r="162" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="162" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A162" s="4" t="s">
         <v>27</v>
       </c>
@@ -5894,10 +5895,10 @@
         <v>10</v>
       </c>
       <c r="J162" t="s">
-        <v>615</v>
-      </c>
-    </row>
-    <row r="163" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="163" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A163" s="4" t="s">
         <v>27</v>
       </c>
@@ -5917,7 +5918,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="164" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A164" s="4" t="s">
         <v>27</v>
       </c>
@@ -5937,7 +5938,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="165" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A165" s="4" t="s">
         <v>27</v>
       </c>
@@ -5957,7 +5958,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="166" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A166" s="4" t="s">
         <v>27</v>
       </c>
@@ -5977,7 +5978,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="167" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A167" s="4" t="s">
         <v>27</v>
       </c>
@@ -5997,7 +5998,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="168" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A168" s="4" t="s">
         <v>27</v>
       </c>
@@ -6017,7 +6018,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="169" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A169" s="4" t="s">
         <v>27</v>
       </c>
@@ -6040,7 +6041,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="170" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A170" s="4" t="s">
         <v>27</v>
       </c>
@@ -6060,7 +6061,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="171" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A171" s="4" t="s">
         <v>27</v>
       </c>
@@ -6080,7 +6081,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="172" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A172" s="4" t="s">
         <v>27</v>
       </c>
@@ -6097,10 +6098,10 @@
         <v>10</v>
       </c>
       <c r="J172" t="s">
-        <v>616</v>
-      </c>
-    </row>
-    <row r="173" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="173" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A173" s="4" t="s">
         <v>27</v>
       </c>
@@ -6117,10 +6118,10 @@
         <v>10</v>
       </c>
       <c r="J173" t="s">
-        <v>617</v>
-      </c>
-    </row>
-    <row r="174" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="174" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A174" s="4" t="s">
         <v>27</v>
       </c>
@@ -6137,10 +6138,10 @@
         <v>10</v>
       </c>
       <c r="J174" t="s">
-        <v>639</v>
-      </c>
-    </row>
-    <row r="175" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="175" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A175" s="4" t="s">
         <v>27</v>
       </c>
@@ -6157,10 +6158,10 @@
         <v>10</v>
       </c>
       <c r="J175" t="s">
-        <v>640</v>
-      </c>
-    </row>
-    <row r="176" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="176" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A176" s="4" t="s">
         <v>27</v>
       </c>
@@ -6177,10 +6178,10 @@
         <v>10</v>
       </c>
       <c r="J176" t="s">
-        <v>641</v>
-      </c>
-    </row>
-    <row r="177" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="177" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A177" s="4" t="s">
         <v>27</v>
       </c>
@@ -6197,10 +6198,10 @@
         <v>10</v>
       </c>
       <c r="J177" t="s">
-        <v>642</v>
-      </c>
-    </row>
-    <row r="178" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="178" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A178" s="4" t="s">
         <v>27</v>
       </c>
@@ -6217,10 +6218,10 @@
         <v>10</v>
       </c>
       <c r="J178" t="s">
-        <v>642</v>
-      </c>
-    </row>
-    <row r="179" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="179" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A179" s="4" t="s">
         <v>27</v>
       </c>
@@ -6237,10 +6238,10 @@
         <v>10</v>
       </c>
       <c r="J179" t="s">
-        <v>643</v>
-      </c>
-    </row>
-    <row r="180" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="180" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A180" s="4" t="s">
         <v>27</v>
       </c>
@@ -6257,7 +6258,7 @@
         <v>10</v>
       </c>
       <c r="J180" t="s">
-        <v>644</v>
+        <v>639</v>
       </c>
     </row>
     <row r="181" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6280,7 +6281,7 @@
         <v>10</v>
       </c>
       <c r="J181" t="s">
-        <v>645</v>
+        <v>640</v>
       </c>
     </row>
     <row r="182" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6303,7 +6304,7 @@
         <v>10</v>
       </c>
       <c r="J182" t="s">
-        <v>646</v>
+        <v>641</v>
       </c>
     </row>
     <row r="183" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6326,7 +6327,7 @@
         <v>10</v>
       </c>
       <c r="J183" t="s">
-        <v>647</v>
+        <v>642</v>
       </c>
     </row>
     <row r="184" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6349,7 +6350,7 @@
         <v>10</v>
       </c>
       <c r="J184" t="s">
-        <v>648</v>
+        <v>643</v>
       </c>
     </row>
     <row r="185" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6372,10 +6373,10 @@
         <v>10</v>
       </c>
       <c r="J185" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="186" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="186" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A186" s="4" t="s">
         <v>27</v>
       </c>
@@ -6392,10 +6393,10 @@
         <v>10</v>
       </c>
       <c r="J186" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="187" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="187" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A187" s="4" t="s">
         <v>27</v>
       </c>
@@ -6412,10 +6413,10 @@
         <v>10</v>
       </c>
       <c r="J187" t="s">
-        <v>651</v>
-      </c>
-    </row>
-    <row r="188" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="188" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A188" s="4" t="s">
         <v>27</v>
       </c>
@@ -6432,10 +6433,10 @@
         <v>10</v>
       </c>
       <c r="J188" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="189" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="189" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A189" s="4" t="s">
         <v>27</v>
       </c>
@@ -6455,7 +6456,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="190" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A190" s="4" t="s">
         <v>27</v>
       </c>
@@ -6475,7 +6476,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="191" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A191" s="4" t="s">
         <v>27</v>
       </c>
@@ -6492,10 +6493,10 @@
         <v>10</v>
       </c>
       <c r="J191" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="192" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="192" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A192" s="4" t="s">
         <v>27</v>
       </c>
@@ -6512,10 +6513,10 @@
         <v>10</v>
       </c>
       <c r="J192" t="s">
-        <v>654</v>
-      </c>
-    </row>
-    <row r="193" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="193" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A193" s="4" t="s">
         <v>27</v>
       </c>
@@ -6532,10 +6533,10 @@
         <v>10</v>
       </c>
       <c r="J193" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="194" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="194" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A194" s="4" t="s">
         <v>27</v>
       </c>
@@ -6552,10 +6553,10 @@
         <v>10</v>
       </c>
       <c r="J194" t="s">
-        <v>656</v>
-      </c>
-    </row>
-    <row r="195" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="195" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A195" s="4" t="s">
         <v>27</v>
       </c>
@@ -6572,10 +6573,10 @@
         <v>10</v>
       </c>
       <c r="J195" t="s">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="196" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="196" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A196" s="4" t="s">
         <v>27</v>
       </c>
@@ -6592,10 +6593,10 @@
         <v>10</v>
       </c>
       <c r="J196" t="s">
-        <v>611</v>
-      </c>
-    </row>
-    <row r="197" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="197" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A197" s="4" t="s">
         <v>27</v>
       </c>
@@ -6612,10 +6613,10 @@
         <v>10</v>
       </c>
       <c r="J197" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="198" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="198" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A198" s="4" t="s">
         <v>27</v>
       </c>
@@ -6632,10 +6633,10 @@
         <v>10</v>
       </c>
       <c r="J198" t="s">
-        <v>659</v>
-      </c>
-    </row>
-    <row r="199" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="199" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A199" s="4" t="s">
         <v>27</v>
       </c>
@@ -6652,10 +6653,10 @@
         <v>10</v>
       </c>
       <c r="J199" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="200" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="200" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A200" s="4" t="s">
         <v>27</v>
       </c>
@@ -6672,10 +6673,10 @@
         <v>10</v>
       </c>
       <c r="J200" t="s">
-        <v>661</v>
-      </c>
-    </row>
-    <row r="201" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="201" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A201" s="4" t="s">
         <v>27</v>
       </c>
@@ -6692,10 +6693,10 @@
         <v>10</v>
       </c>
       <c r="J201" t="s">
-        <v>662</v>
-      </c>
-    </row>
-    <row r="202" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="202" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A202" s="4" t="s">
         <v>27</v>
       </c>
@@ -6712,10 +6713,10 @@
         <v>10</v>
       </c>
       <c r="J202" t="s">
-        <v>663</v>
-      </c>
-    </row>
-    <row r="203" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="203" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A203" s="4" t="s">
         <v>27</v>
       </c>
@@ -6732,7 +6733,7 @@
         <v>10</v>
       </c>
       <c r="J203" t="s">
-        <v>664</v>
+        <v>659</v>
       </c>
     </row>
     <row r="204" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6755,7 +6756,7 @@
         <v>10</v>
       </c>
       <c r="J204" t="s">
-        <v>665</v>
+        <v>660</v>
       </c>
     </row>
     <row r="205" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6778,7 +6779,7 @@
         <v>10</v>
       </c>
       <c r="J205" t="s">
-        <v>666</v>
+        <v>661</v>
       </c>
     </row>
     <row r="206" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6801,7 +6802,7 @@
         <v>10</v>
       </c>
       <c r="J206" t="s">
-        <v>667</v>
+        <v>662</v>
       </c>
     </row>
     <row r="207" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6824,7 +6825,7 @@
         <v>10</v>
       </c>
       <c r="J207" t="s">
-        <v>668</v>
+        <v>663</v>
       </c>
     </row>
     <row r="208" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -6965,7 +6966,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="214" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A214" s="4" t="s">
         <v>27</v>
       </c>
@@ -6985,7 +6986,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="215" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A215" s="4" t="s">
         <v>27</v>
       </c>
@@ -7005,7 +7006,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="216" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A216" s="4" t="s">
         <v>27</v>
       </c>
@@ -7094,7 +7095,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="220" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A220" s="4" t="s">
         <v>27</v>
       </c>
@@ -7114,7 +7115,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="221" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A221" s="4" t="s">
         <v>27</v>
       </c>
@@ -7134,7 +7135,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="222" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A222" s="4" t="s">
         <v>27</v>
       </c>
@@ -7154,7 +7155,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="223" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A223" s="4" t="s">
         <v>27</v>
       </c>
@@ -7174,7 +7175,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="224" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A224" s="4" t="s">
         <v>27</v>
       </c>
@@ -7194,7 +7195,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="225" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A225" s="4" t="s">
         <v>27</v>
       </c>
@@ -7214,7 +7215,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="226" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A226" s="4" t="s">
         <v>27</v>
       </c>
@@ -7234,7 +7235,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="227" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A227" s="4" t="s">
         <v>27</v>
       </c>
@@ -7254,7 +7255,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="228" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A228" s="4" t="s">
         <v>27</v>
       </c>
@@ -7274,7 +7275,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="229" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A229" s="4" t="s">
         <v>27</v>
       </c>
@@ -7294,7 +7295,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="230" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A230" s="4" t="s">
         <v>27</v>
       </c>
@@ -7311,7 +7312,7 @@
         <v>10</v>
       </c>
       <c r="J230" s="5" t="s">
-        <v>692</v>
+        <v>687</v>
       </c>
     </row>
     <row r="231" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -7498,7 +7499,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="239" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A239" s="4" t="s">
         <v>27</v>
       </c>
@@ -7538,10 +7539,10 @@
         <v>10</v>
       </c>
       <c r="J240" s="5" t="s">
-        <v>488</v>
-      </c>
-    </row>
-    <row r="241" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="241" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A241" s="4" t="s">
         <v>27</v>
       </c>
@@ -7558,10 +7559,10 @@
         <v>10</v>
       </c>
       <c r="J241" s="5" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="242" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="242" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A242" s="4" t="s">
         <v>29</v>
       </c>
@@ -7581,10 +7582,10 @@
         <v>10</v>
       </c>
       <c r="J242" s="5" t="s">
-        <v>683</v>
-      </c>
-    </row>
-    <row r="243" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="243" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A243" s="4" t="s">
         <v>29</v>
       </c>
@@ -7601,10 +7602,10 @@
         <v>10</v>
       </c>
       <c r="J243" s="5" t="s">
-        <v>693</v>
-      </c>
-    </row>
-    <row r="244" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="244" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A244" s="4" t="s">
         <v>29</v>
       </c>
@@ -7621,10 +7622,10 @@
         <v>10</v>
       </c>
       <c r="J244" s="5" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="245" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="245" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A245" s="4" t="s">
         <v>29</v>
       </c>
@@ -7644,10 +7645,10 @@
         <v>10</v>
       </c>
       <c r="J245" s="5" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="246" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="246" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A246" s="4" t="s">
         <v>29</v>
       </c>
@@ -7664,10 +7665,10 @@
         <v>10</v>
       </c>
       <c r="J246" s="5" t="s">
-        <v>669</v>
-      </c>
-    </row>
-    <row r="247" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="247" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A247" s="4" t="s">
         <v>29</v>
       </c>
@@ -7684,10 +7685,10 @@
         <v>10</v>
       </c>
       <c r="J247" t="s">
-        <v>696</v>
-      </c>
-    </row>
-    <row r="248" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="248" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A248" s="4" t="s">
         <v>29</v>
       </c>
@@ -7704,10 +7705,10 @@
         <v>10</v>
       </c>
       <c r="J248" t="s">
-        <v>699</v>
-      </c>
-    </row>
-    <row r="249" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="249" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A249" s="4" t="s">
         <v>29</v>
       </c>
@@ -7724,10 +7725,10 @@
         <v>10</v>
       </c>
       <c r="J249" s="5" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="250" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="250" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A250" s="4" t="s">
         <v>29</v>
       </c>
@@ -7744,10 +7745,10 @@
         <v>10</v>
       </c>
       <c r="J250" s="5" t="s">
-        <v>493</v>
-      </c>
-    </row>
-    <row r="251" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="251" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A251" s="4" t="s">
         <v>29</v>
       </c>
@@ -7764,10 +7765,10 @@
         <v>10</v>
       </c>
       <c r="J251" s="5" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="252" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="252" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A252" s="4" t="s">
         <v>29</v>
       </c>
@@ -7784,10 +7785,10 @@
         <v>10</v>
       </c>
       <c r="J252" s="5" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="253" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="253" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A253" s="4" t="s">
         <v>29</v>
       </c>
@@ -7804,10 +7805,10 @@
         <v>10</v>
       </c>
       <c r="J253" s="5" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="254" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="254" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A254" s="4" t="s">
         <v>29</v>
       </c>
@@ -7824,10 +7825,10 @@
         <v>10</v>
       </c>
       <c r="J254" s="5" t="s">
-        <v>691</v>
-      </c>
-    </row>
-    <row r="255" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="255" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A255" s="4" t="s">
         <v>29</v>
       </c>
@@ -7844,10 +7845,10 @@
         <v>10</v>
       </c>
       <c r="J255" s="5" t="s">
-        <v>670</v>
-      </c>
-    </row>
-    <row r="256" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="256" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A256" s="4" t="s">
         <v>29</v>
       </c>
@@ -7864,10 +7865,10 @@
         <v>10</v>
       </c>
       <c r="J256" s="5" t="s">
-        <v>671</v>
-      </c>
-    </row>
-    <row r="257" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="257" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A257" s="4" t="s">
         <v>29</v>
       </c>
@@ -7884,10 +7885,10 @@
         <v>10</v>
       </c>
       <c r="J257" s="5" t="s">
-        <v>497</v>
-      </c>
-    </row>
-    <row r="258" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="258" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A258" s="4" t="s">
         <v>29</v>
       </c>
@@ -7904,10 +7905,10 @@
         <v>10</v>
       </c>
       <c r="J258" s="5" t="s">
-        <v>672</v>
-      </c>
-    </row>
-    <row r="259" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="259" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A259" s="4" t="s">
         <v>29</v>
       </c>
@@ -7924,10 +7925,10 @@
         <v>10</v>
       </c>
       <c r="J259" s="5" t="s">
-        <v>673</v>
-      </c>
-    </row>
-    <row r="260" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="260" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A260" s="4" t="s">
         <v>29</v>
       </c>
@@ -7944,10 +7945,10 @@
         <v>10</v>
       </c>
       <c r="J260" s="5" t="s">
-        <v>694</v>
-      </c>
-    </row>
-    <row r="261" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="261" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A261" s="4" t="s">
         <v>29</v>
       </c>
@@ -7964,10 +7965,10 @@
         <v>10</v>
       </c>
       <c r="J261" s="5" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="262" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="262" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A262" s="4" t="s">
         <v>29</v>
       </c>
@@ -7984,10 +7985,10 @@
         <v>10</v>
       </c>
       <c r="J262" s="5" t="s">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="263" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="263" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A263" s="4" t="s">
         <v>29</v>
       </c>
@@ -8004,10 +8005,10 @@
         <v>10</v>
       </c>
       <c r="J263" s="5" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="264" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="264" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A264" s="4" t="s">
         <v>29</v>
       </c>
@@ -8024,10 +8025,10 @@
         <v>10</v>
       </c>
       <c r="J264" s="5" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="265" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="265" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A265" s="4" t="s">
         <v>29</v>
       </c>
@@ -8044,10 +8045,10 @@
         <v>10</v>
       </c>
       <c r="J265" s="5" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="266" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="266" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A266" s="4" t="s">
         <v>29</v>
       </c>
@@ -8064,10 +8065,10 @@
         <v>10</v>
       </c>
       <c r="J266" s="5" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="267" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="267" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A267" s="4" t="s">
         <v>29</v>
       </c>
@@ -8084,10 +8085,10 @@
         <v>10</v>
       </c>
       <c r="J267" s="5" t="s">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="268" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="268" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A268" s="4" t="s">
         <v>29</v>
       </c>
@@ -8104,10 +8105,10 @@
         <v>10</v>
       </c>
       <c r="J268" s="5" t="s">
-        <v>505</v>
-      </c>
-    </row>
-    <row r="269" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="269" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A269" s="4" t="s">
         <v>29</v>
       </c>
@@ -8124,10 +8125,10 @@
         <v>10</v>
       </c>
       <c r="J269" s="5" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="270" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="270" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A270" s="4" t="s">
         <v>29</v>
       </c>
@@ -8144,10 +8145,10 @@
         <v>10</v>
       </c>
       <c r="J270" s="5" t="s">
-        <v>507</v>
-      </c>
-    </row>
-    <row r="271" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="271" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A271" s="4" t="s">
         <v>29</v>
       </c>
@@ -8164,10 +8165,10 @@
         <v>10</v>
       </c>
       <c r="J271" s="5" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="272" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="272" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A272" s="4" t="s">
         <v>29</v>
       </c>
@@ -8184,10 +8185,10 @@
         <v>10</v>
       </c>
       <c r="J272" s="5" t="s">
-        <v>509</v>
-      </c>
-    </row>
-    <row r="273" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="273" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A273" s="4" t="s">
         <v>29</v>
       </c>
@@ -8204,10 +8205,10 @@
         <v>10</v>
       </c>
       <c r="J273" s="5" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="274" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="274" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A274" s="4" t="s">
         <v>29</v>
       </c>
@@ -8224,10 +8225,10 @@
         <v>10</v>
       </c>
       <c r="J274" s="5" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="275" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="275" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A275" s="4" t="s">
         <v>29</v>
       </c>
@@ -8244,10 +8245,10 @@
         <v>10</v>
       </c>
       <c r="J275" s="5" t="s">
-        <v>512</v>
-      </c>
-    </row>
-    <row r="276" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="276" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A276" s="4" t="s">
         <v>29</v>
       </c>
@@ -8264,10 +8265,10 @@
         <v>10</v>
       </c>
       <c r="J276" s="5" t="s">
-        <v>513</v>
-      </c>
-    </row>
-    <row r="277" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="277" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A277" s="4" t="s">
         <v>29</v>
       </c>
@@ -8284,10 +8285,10 @@
         <v>10</v>
       </c>
       <c r="J277" s="5" t="s">
-        <v>514</v>
-      </c>
-    </row>
-    <row r="278" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="278" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A278" s="4" t="s">
         <v>29</v>
       </c>
@@ -8304,10 +8305,10 @@
         <v>10</v>
       </c>
       <c r="J278" s="5" t="s">
-        <v>674</v>
-      </c>
-    </row>
-    <row r="279" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="279" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A279" s="4" t="s">
         <v>29</v>
       </c>
@@ -8324,10 +8325,10 @@
         <v>10</v>
       </c>
       <c r="J279" s="5" t="s">
-        <v>675</v>
-      </c>
-    </row>
-    <row r="280" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="280" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A280" s="4" t="s">
         <v>29</v>
       </c>
@@ -8344,10 +8345,10 @@
         <v>10</v>
       </c>
       <c r="J280" s="5" t="s">
-        <v>515</v>
-      </c>
-    </row>
-    <row r="281" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="281" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A281" s="4" t="s">
         <v>29</v>
       </c>
@@ -8364,10 +8365,10 @@
         <v>10</v>
       </c>
       <c r="J281" s="5" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="282" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="282" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A282" s="4" t="s">
         <v>29</v>
       </c>
@@ -8384,10 +8385,10 @@
         <v>10</v>
       </c>
       <c r="J282" s="5" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="283" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="283" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A283" s="4" t="s">
         <v>29</v>
       </c>
@@ -8404,10 +8405,10 @@
         <v>10</v>
       </c>
       <c r="J283" s="5" t="s">
-        <v>676</v>
-      </c>
-    </row>
-    <row r="284" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="284" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A284" s="4" t="s">
         <v>29</v>
       </c>
@@ -8424,10 +8425,10 @@
         <v>10</v>
       </c>
       <c r="J284" s="5" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="285" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="285" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A285" s="4" t="s">
         <v>29</v>
       </c>
@@ -8444,10 +8445,10 @@
         <v>10</v>
       </c>
       <c r="J285" s="5" t="s">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="286" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="286" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A286" s="4" t="s">
         <v>29</v>
       </c>
@@ -8464,10 +8465,10 @@
         <v>10</v>
       </c>
       <c r="J286" s="5" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="287" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="287" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A287" s="4" t="s">
         <v>29</v>
       </c>
@@ -8484,10 +8485,10 @@
         <v>10</v>
       </c>
       <c r="J287" s="5" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="288" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="288" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A288" s="4" t="s">
         <v>29</v>
       </c>
@@ -8504,10 +8505,10 @@
         <v>10</v>
       </c>
       <c r="J288" s="5" t="s">
-        <v>522</v>
-      </c>
-    </row>
-    <row r="289" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="289" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A289" s="4" t="s">
         <v>29</v>
       </c>
@@ -8524,10 +8525,10 @@
         <v>10</v>
       </c>
       <c r="J289" s="5" t="s">
-        <v>523</v>
-      </c>
-    </row>
-    <row r="290" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="290" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A290" s="4" t="s">
         <v>29</v>
       </c>
@@ -8544,10 +8545,10 @@
         <v>10</v>
       </c>
       <c r="J290" s="5" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="291" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="291" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A291" s="4" t="s">
         <v>29</v>
       </c>
@@ -8564,10 +8565,10 @@
         <v>10</v>
       </c>
       <c r="J291" s="5" t="s">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="292" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="292" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A292" s="4" t="s">
         <v>29</v>
       </c>
@@ -8584,10 +8585,10 @@
         <v>10</v>
       </c>
       <c r="J292" s="5" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="293" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="293" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A293" s="4" t="s">
         <v>29</v>
       </c>
@@ -8604,10 +8605,10 @@
         <v>10</v>
       </c>
       <c r="J293" s="5" t="s">
-        <v>527</v>
-      </c>
-    </row>
-    <row r="294" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="294" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A294" s="4" t="s">
         <v>29</v>
       </c>
@@ -8624,10 +8625,10 @@
         <v>10</v>
       </c>
       <c r="J294" s="5" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="295" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="295" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A295" s="4" t="s">
         <v>29</v>
       </c>
@@ -8644,10 +8645,10 @@
         <v>10</v>
       </c>
       <c r="J295" s="5" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="296" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="296" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A296" s="4" t="s">
         <v>29</v>
       </c>
@@ -8664,10 +8665,10 @@
         <v>10</v>
       </c>
       <c r="J296" s="5" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="297" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="297" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A297" s="4" t="s">
         <v>29</v>
       </c>
@@ -8684,10 +8685,10 @@
         <v>10</v>
       </c>
       <c r="J297" s="5" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="298" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="298" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A298" s="4" t="s">
         <v>29</v>
       </c>
@@ -8704,7 +8705,7 @@
         <v>10</v>
       </c>
       <c r="J298" s="5" t="s">
-        <v>677</v>
+        <v>672</v>
       </c>
     </row>
     <row r="299" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8727,7 +8728,7 @@
         <v>10</v>
       </c>
       <c r="J299" s="5" t="s">
-        <v>532</v>
+        <v>698</v>
       </c>
     </row>
     <row r="300" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8750,7 +8751,7 @@
         <v>10</v>
       </c>
       <c r="J300" s="5" t="s">
-        <v>533</v>
+        <v>699</v>
       </c>
     </row>
     <row r="301" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8773,7 +8774,7 @@
         <v>10</v>
       </c>
       <c r="J301" s="5" t="s">
-        <v>534</v>
+        <v>700</v>
       </c>
     </row>
     <row r="302" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8796,7 +8797,7 @@
         <v>10</v>
       </c>
       <c r="J302" s="5" t="s">
-        <v>535</v>
+        <v>701</v>
       </c>
     </row>
     <row r="303" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8819,7 +8820,7 @@
         <v>10</v>
       </c>
       <c r="J303" s="5" t="s">
-        <v>536</v>
+        <v>531</v>
       </c>
     </row>
     <row r="304" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8842,7 +8843,7 @@
         <v>10</v>
       </c>
       <c r="J304" s="5" t="s">
-        <v>537</v>
+        <v>532</v>
       </c>
     </row>
     <row r="305" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8865,7 +8866,7 @@
         <v>10</v>
       </c>
       <c r="J305" s="5" t="s">
-        <v>538</v>
+        <v>533</v>
       </c>
     </row>
     <row r="306" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8888,7 +8889,7 @@
         <v>10</v>
       </c>
       <c r="J306" s="5" t="s">
-        <v>539</v>
+        <v>534</v>
       </c>
     </row>
     <row r="307" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8911,7 +8912,7 @@
         <v>10</v>
       </c>
       <c r="J307" s="5" t="s">
-        <v>540</v>
+        <v>535</v>
       </c>
     </row>
     <row r="308" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8934,7 +8935,7 @@
         <v>10</v>
       </c>
       <c r="J308" s="5" t="s">
-        <v>541</v>
+        <v>536</v>
       </c>
     </row>
     <row r="309" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8957,7 +8958,7 @@
         <v>10</v>
       </c>
       <c r="J309" s="5" t="s">
-        <v>542</v>
+        <v>537</v>
       </c>
     </row>
     <row r="310" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -8980,7 +8981,7 @@
         <v>10</v>
       </c>
       <c r="J310" s="5" t="s">
-        <v>543</v>
+        <v>538</v>
       </c>
     </row>
     <row r="311" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9003,7 +9004,7 @@
         <v>10</v>
       </c>
       <c r="J311" s="5" t="s">
-        <v>544</v>
+        <v>539</v>
       </c>
     </row>
     <row r="312" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9026,7 +9027,7 @@
         <v>10</v>
       </c>
       <c r="J312" s="5" t="s">
-        <v>545</v>
+        <v>540</v>
       </c>
     </row>
     <row r="313" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9049,7 +9050,7 @@
         <v>10</v>
       </c>
       <c r="J313" s="5" t="s">
-        <v>546</v>
+        <v>541</v>
       </c>
     </row>
     <row r="314" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9072,7 +9073,7 @@
         <v>10</v>
       </c>
       <c r="J314" s="5" t="s">
-        <v>547</v>
+        <v>542</v>
       </c>
     </row>
     <row r="315" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9095,10 +9096,10 @@
         <v>10</v>
       </c>
       <c r="J315" s="5" t="s">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="316" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="316" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A316" s="4" t="s">
         <v>29</v>
       </c>
@@ -9115,10 +9116,10 @@
         <v>10</v>
       </c>
       <c r="J316" s="5" t="s">
-        <v>549</v>
-      </c>
-    </row>
-    <row r="317" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="317" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A317" s="4" t="s">
         <v>29</v>
       </c>
@@ -9135,10 +9136,10 @@
         <v>10</v>
       </c>
       <c r="J317" s="5" t="s">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="318" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="318" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A318" s="4" t="s">
         <v>29</v>
       </c>
@@ -9155,10 +9156,10 @@
         <v>10</v>
       </c>
       <c r="J318" s="5" t="s">
-        <v>551</v>
-      </c>
-    </row>
-    <row r="319" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="319" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A319" s="4" t="s">
         <v>29</v>
       </c>
@@ -9175,10 +9176,10 @@
         <v>10</v>
       </c>
       <c r="J319" s="5" t="s">
-        <v>552</v>
-      </c>
-    </row>
-    <row r="320" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="320" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A320" s="4" t="s">
         <v>29</v>
       </c>
@@ -9195,10 +9196,10 @@
         <v>10</v>
       </c>
       <c r="J320" s="5" t="s">
-        <v>553</v>
-      </c>
-    </row>
-    <row r="321" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="321" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A321" s="4" t="s">
         <v>29</v>
       </c>
@@ -9215,10 +9216,10 @@
         <v>10</v>
       </c>
       <c r="J321" s="5" t="s">
-        <v>554</v>
-      </c>
-    </row>
-    <row r="322" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="322" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A322" s="4" t="s">
         <v>29</v>
       </c>
@@ -9235,10 +9236,10 @@
         <v>10</v>
       </c>
       <c r="J322" s="5" t="s">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="323" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="323" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A323" s="4" t="s">
         <v>29</v>
       </c>
@@ -9255,10 +9256,10 @@
         <v>10</v>
       </c>
       <c r="J323" s="5" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="324" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="324" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A324" s="4" t="s">
         <v>29</v>
       </c>
@@ -9275,10 +9276,10 @@
         <v>10</v>
       </c>
       <c r="J324" s="5" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="325" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="325" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A325" s="4" t="s">
         <v>29</v>
       </c>
@@ -9295,10 +9296,10 @@
         <v>10</v>
       </c>
       <c r="J325" s="5" t="s">
-        <v>558</v>
-      </c>
-    </row>
-    <row r="326" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="326" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A326" s="4" t="s">
         <v>29</v>
       </c>
@@ -9315,7 +9316,7 @@
         <v>10</v>
       </c>
       <c r="J326" s="5" t="s">
-        <v>559</v>
+        <v>554</v>
       </c>
     </row>
     <row r="327" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9338,7 +9339,7 @@
         <v>10</v>
       </c>
       <c r="J327" s="5" t="s">
-        <v>560</v>
+        <v>555</v>
       </c>
     </row>
     <row r="328" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9361,7 +9362,7 @@
         <v>10</v>
       </c>
       <c r="J328" s="5" t="s">
-        <v>561</v>
+        <v>556</v>
       </c>
     </row>
     <row r="329" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9384,10 +9385,10 @@
         <v>10</v>
       </c>
       <c r="J329" s="5" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="330" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="330" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A330" s="4" t="s">
         <v>29</v>
       </c>
@@ -9404,10 +9405,10 @@
         <v>10</v>
       </c>
       <c r="J330" s="5" t="s">
-        <v>563</v>
-      </c>
-    </row>
-    <row r="331" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="331" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A331" s="4" t="s">
         <v>29</v>
       </c>
@@ -9424,10 +9425,10 @@
         <v>10</v>
       </c>
       <c r="J331" s="5" t="s">
-        <v>564</v>
-      </c>
-    </row>
-    <row r="332" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="332" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A332" s="4" t="s">
         <v>29</v>
       </c>
@@ -9444,10 +9445,10 @@
         <v>10</v>
       </c>
       <c r="J332" s="5" t="s">
-        <v>565</v>
-      </c>
-    </row>
-    <row r="333" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="333" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A333" s="4" t="s">
         <v>29</v>
       </c>
@@ -9464,10 +9465,10 @@
         <v>10</v>
       </c>
       <c r="J333" s="5" t="s">
-        <v>566</v>
-      </c>
-    </row>
-    <row r="334" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="334" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A334" s="4" t="s">
         <v>29</v>
       </c>
@@ -9484,7 +9485,7 @@
         <v>10</v>
       </c>
       <c r="J334" s="5" t="s">
-        <v>567</v>
+        <v>562</v>
       </c>
     </row>
     <row r="335" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9507,7 +9508,7 @@
         <v>10</v>
       </c>
       <c r="J335" s="5" t="s">
-        <v>568</v>
+        <v>563</v>
       </c>
     </row>
     <row r="336" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9530,10 +9531,10 @@
         <v>10</v>
       </c>
       <c r="J336" s="5" t="s">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="337" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="337" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A337" s="4" t="s">
         <v>29</v>
       </c>
@@ -9550,10 +9551,10 @@
         <v>10</v>
       </c>
       <c r="J337" s="5" t="s">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="338" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="338" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A338" s="4" t="s">
         <v>29</v>
       </c>
@@ -9570,7 +9571,7 @@
         <v>10</v>
       </c>
       <c r="J338" s="5" t="s">
-        <v>678</v>
+        <v>673</v>
       </c>
     </row>
     <row r="339" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9593,7 +9594,7 @@
         <v>10</v>
       </c>
       <c r="J339" s="5" t="s">
-        <v>571</v>
+        <v>566</v>
       </c>
     </row>
     <row r="340" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9616,10 +9617,10 @@
         <v>10</v>
       </c>
       <c r="J340" s="5" t="s">
-        <v>572</v>
-      </c>
-    </row>
-    <row r="341" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="341" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A341" s="4" t="s">
         <v>29</v>
       </c>
@@ -9636,10 +9637,10 @@
         <v>10</v>
       </c>
       <c r="J341" s="5" t="s">
-        <v>679</v>
-      </c>
-    </row>
-    <row r="342" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="342" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A342" s="4" t="s">
         <v>399</v>
       </c>
@@ -9659,10 +9660,10 @@
         <v>10</v>
       </c>
       <c r="J342" s="5" t="s">
-        <v>687</v>
-      </c>
-    </row>
-    <row r="343" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="343" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A343" s="4" t="s">
         <v>399</v>
       </c>
@@ -9679,10 +9680,10 @@
         <v>10</v>
       </c>
       <c r="J343" s="5" t="s">
-        <v>695</v>
-      </c>
-    </row>
-    <row r="344" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="344" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A344" s="4" t="s">
         <v>399</v>
       </c>
@@ -9699,10 +9700,10 @@
         <v>10</v>
       </c>
       <c r="J344" s="5" t="s">
-        <v>680</v>
-      </c>
-    </row>
-    <row r="345" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="345" spans="1:10" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A345" s="4" t="s">
         <v>399</v>
       </c>
@@ -9722,11 +9723,17 @@
         <v>10</v>
       </c>
       <c r="J345" s="5" t="s">
-        <v>684</v>
+        <v>679</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J345" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <autoFilter ref="A1:J345" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <filterColumn colId="6">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: Update expression in measures to handle null values with NVL function
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C754AB3D-C3D6-C14F-B16A-88F9CC6C398F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E52AE528-E134-BC42-9681-B70393F809E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3820" yWindow="600" windowWidth="30680" windowHeight="19060" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="200" yWindow="660" windowWidth="31440" windowHeight="19740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tables" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1891" uniqueCount="703">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1894" uniqueCount="705">
   <si>
     <t>Table Name</t>
   </si>
@@ -2135,6 +2135,12 @@
   </si>
   <si>
     <t>Table datamart informasi funding nasabah, berisi informasi terkait account funding nasabah (tabungan, giro, deposito). Table funding juga disebut dengan table DPK.</t>
+  </si>
+  <si>
+    <t>Informasi DPK</t>
+  </si>
+  <si>
+    <t>SELECT cur_book_bal FROM dm_funding.funding;</t>
   </si>
 </sst>
 </file>
@@ -6033,9 +6039,6 @@
       <c r="D169" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="E169" s="4" t="b">
-        <v>1</v>
-      </c>
       <c r="H169" s="4" t="s">
         <v>10</v>
       </c>
@@ -10011,7 +10014,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30159596-74E1-AB4A-8605-D929B81467D2}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="43.1640625" bestFit="1" customWidth="1"/>
@@ -10055,6 +10058,17 @@
         <v>21</v>
       </c>
     </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>703</v>
+      </c>
+      <c r="C4" t="s">
+        <v>704</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Enhance golden queries processing by adding description handling and output
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FB881D9-1994-1E4C-B0EA-6502DAF1269F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6FAA4D2-03BF-2941-A2F5-55B73B688510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="200" yWindow="660" windowWidth="31440" windowHeight="19740" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1894" uniqueCount="705">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1895" uniqueCount="706">
   <si>
     <t>Table Name</t>
   </si>
@@ -2141,6 +2141,9 @@
   </si>
   <si>
     <t>Informasi DPK / total DPK</t>
+  </si>
+  <si>
+    <t>funding.as_of_date; lending.as_of_date</t>
   </si>
 </sst>
 </file>
@@ -2651,7 +2654,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>22</v>
       </c>
@@ -2666,6 +2669,9 @@
       </c>
       <c r="E2" s="4" t="b">
         <v>1</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>705</v>
       </c>
       <c r="H2" s="4" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
feat: Add descriptions to golden queries for improved clarity
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CEF160A-98D4-7348-9CC3-71D541276420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A89796E-C692-D44E-A5AC-0F8EA9733354}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="200" yWindow="660" windowWidth="31440" windowHeight="19740" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1915" uniqueCount="726">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1918" uniqueCount="729">
   <si>
     <t>Table Name</t>
   </si>
@@ -2473,6 +2473,15 @@
       </rPr>
       <t>.</t>
     </r>
+  </si>
+  <si>
+    <t>Mencari nasabah aktif</t>
+  </si>
+  <si>
+    <t>Mencari aktivitas cash out</t>
+  </si>
+  <si>
+    <t>Mencari informasi DPK / total DPK</t>
   </si>
 </sst>
 </file>
@@ -10384,6 +10393,9 @@
       <c r="A2" t="s">
         <v>443</v>
       </c>
+      <c r="B2" t="s">
+        <v>726</v>
+      </c>
       <c r="C2" t="s">
         <v>397</v>
       </c>
@@ -10395,6 +10407,9 @@
       <c r="A3" t="s">
         <v>442</v>
       </c>
+      <c r="B3" t="s">
+        <v>727</v>
+      </c>
       <c r="C3" s="4" t="s">
         <v>441</v>
       </c>
@@ -10405,6 +10420,9 @@
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>704</v>
+      </c>
+      <c r="B4" t="s">
+        <v>728</v>
       </c>
       <c r="C4" t="s">
         <v>703</v>

</xml_diff>

<commit_message>
feat: Add availability date handling to schema definitions and ingestion process
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A89796E-C692-D44E-A5AC-0F8EA9733354}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AE9408C-A571-0842-AFB9-D4C6C2115E86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="200" yWindow="660" windowWidth="31440" windowHeight="19740" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1918" uniqueCount="729">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1922" uniqueCount="731">
   <si>
     <t>Table Name</t>
   </si>
@@ -2482,6 +2482,12 @@
   </si>
   <si>
     <t>Mencari informasi DPK / total DPK</t>
+  </si>
+  <si>
+    <t>Availability Date</t>
+  </si>
+  <si>
+    <t>D-1</t>
   </si>
 </sst>
 </file>
@@ -2872,15 +2878,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="91.33203125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -2890,8 +2897,11 @@
       <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="D1" s="3" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -2902,7 +2912,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -2912,8 +2922,11 @@
       <c r="C3" s="4" t="s">
         <v>400</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+      <c r="D3" s="4" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -2923,8 +2936,11 @@
       <c r="C4" s="4" t="s">
         <v>702</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="D4" s="4" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -2934,8 +2950,11 @@
       <c r="C5" s="4" t="s">
         <v>401</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="D5" s="4" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>398</v>
       </c>

</xml_diff>

<commit_message>
feat: Clear descriptions in golden queries for improved consistency
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AE9408C-A571-0842-AFB9-D4C6C2115E86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{379F0FC9-5595-5D4C-92A2-9B89846278BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="200" yWindow="660" windowWidth="31440" windowHeight="19740" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1922" uniqueCount="731">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1919" uniqueCount="728">
   <si>
     <t>Table Name</t>
   </si>
@@ -2473,15 +2473,6 @@
       </rPr>
       <t>.</t>
     </r>
-  </si>
-  <si>
-    <t>Mencari nasabah aktif</t>
-  </si>
-  <si>
-    <t>Mencari aktivitas cash out</t>
-  </si>
-  <si>
-    <t>Mencari informasi DPK / total DPK</t>
   </si>
   <si>
     <t>Availability Date</t>
@@ -2898,7 +2889,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -2923,7 +2914,7 @@
         <v>400</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="32" x14ac:dyDescent="0.2">
@@ -2937,7 +2928,7 @@
         <v>702</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -2951,7 +2942,7 @@
         <v>401</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -10412,9 +10403,6 @@
       <c r="A2" t="s">
         <v>443</v>
       </c>
-      <c r="B2" t="s">
-        <v>726</v>
-      </c>
       <c r="C2" t="s">
         <v>397</v>
       </c>
@@ -10426,9 +10414,6 @@
       <c r="A3" t="s">
         <v>442</v>
       </c>
-      <c r="B3" t="s">
-        <v>727</v>
-      </c>
       <c r="C3" s="4" t="s">
         <v>441</v>
       </c>
@@ -10439,9 +10424,6 @@
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>704</v>
-      </c>
-      <c r="B4" t="s">
-        <v>728</v>
       </c>
       <c r="C4" t="s">
         <v>703</v>

</xml_diff>

<commit_message>
feat: Refactor excel_to_dbt.py for improved clarity and dynamic time dimension detection
</commit_message>
<xml_diff>
--- a/ask-data/data/bni_dbt_definitions.xlsx
+++ b/ask-data/data/bni_dbt_definitions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevin/Documents/Work/Cloudera/GitHub/bni-ai-dev/ask-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{379F0FC9-5595-5D4C-92A2-9B89846278BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A575BB0E-D092-4D41-AC1E-C7FD184E93BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="200" yWindow="660" windowWidth="31440" windowHeight="19740" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="200" yWindow="660" windowWidth="31440" windowHeight="19740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tables" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1919" uniqueCount="728">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1918" uniqueCount="727">
   <si>
     <t>Table Name</t>
   </si>
@@ -2141,9 +2141,6 @@
   </si>
   <si>
     <t>Informasi DPK / total DPK</t>
-  </si>
-  <si>
-    <t>funding.as_of_date; lending.as_of_date</t>
   </si>
   <si>
     <t>Balance</t>
@@ -2889,7 +2886,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -2914,7 +2911,7 @@
         <v>400</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="32" x14ac:dyDescent="0.2">
@@ -2928,7 +2925,7 @@
         <v>702</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -2942,7 +2939,7 @@
         <v>401</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -3011,7 +3008,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>22</v>
       </c>
@@ -3026,9 +3023,6 @@
       </c>
       <c r="E2" s="4" t="b">
         <v>1</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>705</v>
       </c>
       <c r="H2" s="4" t="s">
         <v>10</v>
@@ -10434,82 +10428,82 @@
     </row>
     <row r="5" spans="1:4" ht="81" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
+        <v>705</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>706</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>707</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="48" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
+        <v>707</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>708</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>709</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="65" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
+        <v>709</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>710</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>711</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="81" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
+        <v>711</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>712</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>713</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="82" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
+        <v>713</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>714</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>715</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="50" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
+        <v>715</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>716</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>717</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="97" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
+        <v>717</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>718</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>719</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="65" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
+        <v>719</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>720</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>721</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="49" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
+        <v>721</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>722</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>723</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="49" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
+        <v>723</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>724</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>725</v>
       </c>
     </row>
   </sheetData>

</xml_diff>